<commit_message>
chore: daily job scan 2026-09-15
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -824,19 +824,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>InnovKaro Solutions</t>
+          <t>HuntingCube</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - AI Native Platform Build</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -846,25 +846,25 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as PRD and roadmap, lowering the ATS score. The biggest keyword gap is the absence of "product roadmap".</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several JD‑specific AI‑native terms, lowering the ATS score; the biggest keyword gap is the absence of "LLM‑in‑the‑loop"/"embeddings".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, PRD, A/B testing, OKRs, NPS improvement</t>
+          <t>LLM-in-the-loop, embeddings, agentic workflows, evaluation suite, real estate marketplace, user interview insights, prototype code (Cursor), product roadmap</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,34 +882,34 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>JUSPAY</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Marketplace</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -925,12 +925,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>No hard‑rule violations; the resume contains many relevant Agile and product‑management terms but lacks several JD‑specific keywords such as OKRs and marketplace terminology, limiting the ATS score.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, personalization, two‑sided marketplace, A/B testing, NPS improvement</t>
+          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,29 +948,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>JUSPAY</t>
+          <t>Arrowhead</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Manager(AI Products)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -981,22 +981,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title). ATS score is moderate due to missing several JD-specific terms like RICE, JTBD, and explicit AI model evaluation, while fit score is high because the candidate's GenAI and enterprise SaaS experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
+          <t>RICE prioritization, Jobs-to-be-Done (JTBD), success metrics/dashboard (e.g., KPI, NPS), AI model evaluation and guardrails, competitor analysis, sales/customer success collaboration, program coordination</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,34 +1014,34 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Arrowhead</t>
+          <t>Kroll</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager(AI Products)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1050,19 +1050,19 @@
         <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). ATS score is moderate due to missing several JD-specific terms like RICE, JTBD, and explicit AI model evaluation, while fit score is high because the candidate's GenAI and enterprise SaaS experience aligns well with the role.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>RICE prioritization, Jobs-to-be-Done (JTBD), success metrics/dashboard (e.g., KPI, NPS), AI model evaluation and guardrails, competitor analysis, sales/customer success collaboration, program coordination</t>
+          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1076,219 +1076,21 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>QS Quacquarelli Symonds</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Bangalore Urban, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many generic product skills but misses several JD‑specific terms, lowering the ATS score; the biggest gap is the lack of education‑focused digital experience keywords.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, OKRs, Mixpanel or product analytics tool, User research / persona development, Customer journey mapping, NPS improvement, MAU/engagement growth metrics, Personalization engine</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Kroll</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Tiger Analytics</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - AC</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD‑specific terms such as OS platforms and telemetry, lowering the ATS score, while the overall SaaS and enterprise experience gives a moderate fit.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Windows, macOS, Linux, Android, telemetry collection, device health monitoring, cross‑platform consistency, platform scalability, operational efficiency, roadmap ownership</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -1302,9 +1104,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1316,7 +1115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1422,12 +1221,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Zynga</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Customer Fulfilment Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1436,26 +1235,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience requirement (4 years) and contains several relevant product management keywords, but lacks many gaming‑specific terms and metrics emphasized in the JD, leading to moderate ATS and fit scores.</t>
+          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>mobile gaming, user acquisition, A/B testing, KPIs, MAU growth, NPS improvement, OKRs</t>
+          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1473,29 +1270,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Robotics</t>
+          <t>Technical Product Manager, CIAM</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1504,26 +1301,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass, but the resume contains few of the robotics‑focused keywords from the JD, leading to a low ATS score; the biggest gap is the lack of any mention of physical AI data collection or robotics.</t>
+          <t>The JD requires 6+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any CIAM‑specific terms such as OAuth, OpenID Connect, SSO, or MFA.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>physical AI data collection, robotics, task assignment, metadata management, quality review workflows, teleoperation, foundation model, RFP, go-to-market messaging</t>
+          <t>OAuth 2.0, OpenID Connect, SAML, SSO / MFA, CIAM, identity lifecycle, session/token management, authorization patterns</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1541,29 +1336,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Mercari India</t>
+          <t>Synthires</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (Japanese/English) - CS &amp; Trust &amp; Safety</t>
+          <t>Product Manager (Remote | $90–$140/hr)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1574,22 +1369,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violation, but the resume lacks many JD-specific keywords (e.g., Japanese language, Trust &amp; Safety, marketplace terminology), resulting in a low ATS score and limited domain fit.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of any mention of OKRs or JTBD.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Japanese language proficiency, Trust &amp; Safety, Customer Support workflows, Marketplace dynamics, Two-sided platform, OKRs, A/B testing, Snowflake, Mixpanel, NPS improvement</t>
+          <t>OKRs, Jobs-to-be-Done, RICE prioritization, Productboard, Mixpanel, A/B testing, platform/API product management, product-led growth</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1607,29 +1402,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Societe Generale Global Solution Centre</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, CIAM</t>
+          <t>Manager- Software Product Owner(SPO)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1640,22 +1435,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 6+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any CIAM‑specific terms such as OAuth, OpenID Connect, SSO, or MFA.</t>
+          <t>The JD requires 15+ years of experience, far exceeding the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any data‑warehouse/ETL tools such as Snowflake or IBM DataStage.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SSO / MFA, CIAM, identity lifecycle, session/token management, authorization patterns</t>
+          <t>Snowflake, IBM DataStage, Credit Risk, ETL, Data Warehouse</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1673,29 +1468,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>TD- Product Manager</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1709,19 +1504,19 @@
         <v>25</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of product‑value management or KPI frameworks.</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>value management, product KPI tracking, OKRs, RICE prioritization, A/B testing, market research methodology, life sciences/healthcare domain experience</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1739,55 +1534,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Nutanix</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of "software licensing" or related licensing terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>software licensing, cloud consumption models, quote to cash, go‑to‑market motions, customer portal UX design, OKRs, NPS improvement</t>
+          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1801,38 +1596,38 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>AskTalos</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Technical Product Manager (B2B SaaS)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -1841,19 +1636,19 @@
         <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1867,59 +1662,59 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>HARMAN India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pimpri Chinchwad, Maharashtra, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>45</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>43</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1933,7 +1728,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1942,78 +1737,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Deutsche Telekom</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner (m/w/d)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 7‑10 years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of ServiceNow or related platform terms.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>ServiceNow, API integration, platform architecture, SAP, Payment Services, customer journey, regulatory compliance, data model design, release management</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -2027,7 +1756,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-16
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ema</t>
+          <t>Versatile Club Employer of Record</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume lacks several core JD terms such as roadmap, product strategy, competitor analysis, user personas and KPIs.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflicts, so hard rules pass; the resume covers most core JD keywords but lacks explicit mentions of product roadmap, PRD, backlog grooming and analytics tools.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>roadmap, product strategy, competitor analysis, user personas, KPIs, OKRs, A/B testing</t>
+          <t>product roadmap, PRD, backlog grooming, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -692,45 +692,45 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Adobe</t>
+          <t>Revantage, A Blackstone Portfolio Company</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Growth - B2B Enterprise)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several PLG‑specific keywords, lowering the ATS score; the strongest gap is the lack of explicit PLG and A/B testing experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Product‑Led Growth (PLG), A/B testing, Go‑to‑market strategy, Usage analytics, Dashboard / funnel analysis, OKRs, Enterprise adoption metrics</t>
+          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,55 +748,55 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Scopely</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager - Gen AI</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant GenAI and SaaS keywords, but it lacks several JD‑specific tools and frameworks, lowering the ATS score; the strongest gap is the absence of explicit product‑strategy terms like "roadmap" and "OKRs".</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+          <t>OKRs, A/B testing, Snowflake, Mixpanel, ML Ops / model monitoring, product vision, roadmap definition, business impact metrics</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -814,29 +814,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HuntingCube</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI Native Platform Build</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +849,22 @@
         <v>2</v>
       </c>
       <c r="F6" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several JD‑specific AI‑native terms, lowering the ATS score; the biggest keyword gap is the absence of "LLM‑in‑the‑loop"/"embeddings".</t>
+          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>LLM-in-the-loop, embeddings, agentic workflows, evaluation suite, real estate marketplace, user interview insights, prototype code (Cursor), product roadmap</t>
+          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>JUSPAY</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II - User Discovery</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -918,19 +918,19 @@
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
+          <t>The resume meets the hard rules and includes many relevant terms, but misses several core user‑discovery keywords from the JD, lowering the ATS score; the strongest gap is the lack of explicit user research and interview experience.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
+          <t>user research, customer interviews, A/B testing, OKRs, RICE prioritization, MVP, prototype testing, market analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,55 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Arrowhead</t>
+          <t>Adobe</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager(AI Products)</t>
+          <t>Product Manager (Growth - B2B Enterprise)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). ATS score is moderate due to missing several JD-specific terms like RICE, JTBD, and explicit AI model evaluation, while fit score is high because the candidate's GenAI and enterprise SaaS experience aligns well with the role.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several PLG‑specific keywords, lowering the ATS score; the strongest gap is the lack of explicit PLG and A/B testing experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>RICE prioritization, Jobs-to-be-Done (JTBD), success metrics/dashboard (e.g., KPI, NPS), AI model evaluation and guardrails, competitor analysis, sales/customer success collaboration, program coordination</t>
+          <t>Product‑Led Growth (PLG), A/B testing, Go‑to‑market strategy, Usage analytics, Dashboard / funnel analysis, OKRs, Enterprise adoption metrics</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,83 +1014,813 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kroll</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Blitz</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Osfin.ai</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru East, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HuntingCube</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - AI Native Platform Build</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several JD‑specific AI‑native terms, lowering the ATS score; the biggest keyword gap is the absence of "LLM‑in‑the‑loop"/"embeddings".</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>LLM-in-the-loop, embeddings, agentic workflows, evaluation suite, real estate marketplace, user interview insights, prototype code (Cursor), product roadmap</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Refold AI</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G13" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Asymmetric Labs</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager(Technical)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Arrowhead</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager(AI Products)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title). ATS score is moderate due to missing several JD-specific terms like RICE, JTBD, and explicit AI model evaluation, while fit score is high because the candidate's GenAI and enterprise SaaS experience aligns well with the role.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>RICE prioritization, Jobs-to-be-Done (JTBD), success metrics/dashboard (e.g., KPI, NPS), AI model evaluation and guardrails, competitor analysis, sales/customer success collaboration, program coordination</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>eBay</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager, Assisted Service</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Kroll</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PepsiCo</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT MANAGER L1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Scoutit</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, correct title) but lacks many JD-specific terms, especially around IoT gateway and energy‑sector processes, leading to a moderate ATS score; the biggest keyword gap is the absence of any mention of IoT gateway or related release documentation.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>IoT gateway, Market Requirements Document (MRD), beta program, release notes, installers, energy management, hardware integration, reliability testing</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -1104,6 +1834,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1115,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1221,12 +1962,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Customer Fulfilment Product Manager</t>
+          <t>Product Manager - Global Trade Solutions</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1237,22 +1978,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
+          <t>Hard rules pass, but the resume lacks many trade‑finance specific terms and tools required by the JD, resulting in a modest ATS score and limited domain fit.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
+          <t>Trade finance, Letters of Credit (LC), Guarantees / SBLCs, Supply Chain Finance (SCF), Straight‑through processing, Pricing automation, Regulatory compliance, Product performance metrics, P&amp;L analysis</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1275,24 +2016,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Thomson Reuters</t>
+          <t>Atlassian</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, CIAM</t>
+          <t>CMK/Encryption Platform Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1303,22 +2044,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 6+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any CIAM‑specific terms such as OAuth, OpenID Connect, SSO, or MFA.</t>
+          <t>The resume lacks core encryption and security keywords required for the CMK/Encryption Platform role, resulting in a low ATS match; the candidate's domain is SaaS/GenAI rather than security, leading to a modest fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SSO / MFA, CIAM, identity lifecycle, session/token management, authorization patterns</t>
+          <t>Customer Managed Keys, encryption platform, bring your own key, security compliance, regulatory readiness, risk reduction, enterprise trust, roadmap definition, platform scalability</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1336,29 +2077,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Synthires</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Remote | $90–$140/hr)</t>
+          <t>Customer Fulfilment Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1369,22 +2110,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of any mention of OKRs or JTBD.</t>
+          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Jobs-to-be-Done, RICE prioritization, Productboard, Mixpanel, A/B testing, platform/API product management, product-led growth</t>
+          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1412,19 +2153,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Societe Generale Global Solution Centre</t>
+          <t>Subex</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Manager- Software Product Owner(SPO)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1435,22 +2176,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 15+ years of experience, far exceeding the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any data‑warehouse/ETL tools such as Snowflake or IBM DataStage.</t>
+          <t>The resume lacks most telecom‑fraud specific terms (SS7, CDRs, Diameter, GDPR, etc.) and only modestly matches generic product management keywords, resulting in a low ATS score; domain mismatch also drives a low fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Snowflake, IBM DataStage, Credit Risk, ETL, Data Warehouse</t>
+          <t>SS7 signaling, CDR analysis, Diameter protocol, GDPR compliance, fraud investigation workflow, MLOps (MLflow, Kubeflow, SageMaker), graph‑based fraud detection, AI coding tools (Copilot, Cursor), network topology</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1468,29 +2209,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>WillWare Technologies</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Tech Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1501,22 +2242,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>The JD explicitly requires 6+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of APIs or platform architecture.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>API lifecycle management, microservices, cloud platforms, SAFe, distributed systems</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1534,55 +2275,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Synthires</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Product Manager (Remote | $90–$140/hr)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of any mention of OKRs or JTBD.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>OKRs, Jobs-to-be-Done, RICE prioritization, Productboard, Mixpanel, A/B testing, platform/API product management, product-led growth</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1596,59 +2337,59 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (B2B SaaS)</t>
+          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1662,87 +2403,285 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HARMAN India</t>
+          <t>People Tech Group Inc</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Pimpri Chinchwad, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SAP PAPM - Product Manager</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AskTalos</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (B2B SaaS)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HARMAN India</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Pimpri Chinchwad, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -1756,6 +2695,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-17
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,14 +626,14 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AbleCredit - GenAI Infra for BFSI</t>
+          <t>Revantage, A Blackstone Portfolio Company</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -649,22 +649,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains most key terms and aligns with the Associate PM level, but lacks explicit API/integration and analytics keywords.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>APIs, integration, analytics, success metrics, feedback loops</t>
+          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revantage, A Blackstone Portfolio Company</t>
+          <t>Scopely</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager - Gen AI</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -718,19 +718,19 @@
         <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant GenAI and SaaS keywords, but it lacks several JD‑specific tools and frameworks, lowering the ATS score; the strongest gap is the absence of explicit product‑strategy terms like "roadmap" and "OKRs".</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
+          <t>OKRs, A/B testing, Snowflake, Mixpanel, ML Ops / model monitoring, product vision, roadmap definition, business impact metrics</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,29 +748,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Scopely</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Gen AI</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -779,24 +779,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant GenAI and SaaS keywords, but it lacks several JD‑specific tools and frameworks, lowering the ATS score; the strongest gap is the absence of explicit product‑strategy terms like "roadmap" and "OKRs".</t>
+          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Snowflake, Mixpanel, ML Ops / model monitoring, product vision, roadmap definition, business impact metrics</t>
+          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -814,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>Zebra Technologies</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Advanced</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -845,26 +847,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
+          <t>No hard‑rule violations; the resume covers many core Agile and stakeholder terms but lacks several explicit JD keywords such as Scrum, product backlog, and roadmap, lowering the ATS score. Domain and experience align well, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
+          <t>Scrum, product backlog, roadmap, OKRs, market trends, emerging technologies, A/B testing</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -887,50 +887,52 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - User Discovery</t>
+          <t>Associate Product Manager (Hotels)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and includes many relevant terms, but misses several core user‑discovery keywords from the JD, lowering the ATS score; the strongest gap is the lack of explicit user research and interview experience.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several JD‑specific product‑management keywords and tools, lowering the ATS score; the strongest gap is the absence of explicit KPI/experiment tracking language.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>user research, customer interviews, A/B testing, OKRs, RICE prioritization, MVP, prototype testing, market analysis</t>
+          <t>A/B testing, OKRs, conversion rate optimization, customer NPS, roadmap planning, experimentation framework, Revenue management, post‑launch performance analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -953,29 +955,29 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Adobe</t>
+          <t>Blitz</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Growth - B2B Enterprise)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -984,19 +986,19 @@
         <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several PLG‑specific keywords, lowering the ATS score; the strongest gap is the lack of explicit PLG and A/B testing experience.</t>
+          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Product‑Led Growth (PLG), A/B testing, Go‑to‑market strategy, Usage analytics, Dashboard / funnel analysis, OKRs, Enterprise adoption metrics</t>
+          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1016,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Osfin.ai</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1050,19 +1052,19 @@
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,29 +1082,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Blitz</t>
+          <t>Narayana Health</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1111,24 +1113,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1151,50 +1155,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Osfin.ai</t>
+          <t>Refold AI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
+          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,7 +1216,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1222,19 +1226,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HuntingCube</t>
+          <t>Asymmetric Labs</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI Native Platform Build</t>
+          <t>Associate Product Manager(Technical)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1244,25 +1248,25 @@
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several JD‑specific AI‑native terms, lowering the ATS score; the biggest keyword gap is the absence of "LLM‑in‑the‑loop"/"embeddings".</t>
+          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>LLM-in-the-loop, embeddings, agentic workflows, evaluation suite, real estate marketplace, user interview insights, prototype code (Cursor), product roadmap</t>
+          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1280,29 +1284,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Refold AI</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Assisted Service</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1313,22 +1317,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
+          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
+          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,57 +1350,55 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Asymmetric Labs</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(Technical)</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
+          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1410,59 +1412,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Arrowhead</t>
+          <t>Chubb</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager(AI Products)</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). ATS score is moderate due to missing several JD-specific terms like RICE, JTBD, and explicit AI model evaluation, while fit score is high because the candidate's GenAI and enterprise SaaS experience aligns well with the role.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the JD lacks many explicit keywords, resulting in moderate ATS coverage and a few key gaps.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>RICE prioritization, Jobs-to-be-Done (JTBD), success metrics/dashboard (e.g., KPI, NPS), AI model evaluation and guardrails, competitor analysis, sales/customer success collaboration, program coordination</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1476,59 +1478,59 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>State Street</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Assisted Service</t>
+          <t>Product Owner - Assistant Vice President</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
+          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
+          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1542,7 +1544,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1551,50 +1553,50 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kroll</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>PRODUCT MANAGER L1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
+          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1608,59 +1610,59 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Enterprise Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
+          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
+          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1674,7 +1676,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -1683,144 +1685,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>PRODUCT MANAGER L1</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Scoutit</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, correct title) but lacks many JD-specific terms, especially around IoT gateway and energy‑sector processes, leading to a moderate ATS score; the biggest keyword gap is the absence of any mention of IoT gateway or related release documentation.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>IoT gateway, Market Requirements Document (MRD), beta program, release notes, installers, energy management, hardware integration, reliability testing</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -1843,8 +1713,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1856,7 +1724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1962,12 +1830,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Global Trade Solutions</t>
+          <t>Product Manager - Backing Services</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1978,22 +1846,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many trade‑finance specific terms and tools required by the JD, resulting in a modest ATS score and limited domain fit.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but lacks many core platform‑service keywords, resulting in a modest ATS score; the biggest gap is the absence of cloud/infrastructure terms like DBaaS and Cache‑aaS.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Trade finance, Letters of Credit (LC), Guarantees / SBLCs, Supply Chain Finance (SCF), Straight‑through processing, Pricing automation, Regulatory compliance, Product performance metrics, P&amp;L analysis</t>
+          <t>Cache-as-a-Service (Cache‑aaS), Database-as-a-Service (DBaaS), Storage-as-a-Service (Storage‑aaS), Couchbase, S3/Object Storage, Cloud platform services, Automation of platform services, Standardisation of onboarding, Operating model design, Security and compliance</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2016,24 +1884,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Atlassian</t>
+          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CMK/Encryption Platform Product Manager</t>
+          <t>Product Manager – Network Services</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2044,22 +1912,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>48</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core encryption and security keywords required for the CMK/Encryption Platform role, resulting in a low ATS match; the candidate's domain is SaaS/GenAI rather than security, leading to a modest fit score.</t>
+          <t>The resume lacks core network‑service terminology required by the JD, resulting in a low ATS keyword match; the candidate's domain (SaaS/GenAI) does not align with the network services focus, leading to a low fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Customer Managed Keys, encryption platform, bring your own key, security compliance, regulatory readiness, risk reduction, enterprise trust, roadmap definition, platform scalability</t>
+          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, product vision, roadmap, service standardisation, self‑service onboarding</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2077,29 +1945,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>Subex</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Customer Fulfilment Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2113,19 +1981,19 @@
         <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
+          <t>The resume lacks most telecom‑fraud specific terms (SS7, CDRs, Diameter, GDPR, etc.) and only modestly matches generic product management keywords, resulting in a low ATS score; domain mismatch also drives a low fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
+          <t>SS7 signaling, CDR analysis, Diameter protocol, GDPR compliance, fraud investigation workflow, MLOps (MLflow, Kubeflow, SageMaker), graph‑based fraud detection, AI coding tools (Copilot, Cursor), network topology</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2143,29 +2011,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Subex</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager – Digital Twin with AI for Manufacturing</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2176,22 +2044,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most telecom‑fraud specific terms (SS7, CDRs, Diameter, GDPR, etc.) and only modestly matches generic product management keywords, resulting in a low ATS score; domain mismatch also drives a low fit score.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering the hard rule which forces both scores below 30. The most important keyword gap is the lack of any mention of "Digital Twin" or related manufacturing terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SS7 signaling, CDR analysis, Diameter protocol, GDPR compliance, fraud investigation workflow, MLOps (MLflow, Kubeflow, SageMaker), graph‑based fraud detection, AI coding tools (Copilot, Cursor), network topology</t>
+          <t>Digital Twin, IoT, Smart Factory, Go‑to‑Market (GTM) strategy, competitive analysis, reference architecture, pricing strategy, sales enablement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2214,24 +2082,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>WillWare Technologies</t>
+          <t>Amadeus</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Tech Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2252,12 +2120,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 6+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of APIs or platform architecture.</t>
+          <t>The JD demands 6+ years of experience while the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of explicit 'SQL' experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API lifecycle management, microservices, cloud platforms, SAFe, distributed systems</t>
+          <t>SQL, SAFe, Confluence, Airline reservations system, Departure Control System (DCS)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2280,24 +2148,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Synthires</t>
+          <t>RELIX HR Consulting Pvt Ltd - Recruitment Partner for Excellence</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Remote | $90–$140/hr)</t>
+          <t>Product Manager  - (EV/ Power Electronics)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2318,12 +2186,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of any mention of OKRs or JTBD.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any EV, battery, powertrain, or hardware‑related terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Jobs-to-be-Done, RICE prioritization, Productboard, Mixpanel, A/B testing, platform/API product management, product-led growth</t>
+          <t>EV mobility, battery management system, power electronics, hardware product development, prototype testing and certification, go‑to‑market strategy for hardware products, product lifecycle management for physical products</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2341,29 +2209,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2374,22 +2242,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>40</v>
-      </c>
       <c r="H8" s="2" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2407,29 +2275,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>People Tech Group Inc</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Healthcare Product Content</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2440,22 +2308,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2478,50 +2346,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Insight International (UK) Ltd</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SAP PAPM - Product Manager</t>
+          <t>Product Owner (DMS-Dealer Management System experience)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2535,7 +2403,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2544,29 +2412,29 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>People Tech Group Inc</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (B2B SaaS)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -2575,19 +2443,19 @@
         <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2601,87 +2469,219 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HARMAN India</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+          <t>SAP PAPM - Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pimpri Chinchwad, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>AskTalos</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (B2B SaaS)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HARMAN India</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pimpri Chinchwad, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -2698,6 +2698,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-18
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Revantage, A Blackstone Portfolio Company</t>
+          <t>Kapture CX</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,24 +647,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
+          <t>The candidate meets the 3‑year minimum and title match, yielding strong keyword overlap; the biggest gap is the lack of explicit market research/competitor analysis terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
+          <t>market research, competitor analysis, roadmap development, OKRs, A/B testing, Mixpanel, NPS improvement, user adoption metrics</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Scopely</t>
+          <t>Revantage, A Blackstone Portfolio Company</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Gen AI</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -718,19 +720,19 @@
         <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant GenAI and SaaS keywords, but it lacks several JD‑specific tools and frameworks, lowering the ATS score; the strongest gap is the absence of explicit product‑strategy terms like "roadmap" and "OKRs".</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Snowflake, Mixpanel, ML Ops / model monitoring, product vision, roadmap definition, business impact metrics</t>
+          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -753,19 +755,19 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -779,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>78</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>68</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
+          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -821,24 +821,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Zebra Technologies</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Advanced</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,24 +847,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>No hard‑rule violations; the resume covers many core Agile and stakeholder terms but lacks several explicit JD keywords such as Scrum, product backlog, and roadmap, lowering the ATS score. Domain and experience align well, giving a solid fit score.</t>
+          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Scrum, product backlog, roadmap, OKRs, market trends, emerging technologies, A/B testing</t>
+          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,57 +884,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>Connect Career</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (Hotels)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several JD‑specific product‑management keywords and tools, lowering the ATS score; the strongest gap is the absence of explicit KPI/experiment tracking language.</t>
+          <t>The candidate meets the 2+ year requirement (hard rule passed) and has strong Agile and stakeholder management experience, but lacks several JD-specific terms such as product backlog and French language, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, conversion rate optimization, customer NPS, roadmap planning, experimentation framework, Revenue management, post‑launch performance analysis</t>
+          <t>product backlog, French language proficiency, value-based decision making, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -955,50 +955,52 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Blitz</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Associate Product Manager (Hotels)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several JD‑specific product‑management keywords and tools, lowering the ATS score; the strongest gap is the absence of explicit KPI/experiment tracking language.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
+          <t>A/B testing, OKRs, conversion rate optimization, customer NPS, roadmap planning, experimentation framework, Revenue management, post‑launch performance analysis</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1021,19 +1023,19 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Osfin.ai</t>
+          <t>Blitz</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1043,7 +1045,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1052,19 +1054,19 @@
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
+          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
+          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,7 +1084,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1092,47 +1094,45 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>Osfin.ai</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1150,24 +1150,24 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Refold AI</t>
+          <t>GobabyGo EV</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1181,24 +1181,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however, several JD‑specific terms (e.g., roadmap, PRD, CRM, IoT, fleet) are missing, limiting the ATS score. The strongest keyword gap is the lack of any mention of a product roadmap or PRD.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
+          <t>product roadmap, PRD, CRM integration, IoT integration, fleet management, payment gateway integration, GPS tracking, automation of operations, KPIs and dashboards</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1216,29 +1218,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Asymmetric Labs</t>
+          <t>Narayana Health</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(Technical)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1248,25 +1250,25 @@
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1284,29 +1286,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Refold AI</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Assisted Service</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1317,22 +1319,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
+          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1350,55 +1352,57 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Asymmetric Labs</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Associate Product Manager(Technical)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
+          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
+          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1412,7 +1416,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1421,50 +1425,50 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Chubb</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the JD lacks many explicit keywords, resulting in moderate ATS coverage and a few key gaps.</t>
+          <t>The resume meets the hard rules (4 years experience, correct title) but lacks many JD-specific terms, especially around IoT gateway and energy‑sector processes, leading to a moderate ATS score; the biggest keyword gap is the absence of any mention of IoT gateway or related release documentation.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+          <t>IoT gateway, Market Requirements Document (MRD), beta program, release notes, installers, energy management, hardware integration, reliability testing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1478,33 +1482,33 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>State Street</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Assistant Vice President</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1518,19 +1522,19 @@
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
+          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,34 +1552,34 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>State Street</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L1</t>
+          <t>Product Owner - Assistant Vice President</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1584,19 +1588,19 @@
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1610,7 +1614,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -1619,24 +1623,24 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Product Manager</t>
+          <t>PRODUCT MANAGER L1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1647,22 +1651,22 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
+          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1680,17 +1684,151 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Vena Solutions</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner, Integrations</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Snowflake</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Product Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -1713,6 +1851,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1724,7 +1864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1830,38 +1970,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
+          <t>NTT DATA, Inc.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Backing Services</t>
+          <t>Product Owner - ServiceNow HRSD AI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but lacks many core platform‑service keywords, resulting in a modest ATS score; the biggest gap is the absence of cloud/infrastructure terms like DBaaS and Cache‑aaS.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Cache-as-a-Service (Cache‑aaS), Database-as-a-Service (DBaaS), Storage-as-a-Service (Storage‑aaS), Couchbase, S3/Object Storage, Cloud platform services, Automation of platform services, Standardisation of onboarding, Operating model design, Security and compliance</t>
+          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1879,29 +2019,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
+          <t>PlaySimple Games</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Network Services</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1915,19 +2055,19 @@
         <v>44</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core network‑service terminology required by the JD, resulting in a low ATS keyword match; the candidate's domain (SaaS/GenAI) does not align with the network services focus, leading to a low fit score.</t>
+          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, product vision, roadmap, service standardisation, self‑service onboarding</t>
+          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1950,24 +2090,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Subex</t>
+          <t>ITC Infotech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Customer Fulfilment Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1981,19 +2121,19 @@
         <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most telecom‑fraud specific terms (SS7, CDRs, Diameter, GDPR, etc.) and only modestly matches generic product management keywords, resulting in a low ATS score; domain mismatch also drives a low fit score.</t>
+          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>SS7 signaling, CDR analysis, Diameter protocol, GDPR compliance, fraud investigation workflow, MLOps (MLflow, Kubeflow, SageMaker), graph‑based fraud detection, AI coding tools (Copilot, Cursor), network topology</t>
+          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2016,24 +2156,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>SPADTEK SOLUTIONS</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Digital Twin with AI for Manufacturing</t>
+          <t>Product Manager – Public Cloud</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2054,12 +2194,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering the hard rule which forces both scores below 30. The most important keyword gap is the lack of any mention of "Digital Twin" or related manufacturing terminology.</t>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks many core cloud platform keywords.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Digital Twin, IoT, Smart Factory, Go‑to‑Market (GTM) strategy, competitive analysis, reference architecture, pricing strategy, sales enablement</t>
+          <t>public cloud, CI/CD pipelines, developer experience, infrastructure as code, cloud monitoring toolkits</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2082,12 +2222,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -2153,19 +2293,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>RELIX HR Consulting Pvt Ltd - Recruitment Partner for Excellence</t>
+          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager  - (EV/ Power Electronics)</t>
+          <t>Product Manager – OpenShift</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2179,19 +2319,19 @@
         <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any EV, battery, powertrain, or hardware‑related terminology.</t>
+          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core OpenShift and container platform keywords.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>EV mobility, battery management system, power electronics, hardware product development, prototype testing and certification, go‑to‑market strategy for hardware products, product lifecycle management for physical products</t>
+          <t>OpenShift, Red Hat OpenShift, container platform, Kubernetes, cloud‑native, on‑premises cloud, KPIs, SLAs, SLOs, capacity management</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2214,50 +2354,50 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>SPADTEK SOLUTIONS</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Reference Standards)</t>
+          <t>Product Manager – Network Services</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any networking-specific terms such as LBaaS, FWaaS, or DDI.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
+          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, network service roadmap, service standardization, self‑service onboarding</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2271,7 +2411,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -2280,24 +2420,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>MCO (MyComplianceOffice)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare Product Content</t>
+          <t>Product Owner - II Enterprise Data</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2311,19 +2451,19 @@
         <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
+          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2346,24 +2486,24 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Insight International (UK) Ltd</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (DMS-Dealer Management System experience)</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2374,22 +2514,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2407,29 +2547,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>People Tech Group Inc</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Healthcare Product Content</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2440,22 +2580,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2478,50 +2618,52 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Liquidnitro Games</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SAP PAPM - Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2535,59 +2677,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>Insight International (UK) Ltd</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (B2B SaaS)</t>
+          <t>Product Owner (DMS-Dealer Management System experience)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2601,87 +2743,617 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HARMAN India</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+          <t>Product Manager - Associate</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pimpri Chinchwad, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G14" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VySystems</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Scrum Product Owner</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 12+ years (and 7+ years as a Product Owner) while the candidate has only 4 years of experience, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of Agentic AI/Generative AI tools such as LangChain, LLMs, or Azure OpenAI.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI, Generative AI, LLM, LangChain, Azure OpenAI, Prompt Engineering (specific to LLMs), SAFe, Pharmaceutical, Life Sciences</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>People Tech Group Inc</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Optum India</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SAP PAPM - Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Zinnia</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="G19" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>AskTalos</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (B2B SaaS)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Saisystems Health</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Zinnia</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any life‑insurance or annuity domain terminology.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>life insurance, annuity, API integration design, incident report documentation, product commercialization</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -2700,6 +3372,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-19
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kapture CX</t>
+          <t>Zebra Technologies</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner, Advanced</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,26 +647,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title match, yielding strong keyword overlap; the biggest gap is the lack of explicit market research/competitor analysis terminology.</t>
+          <t>No hard‑rule violations; the resume covers many core Agile and stakeholder terms but lacks several explicit JD keywords such as Scrum, product backlog, and roadmap, lowering the ATS score. Domain and experience align well, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>market research, competitor analysis, roadmap development, OKRs, A/B testing, Mixpanel, NPS improvement, user adoption metrics</t>
+          <t>Scrum, product backlog, roadmap, OKRs, market trends, emerging technologies, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revantage, A Blackstone Portfolio Company</t>
+          <t>State Street</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - Assistant Vice President</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,22 +715,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
+          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
+          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +748,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,22 +781,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
+          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
+          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +814,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager- Return defect eliminaiton , RBS Return reduction</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,26 +845,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑3 year requirement and title level, but lacks fintech/payment specific terms, lowering the fit score; the biggest keyword gap is the absence of digital payments/fintech terminology.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant AI, GenAI, Agile, and stakeholder management terms but misses several JD‑specific keywords, lowering the ATS score. The candidate’s SaaS and AI background aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>digital payments, fintech, payment processing, A/B testing, OKRs, NPS improvement</t>
+          <t>FMEA Simulation, Pilot Simulation, Business Case Modeling, PRFAQ, Stage‑gate criteria, RBS Tech, Returns Finance, seller adoption, AI model accuracy, UAT coordination</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -884,29 +880,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Connect Career</t>
+          <t>Narayana Health</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,24 +911,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2+ year requirement (hard rule passed) and has strong Agile and stakeholder management experience, but lacks several JD-specific terms such as product backlog and French language, lowering the ATS score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>product backlog, French language proficiency, value-based decision making, OKRs, A/B testing</t>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,57 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (Hotels)</t>
+          <t>Product Manager, Product Platform</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
         <v>66</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several JD‑specific product‑management keywords and tools, lowering the ATS score; the strongest gap is the absence of explicit KPI/experiment tracking language.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, conversion rate optimization, customer NPS, roadmap planning, experimentation framework, Revenue management, post‑launch performance analysis</t>
+          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,29 +1014,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Blitz</t>
+          <t>Refold AI</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1051,22 +1047,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, appropriate title). The resume covers many core product skills but misses several JD‑specific terms like user research, GTM launches, and experimentation, lowering the ATS score. The strongest keyword gap is the lack of explicit "user research" experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>user research, product GTM launch, PRD (Product Requirements Document), experimentation / A/B testing, success metrics, feature adoption tracking, OKRs or RICE prioritization</t>
+          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1094,24 +1090,24 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Osfin.ai</t>
+          <t>ModMed India</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1120,19 +1116,19 @@
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, correct title). The resume covers most core ATS keywords but lacks fintech‑specific terms and explicit PRD/GTM language, causing a moderate ATS score; the biggest gap is the missing PRD/roadmap terminology.</t>
+          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Product Requirement Document (PRD), Go-to-Market (GTM) strategy, FinTech, Transaction intelligence, Roadmap, A/B testing, Competitor analysis</t>
+          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1146,76 +1142,74 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GobabyGo EV</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Specialist Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however, several JD‑specific terms (e.g., roadmap, PRD, CRM, IoT, fleet) are missing, limiting the ATS score. The strongest keyword gap is the lack of any mention of a product roadmap or PRD.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, PRD, CRM integration, IoT integration, fleet management, payment gateway integration, GPS tracking, automation of operations, KPIs and dashboards</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>nan</t>
@@ -1223,29 +1217,29 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>Vena Solutions</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Integrations</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -1253,22 +1247,22 @@
         <v>3</v>
       </c>
       <c r="F12" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>66</v>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1282,7 +1276,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1291,29 +1285,29 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Refold AI</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Enterprise Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1322,19 +1316,19 @@
         <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
+          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,7 +1342,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1357,478 +1351,12 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Asymmetric Labs</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager(Technical)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Scoutit</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, correct title) but lacks many JD-specific terms, especially around IoT gateway and energy‑sector processes, leading to a moderate ATS score; the biggest keyword gap is the absence of any mention of IoT gateway or related release documentation.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>IoT gateway, Market Requirements Document (MRD), beta program, release notes, installers, energy management, hardware integration, reliability testing</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>PepsiCo</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>State Street</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Assistant Vice President</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>PRODUCT MANAGER L1</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Vena Solutions</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner, Integrations</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Snowflake</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Enterprise Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -1846,13 +1374,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1864,7 +1385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1970,38 +1491,40 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NTT DATA, Inc.</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - ServiceNow HRSD AI</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2019,29 +1542,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PlaySimple Games</t>
+          <t>Viraaj HR Solutions Private Limited</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>OpenShift-Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2052,22 +1575,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume lacks most core OpenShift/Kubernetes keywords, lowering the ATS score, while domain experience is somewhat relevant but not a strong match for the cloud platform focus.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
+          <t>OpenShift, Kubernetes, CI/CD, Platform Engineering, Service Level Indicators (SLIs), Product Roadmapping, Beta program, Dogfooding, GitOps (ArgoCD, Flux), Terraform or Ansible</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2085,29 +1608,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ITC Infotech</t>
+          <t>Flam</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Customer Fulfilment Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2116,24 +1639,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most JD-specific terms such as SAP TMS, IDT platform, and supply chain fulfillment, resulting in a low ATS match; the biggest gap is the absence of supply chain and vendor governance keywords.</t>
+          <t>The candidate meets the years requirement and title level, but lacks many ad‑tech specific keywords and domain experience, leading to a modest ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>SAP TMS, IDT platform, OKRs, DevSecOps, Total Cost of Ownership, vendor governance, supply chain fulfillment, data privacy, regulatory compliance</t>
+          <t>DSP, SSP, RTB, Google Ad Manager, DV360, The Trade Desk, digital advertising metrics, programmatic advertising, Excel</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2151,29 +1676,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SPADTEK SOLUTIONS</t>
+          <t>LSEG</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Public Cloud</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2184,22 +1709,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks many core cloud platform keywords.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the JD's specific financial‑data and multi‑cloud keywords, leading to a modest ATS score; the biggest gap is the lack of terms like Azure, Snowflake, and ETL pipelines.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>public cloud, CI/CD pipelines, developer experience, infrastructure as code, cloud monitoring toolkits</t>
+          <t>Azure, Snowflake, ETL pipelines, logical data model, financial market data, Refinitiv, multi‑cloud, data warehousing, licensing compliance</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2222,24 +1747,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amadeus</t>
+          <t>PlaySimple Games</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2250,22 +1775,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 6+ years of experience while the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of explicit 'SQL' experience.</t>
+          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>SQL, SAFe, Confluence, Airline reservations system, Departure Control System (DCS)</t>
+          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2288,24 +1813,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – OpenShift</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2316,22 +1841,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core OpenShift and container platform keywords.</t>
+          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OpenShift, Red Hat OpenShift, container platform, Kubernetes, cloud‑native, on‑premises cloud, KPIs, SLAs, SLOs, capacity management</t>
+          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2354,24 +1879,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SPADTEK SOLUTIONS</t>
+          <t>Pragmatike</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Network Services</t>
+          <t>Product Manager – AI Security</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2382,22 +1907,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any networking-specific terms such as LBaaS, FWaaS, or DDI.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, network service roadmap, service standardization, self‑service onboarding</t>
+          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2420,50 +1945,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MCO (MyComplianceOffice)</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - II Enterprise Data</t>
+          <t>Product Manager – Digital Twin with AI for Manufacturing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering the hard rule which forces both scores below 30. The most important keyword gap is the lack of any mention of "Digital Twin" or related manufacturing terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
+          <t>Digital Twin, IoT, Smart Factory, Go‑to‑Market (GTM) strategy, competitive analysis, reference architecture, pricing strategy, sales enablement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2477,59 +2002,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Reference Standards)</t>
+          <t>Product Manager – OpenShift</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
+          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core OpenShift and container platform keywords.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
+          <t>OpenShift, Red Hat OpenShift, container platform, Kubernetes, cloud‑native, on‑premises cloud, KPIs, SLAs, SLOs, capacity management</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2543,59 +2068,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare Product Content</t>
+          <t>Sr, Product Manager II - Gantt View (Hybrid, Bangalore)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
+          <t>The JD requires 7+ years of product management experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "Gantt", "project management", and "executive alignment".</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
+          <t>Gantt View, project management, executive alignment, roadmap planning, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2609,61 +2134,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Liquidnitro Games</t>
+          <t>Aptiv</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner - AUTOSAR, Embedded Systems</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
+          <t>The JD requires 14+ years of embedded software experience, far exceeding the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks core automotive and embedded keywords.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
+          <t>ISO 26262, ASPICE, embedded software development, configuration management, gateway/zonal controller, BCM, V2X, automotive product lifecycle</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2677,7 +2200,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2686,50 +2209,50 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Insight International (UK) Ltd</t>
+          <t>Cytiva</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (DMS-Dealer Management System experience)</t>
+          <t>Product Manager Biosimilars</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>38</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>42</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>40</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
+          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
+          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2743,33 +2266,33 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>MCO (MyComplianceOffice)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Associate</t>
+          <t>Product Owner - II Enterprise Data</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2780,22 +2303,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
+          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2813,29 +2336,29 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>VySystems</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Scrum Product Owner</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2846,22 +2369,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years (and 7+ years as a Product Owner) while the candidate has only 4 years of experience, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of Agentic AI/Generative AI tools such as LangChain, LLMs, or Azure OpenAI.</t>
+          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Agentic AI, Generative AI, LLM, LangChain, Azure OpenAI, Prompt Engineering (specific to LLMs), SAFe, Pharmaceutical, Life Sciences</t>
+          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2884,24 +2407,24 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>People Tech Group Inc</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2912,22 +2435,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; additionally, key terms like "OKRs" and "A/B testing" are missing.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2950,12 +2473,12 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2490,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Healthcare Product Content</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2978,22 +2501,22 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
+          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3011,55 +2534,57 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Liquidnitro Games</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SAP PAPM - Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume matches many general product management keywords but lacks finance‑specific terms like SAP, regulatory metrics, and risk management, leading to moderate ATS and fit scores.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SAP, Regulatory compliance, RWA, LCR, NSFR, Financial controlling, Risk management, Calculator design, AI-driven process simplification</t>
+          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3073,59 +2598,59 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Zinnia</t>
+          <t>Insight International (UK) Ltd</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
+          <t>Product Owner (DMS-Dealer Management System experience)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G19" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="H19" s="2" t="n">
-        <v>43</v>
-      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
+          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
+          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3139,59 +2664,59 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (B2B SaaS)</t>
+          <t>Product Manager - Associate</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H20" s="2" t="n">
-        <v>26</v>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate does not meet the minimum 4 years of experience required, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit experience with "product demonstrations" and "CRM integrations".</t>
+          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>product demonstrations, CRM integrations, API integrations, customer onboarding, solution consulting</t>
+          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3205,7 +2730,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -3214,52 +2739,50 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Saisystems Health</t>
+          <t>VySystems</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
         <v>25</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
+          <t>The JD requires 12+ years overall and 7+ years as Product Owner, but the candidate has only 4 years, triggering a hard rule so both scores are forced below 30; the biggest keyword gap is the lack of explicit AI/Agentic AI experience.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
+          <t>Agentic AI, drug discovery, pharmaceutical industry, product vision and roadmap, backlog prioritization, Scrum Master certification, AI/ML model deployment</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3273,7 +2796,7 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
@@ -3282,29 +2805,29 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Zinnia</t>
+          <t>VySystems</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
+          <t>Scrum Product Owner</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -3320,40 +2843,372 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
+          <t>The JD requires 12+ years (and 7+ years as a Product Owner) while the candidate has only 4 years of experience, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of Agentic AI/Generative AI tools such as LangChain, LLMs, or Azure OpenAI.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI, Generative AI, LLM, LangChain, Azure OpenAI, Prompt Engineering (specific to LLMs), SAFe, Pharmaceutical, Life Sciences</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Optum India</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Zinnia</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Accelya</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Specialist - Product Owner</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Saisystems Health</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Zinnia</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
           <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any life‑insurance or annuity domain terminology.</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>life insurance, annuity, API integration design, incident report documentation, product commercialization</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -3380,6 +3235,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-20
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Zebra Technologies</t>
+          <t>Availity</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Advanced</t>
+          <t>Product Owner II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,22 +649,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>No hard‑rule violations; the resume covers many core Agile and stakeholder terms but lacks several explicit JD keywords such as Scrum, product backlog, and roadmap, lowering the ATS score. Domain and experience align well, giving a solid fit score.</t>
+          <t>The resume meets the hard‑rule criteria and contains many relevant product management keywords, but lacks healthcare‑specific terminology and a few JD‑specific tools, leading to a solid ATS score and a moderate job‑fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Scrum, product backlog, roadmap, OKRs, market trends, emerging technologies, A/B testing</t>
+          <t>Healthcare, Clearinghouse, Intelligent Gateway, Revenue cycle, Regulatory compliance (e.g., HIPAA, FHIR), Go‑to‑market planning, Roadmap development</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>State Street</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Assistant Vice President</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -718,19 +718,19 @@
         <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
+          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
+          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,55 +748,57 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Google Operations Center</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager - Applied AI and Engineering</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
+          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume lacks several JD‑specific terms such as LLMs, go‑to‑market, and ranking metrics, lowering the ATS score, while the strong GenAI and SaaS experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
+          <t>large language models (LLM), go‑to‑market strategy, ranking quality metrics, A/B testing, OKRs, user research, activation funnel, experiment design</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -819,24 +821,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Return defect eliminaiton , RBS Return reduction</t>
+          <t>Product Manager, Product Platform</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant AI, GenAI, Agile, and stakeholder management terms but misses several JD‑specific keywords, lowering the ATS score. The candidate’s SaaS and AI background aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>FMEA Simulation, Pilot Simulation, Business Case Modeling, PRFAQ, Stage‑gate criteria, RBS Tech, Returns Finance, seller adoption, AI model accuracy, UAT coordination</t>
+          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -880,29 +882,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Finance Product Owner Associate</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -911,26 +913,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>The resume meets the hard rules but lacks several finance‑specific keywords (e.g., Confluence, dashboards, GL reporting) and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>Confluence, financial reporting dashboards, General Ledger (GL) integration, exception management workflow, data modeling and aggregation</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,55 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Okta</t>
+          <t>MCO (MyComplianceOffice)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Product Platform</t>
+          <t>Data Product Owner</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product and SaaS keywords but lacks several data‑governance and compliance terms critical to the JD, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
+          <t>data governance, data quality, compliance, enterprise data platform, Snowflake, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1019,50 +1019,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Refold AI</t>
+          <t>ModMed India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to limited exact keyword overlap with the JD; the most important gap is the lack of integration‑specific terminology.</t>
+          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>integration platform, AI agents, pricing outcomes, reliability engineering, judgment layer, automation trust, OKRs, RICE prioritization, A/B testing</t>
+          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1076,59 +1076,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ModMed India</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Specialist Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H10" s="2" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
+          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1142,33 +1142,33 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Vena Solutions</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Specialist Product Manager</t>
+          <t>Product Owner, Integrations</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1177,24 +1177,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H11" s="2" t="n">
-        <v>74</v>
-      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,151 +1214,17 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Vena Solutions</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner, Integrations</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Snowflake</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Enterprise Product Manager</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains relevant SaaS and GenAI experience, but it lacks many JD‑specific terms such as Workday and OTC, resulting in a moderate ATS score; the strongest keyword gap is the absence of any mention of Workday/OTC processes.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Workday, Order to Cash (OTC), Billing, Collections, Invoices, Settlements, Snowflake, Data warehousing, OKRs</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1372,8 +1240,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1385,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1491,12 +1357,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Endava</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1505,26 +1371,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1542,29 +1406,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Viraaj HR Solutions Private Limited</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>OpenShift-Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1573,24 +1437,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume lacks most core OpenShift/Kubernetes keywords, lowering the ATS score, while domain experience is somewhat relevant but not a strong match for the cloud platform focus.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OpenShift, Kubernetes, CI/CD, Platform Engineering, Service Level Indicators (SLIs), Product Roadmapping, Beta program, Dogfooding, GitOps (ArgoCD, Flux), Terraform or Ansible</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1608,17 +1474,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1686,19 +1552,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LSEG</t>
+          <t>Cyient</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1712,19 +1578,19 @@
         <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the JD's specific financial‑data and multi‑cloud keywords, leading to a modest ATS score; the biggest gap is the lack of terms like Azure, Snowflake, and ETL pipelines.</t>
+          <t>The resume lacks many core AI‑agent and manufacturing supply‑chain keywords from the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background only loosely aligns with the AI product manager role focused on manufacturing workflows.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Azure, Snowflake, ETL pipelines, logical data model, financial market data, Refinitiv, multi‑cloud, data warehousing, licensing compliance</t>
+          <t>RFQ, Supply Chain, Manufacturing processes, MRP, S&amp;OP, human‑in‑the‑loop, adoption metrics, ROI, KPIs for AI agents</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1742,29 +1608,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PlaySimple Games</t>
+          <t>First Citizens India</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Process Manager - Product Owner, MDM</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1775,22 +1641,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>45</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
+          <t>Hard rules pass, but the resume lacks core MDM and data‑governance terminology required by the JD, resulting in low keyword density and limited domain alignment.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
+          <t>Master Data Management (MDM), Data Quality, Data Governance, Reference Data Management, Unified Master Data Management (UMDM) platform, Compliance, Roadmap development</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1808,29 +1674,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>PlaySimple Games</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1841,22 +1707,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>43</v>
-      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
+          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
+          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1874,29 +1740,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Pragmatike</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI Security</t>
+          <t>Product Owner (MR Scanner Software)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1907,22 +1773,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
+          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
+          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1945,24 +1811,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>Pragmatike</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Digital Twin with AI for Manufacturing</t>
+          <t>Product Manager – AI Security</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1983,12 +1849,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering the hard rule which forces both scores below 30. The most important keyword gap is the lack of any mention of "Digital Twin" or related manufacturing terminology.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Digital Twin, IoT, Smart Factory, Go‑to‑Market (GTM) strategy, competitive analysis, reference architecture, pricing strategy, sales enablement</t>
+          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2006,29 +1872,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TekIT Software Solutions Pvt. Ltd. (India &amp; USA)</t>
+          <t>Wells Fargo</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – OpenShift</t>
+          <t>Product Owner: Markets Repo and Securities Lending Platform (VP)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2049,12 +1915,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core OpenShift and container platform keywords.</t>
+          <t>The job title includes 'VP', triggering a hard rule that forces both scores below 30 regardless of experience or keyword match; the resume lacks several core repo and securities‑lending terms.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OpenShift, Red Hat OpenShift, container platform, Kubernetes, cloud‑native, on‑premises cloud, KPIs, SLAs, SLOs, capacity management</t>
+          <t>collateral optimization, repo trading lifecycle, securities lending, inventory utilization, risk management tools</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2072,55 +1938,55 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Cytiva</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sr, Product Manager II - Gantt View (Hybrid, Bangalore)</t>
+          <t>Product Manager Biosimilars</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "Gantt", "project management", and "executive alignment".</t>
+          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Gantt View, project management, executive alignment, roadmap planning, OKRs, A/B testing</t>
+          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2134,59 +2000,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Aptiv</t>
+          <t>MCO (MyComplianceOffice)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - AUTOSAR, Embedded Systems</t>
+          <t>Product Owner - II Enterprise Data</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 14+ years of embedded software experience, far exceeding the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks core automotive and embedded keywords.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>ISO 26262, ASPICE, embedded software development, configuration management, gateway/zonal controller, BCM, V2X, automotive product lifecycle</t>
+          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2200,59 +2066,61 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Cytiva</t>
+          <t>Liquidnitro Games</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Biosimilars</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F13" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="G13" s="2" t="n">
-        <v>38</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
+          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2266,33 +2134,33 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>MCO (MyComplianceOffice)</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - II Enterprise Data</t>
+          <t>Product Manager - Associate</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2303,22 +2171,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
+          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
+          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2341,12 +2209,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2226,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2369,22 +2237,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
+          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
+          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2402,29 +2270,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>VySystems</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Reference Standards)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2435,22 +2303,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
+          <t>The JD requires 12+ years overall and 7+ years as Product Owner, but the candidate has only 4 years, triggering a hard rule so both scores are forced below 30; the biggest keyword gap is the lack of explicit AI/Agentic AI experience.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
+          <t>Agentic AI, drug discovery, pharmaceutical industry, product vision and roadmap, backlog prioritization, Scrum Master certification, AI/ML model deployment</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2468,55 +2336,55 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Zinnia</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare Product Content</t>
+          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD keywords such as root cause analysis, coding intelligence, and product content loading, lowering the ATS score; domain mismatch reduces the fit score.</t>
+          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>root cause analysis, 5 Whys, content accuracy, coding intelligence, product content loading, AP, story boarding, user interface requirements, regulatory content research</t>
+          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2530,61 +2398,59 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Liquidnitro Games</t>
+          <t>Accelya</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Specialist - Product Owner</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
+          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
+          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2598,7 +2464,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -2607,50 +2473,52 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Insight International (UK) Ltd</t>
+          <t>Saisystems Health</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (DMS-Dealer Management System experience)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F19" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core domain keywords (Dealer Management System, automobile) and the title does not match the Product Owner role, resulting in low ATS and fit scores; the biggest gap is the missing DME/Dealer Management System experience.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Dealer Management System, DME, Automobile domain, Product Owner, OKRs</t>
+          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2664,7 +2532,7 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
@@ -2673,50 +2541,50 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Zinnia</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Associate</t>
+          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any life‑insurance or annuity domain terminology.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
+          <t>life insurance, annuity, API integration design, incident report documentation, product commercialization</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2730,7 +2598,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -2739,476 +2607,12 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>VySystems</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 12+ years overall and 7+ years as Product Owner, but the candidate has only 4 years, triggering a hard rule so both scores are forced below 30; the biggest keyword gap is the lack of explicit AI/Agentic AI experience.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Agentic AI, drug discovery, pharmaceutical industry, product vision and roadmap, backlog prioritization, Scrum Master certification, AI/ML model deployment</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>VySystems</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Scrum Product Owner</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 12+ years (and 7+ years as a Product Owner) while the candidate has only 4 years of experience, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of Agentic AI/Generative AI tools such as LangChain, LLMs, or Azure OpenAI.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Agentic AI, Generative AI, LLM, LangChain, Azure OpenAI, Prompt Engineering (specific to LLMs), SAFe, Pharmaceutical, Life Sciences</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Optum India</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Zinnia</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Accelya</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Specialist - Product Owner</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Saisystems Health</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Zinnia</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any life‑insurance or annuity domain terminology.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>life insurance, annuity, API integration design, incident report documentation, product commercialization</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3233,13 +2637,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-21
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versatile Club Employer of Record</t>
+          <t>WisdomAI</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -583,22 +583,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>81</v>
-      </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflicts, so hard rules pass; the resume covers most core JD keywords but lacks explicit mentions of product roadmap, PRD, backlog grooming and analytics tools.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, PRD, backlog grooming, A/B testing, Mixpanel, NPS improvement</t>
+          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -692,19 +692,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Aerchain</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -713,24 +713,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>67</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
+          <t>The candidate meets the 4‑year requirement and title seniority is appropriate, but the resume lacks several procurement‑specific terms and AI‑prototyping methodology keywords, lowering the ATS score. The strongest gap is the absence of explicit procurement experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
+          <t>procurement, AI prototyping, OKRs, RICE prioritization, customer NPS</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,57 +750,55 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Google Operations Center</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Applied AI and Engineering</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume lacks several JD‑specific terms such as LLMs, go‑to‑market, and ranking metrics, lowering the ATS score, while the strong GenAI and SaaS experience drives a solid fit score.</t>
+          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>large language models (LLM), go‑to‑market strategy, ranking quality metrics, A/B testing, OKRs, user research, activation funnel, experiment design</t>
+          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Okta</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Product Platform</t>
+          <t>Product Manager- Return defect eliminaiton , RBS Return reduction</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant AI, GenAI, Agile, and stakeholder management terms but misses several JD‑specific keywords, lowering the ATS score. The candidate’s SaaS and AI background aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
+          <t>FMEA Simulation, Pilot Simulation, Business Case Modeling, PRFAQ, Stage‑gate criteria, RBS Tech, Returns Finance, seller adoption, AI model accuracy, UAT coordination</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,17 +882,17 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -958,19 +958,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MCO (MyComplianceOffice)</t>
+          <t>EchorTech</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -979,24 +979,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product and SaaS keywords but lacks several data‑governance and compliance terms critical to the JD, lowering the ATS score.</t>
+          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior title triggers hard rules; most JD keywords are present but key terms like "product roadmap", "API integration" and "PRD" are missing.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>data governance, data quality, compliance, enterprise data platform, Snowflake, OKRs, RICE prioritization</t>
+          <t>API integration, product roadmap, PRD (Product Requirements Document), product analytics tool (e.g., Mixpanel), OKRs or RICE prioritization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1016,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ModMed India</t>
+          <t>Kanerika Inc</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1047,22 +1049,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
+          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,55 +1082,55 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>ModMed India</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Specialist Product Manager</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
+          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
+          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1142,7 +1144,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1151,24 +1153,24 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Vena Solutions</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Integrations</t>
+          <t>Specialist Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1177,26 +1179,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,17 +1214,83 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Qualys</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
           <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -1240,6 +1306,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1251,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1357,12 +1424,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Endava</t>
+          <t>Jupiter</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager- Unsecured Lending</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1371,24 +1438,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
+          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
+          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1406,29 +1475,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>LSEG</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1437,26 +1506,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the JD's specific financial‑data and multi‑cloud keywords, leading to a modest ATS score; the biggest gap is the lack of terms like Azure, Snowflake, and ETL pipelines.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>Azure, Snowflake, ETL pipelines, logical data model, financial market data, Refinitiv, multi‑cloud, data warehousing, licensing compliance</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1479,24 +1546,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Flam</t>
+          <t>Cyient</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1505,26 +1572,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but lacks many ad‑tech specific keywords and domain experience, leading to a modest ATS score and a lower fit score.</t>
+          <t>The resume lacks many core AI‑agent and manufacturing supply‑chain keywords from the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background only loosely aligns with the AI product manager role focused on manufacturing workflows.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>DSP, SSP, RTB, Google Ad Manager, DV360, The Trade Desk, digital advertising metrics, programmatic advertising, Excel</t>
+          <t>RFQ, Supply Chain, Manufacturing processes, MRP, S&amp;OP, human‑in‑the‑loop, adoption metrics, ROI, KPIs for AI agents</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1547,24 +1612,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Cyient</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Owner (MR Scanner Software)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1578,19 +1643,19 @@
         <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>45</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many core AI‑agent and manufacturing supply‑chain keywords from the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background only loosely aligns with the AI product manager role focused on manufacturing workflows.</t>
+          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>RFQ, Supply Chain, Manufacturing processes, MRP, S&amp;OP, human‑in‑the‑loop, adoption metrics, ROI, KPIs for AI agents</t>
+          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1608,29 +1673,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>First Citizens India</t>
+          <t>Pragmatike</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Process Manager - Product Owner, MDM</t>
+          <t>Product Manager – AI Security</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1641,22 +1706,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core MDM and data‑governance terminology required by the JD, resulting in low keyword density and limited domain alignment.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Master Data Management (MDM), Data Quality, Data Governance, Reference Data Management, Unified Master Data Management (UMDM) platform, Compliance, Roadmap development</t>
+          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1674,55 +1739,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PlaySimple Games</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Sr, Product Manager II - Gantt View (Hybrid, Bangalore)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
+          <t>The JD requires 7+ years of product management experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "Gantt", "project management", and "executive alignment".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
+          <t>Gantt View, project management, executive alignment, roadmap planning, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1745,24 +1810,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>SPADTEK SOLUTIONS</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (MR Scanner Software)</t>
+          <t>Product Manager – Network Services</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1773,22 +1838,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any networking-specific terms such as LBaaS, FWaaS, or DDI.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
+          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, network service roadmap, service standardization, self‑service onboarding</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1811,50 +1876,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Pragmatike</t>
+          <t>Cytiva</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI Security</t>
+          <t>Product Manager Biosimilars</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
+          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
+          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1868,7 +1933,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1877,50 +1942,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Wells Fargo</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner: Markets Repo and Securities Lending Platform (VP)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The job title includes 'VP', triggering a hard rule that forces both scores below 30 regardless of experience or keyword match; the resume lacks several core repo and securities‑lending terms.</t>
+          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>collateral optimization, repo trading lifecycle, securities lending, inventory utilization, risk management tools</t>
+          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1934,7 +1999,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1943,50 +2008,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cytiva</t>
+          <t>Golden Opportunities</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Biosimilars</t>
+          <t>Product Manager - GO/JC/4605/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
+          <t>The candidate has only 4 years experience while the JD requires 12+ years, triggering a hard rule that forces both scores below 30; also missing key terms like 'data warehousing' and 'GTM strategy'.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
+          <t>data warehousing, ETL pipelines, business intelligence dashboards, GTM strategy, product strategy</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2000,7 +2065,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2009,50 +2074,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MCO (MyComplianceOffice)</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - II Enterprise Data</t>
+          <t>Product Manager - Ruminant</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core data‑management keywords from the JD, lowering the ATS score, while the overall domain fit is moderate.</t>
+          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Data Governance, Master Data Management (MDM), Data Profiling / Data Mapping / Data Modelling, Data Quality Management, Data De‑Duplication, User Acceptance Testing, Impact Analysis, Backlog Refinement</t>
+          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2066,61 +2131,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Liquidnitro Games</t>
+          <t>Accelya</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Specialist - Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks most gaming‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of player‑behavior and A/B testing terminology.</t>
+          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, player retention, live events, cohort analysis, game economy, player segmentation, monetization, core loop</t>
+          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2134,7 +2197,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -2143,476 +2206,12 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>JPMorganChase</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Associate</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The JD explicitly requires 5+ years of product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of MLOps/ModelOps or responsible AI controls.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>MLOps, ModelOps, responsible AI controls, PII handling, prompt safety, semantic search, model governance, A/B testing, OKRs</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Optum India</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The JD implies a 5+ years experience requirement, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'capital budgeting', 'OKRs', and 'value connect'.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>capital budgeting, OKRs, Value Connect, knowledge center, A/B testing, Snowflake</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>VySystems</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 12+ years overall and 7+ years as Product Owner, but the candidate has only 4 years, triggering a hard rule so both scores are forced below 30; the biggest keyword gap is the lack of explicit AI/Agentic AI experience.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Agentic AI, drug discovery, pharmaceutical industry, product vision and roadmap, backlog prioritization, Scrum Master certification, AI/ML model deployment</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Zinnia</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Accelya</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Specialist - Product Owner</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Saisystems Health</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any healthcare data standards (e.g., FHIR, HL7).</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>FHIR, HL7, Mirth, API documentation, data cataloging, SQL performance tuning, Confluence, healthcare integration engine</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Zinnia</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager -Technical (Life Insurance &amp; Annuity)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any life‑insurance or annuity domain terminology.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>life insurance, annuity, API integration design, incident report documentation, product commercialization</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -2630,13 +2229,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-22
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Availity</t>
+          <t>Aerchain</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,24 +647,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G3" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>74</v>
-      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard‑rule criteria and contains many relevant product management keywords, but lacks healthcare‑specific terminology and a few JD‑specific tools, leading to a solid ATS score and a moderate job‑fit score.</t>
+          <t>The candidate meets the 4‑year requirement and title seniority is appropriate, but the resume lacks several procurement‑specific terms and AI‑prototyping methodology keywords, lowering the ATS score. The strongest gap is the absence of explicit procurement experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Healthcare, Clearinghouse, Intelligent Gateway, Revenue cycle, Regulatory compliance (e.g., HIPAA, FHIR), Go‑to‑market planning, Roadmap development</t>
+          <t>procurement, AI prototyping, OKRs, RICE prioritization, customer NPS</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,24 +684,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Aerchain</t>
+          <t>Empower India</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -713,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and title seniority is appropriate, but the resume lacks several procurement‑specific terms and AI‑prototyping methodology keywords, lowering the ATS score. The strongest gap is the absence of explicit procurement experience.</t>
+          <t>The resume meets the basic experience and seniority requirements, but lacks several JD-specific keywords such as A/B testing and product roadmap, lowering the ATS score; the domain shift from SaaS/enterprise tools to financial services creates a moderate fit gap.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>procurement, AI prototyping, OKRs, RICE prioritization, customer NPS</t>
+          <t>A/B testing, Usability testing, Customer research, Product roadmap, Compliance, Key performance indicators (KPIs), OKRs, Product strategy</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -755,24 +755,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Chevron</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Digital Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,24 +781,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume covers many agile and data-driven keywords but lacks several JD-specific terms such as OKRs and contact‑center language, lowering the ATS score. Domain experience is relevant but not health‑care specific, resulting in a moderate fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific terms like roadmap, OKRs, and integration, lowering the ATS score; domain alignment is moderate but not a direct energy‑wells focus.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Contact Center, Consumer Insights, Experience Analytics, NPS improvement, MLP (Minimum Lovable Product), Release strategy</t>
+          <t>product roadmap, OKRs, KPIs, integration with IT systems, digital platform governance, release management, value‑based prioritization</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,55 +818,57 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Google Operations Center</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Return defect eliminaiton , RBS Return reduction</t>
+          <t>Product Manager - Applied AI and Engineering</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant AI, GenAI, Agile, and stakeholder management terms but misses several JD‑specific keywords, lowering the ATS score. The candidate’s SaaS and AI background aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume lacks several JD‑specific terms such as LLMs, go‑to‑market, and ranking metrics, lowering the ATS score, while the strong GenAI and SaaS experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>FMEA Simulation, Pilot Simulation, Business Case Modeling, PRFAQ, Stage‑gate criteria, RBS Tech, Returns Finance, seller adoption, AI model accuracy, UAT coordination</t>
+          <t>large language models (LLM), go‑to‑market strategy, ranking quality metrics, A/B testing, OKRs, user research, activation funnel, experiment design</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,17 +886,17 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -958,7 +962,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1020,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1026,19 +1030,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kanerika Inc</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1049,22 +1053,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1087,24 +1091,24 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ModMed India</t>
+          <t>Kanerika Inc</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1115,22 +1119,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
+          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,29 +1152,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Specialist Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,22 +1185,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several payment‑specific and experimentation terms, lowering the ATS score slightly; the biggest gap is the absence of explicit experimentation/A‑B testing language.</t>
+          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Experimentation framework, Payments industry experience, Risk management, Snowflake</t>
+          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,83 +1218,17 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Qualys</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1244,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1318,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1424,12 +1361,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Jupiter</t>
+          <t>Philips</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Unsecured Lending</t>
+          <t>Product Manager, G&amp;B Digital Products, PHDSI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1438,26 +1375,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core JD terms such as product roadmap, go‑to‑market, business case, and KPI tracking, lowering the ATS score; the biggest keyword gap is the absence of any mention of a product roadmap.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
+          <t>product roadmap, go-to-market strategy, business case development, KPIs (adoption, engagement, funnel performance), claims strategy, regulatory compliance, consumer insights, launch readiness, market readiness</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1480,24 +1415,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LSEG</t>
+          <t>Jupiter</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager- Unsecured Lending</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1506,24 +1441,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the JD's specific financial‑data and multi‑cloud keywords, leading to a modest ATS score; the biggest gap is the lack of terms like Azure, Snowflake, and ETL pipelines.</t>
+          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Azure, Snowflake, ETL pipelines, logical data model, financial market data, Refinitiv, multi‑cloud, data warehousing, licensing compliance</t>
+          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1541,24 +1478,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Cyient</t>
+          <t>GE Vernova</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1577,19 +1514,19 @@
         <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many core AI‑agent and manufacturing supply‑chain keywords from the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background only loosely aligns with the AI product manager role focused on manufacturing workflows.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title or explicit 5+ year requirement), but the resume lacks many JD-specific terms and the title does not align closely, lowering the ATS score; the biggest keyword gap is the absence of program‑management terminology like NPI/CTQ.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>RFQ, Supply Chain, Manufacturing processes, MRP, S&amp;OP, human‑in‑the‑loop, adoption metrics, ROI, KPIs for AI agents</t>
+          <t>NPI (New Product Introduction), CTQ (Critical to Quality), budget management, program management, dashboards, metrics reporting, OKRs, cross‑functional program coordination</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1607,29 +1544,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>Freight Tiger</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (MR Scanner Software)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1638,24 +1575,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
+          <t>Hard rules pass (4 years meets the 2‑year minimum and no senior title). The resume contains many generic product management keywords but lacks logistics‑specific terms such as freight invoicing, ERP integration, and payments, leading to a moderate ATS score and only a tangential domain fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
+          <t>freight invoicing, payment reconciliation, ERP integration (SAP, Oracle, Tally), B2B payments workflow, logistics platform scalability, predictive AI models, anomaly detection, NPS tracking, financial integrations (banks, NBFCs, payment gateways)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1673,29 +1612,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pragmatike</t>
+          <t>Pharmed Limited</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI Security</t>
+          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1704,24 +1643,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of cloud security or AI security-specific terms.</t>
+          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>cloud security, AI security platform, CISO interviews, security research partnership, AI agent inventory</t>
+          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1739,55 +1680,57 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pharmed Limited</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Sr, Product Manager II - Gantt View (Hybrid, Bangalore)</t>
+          <t>Product Manager - Pharmaceuticals (Gynae Portfolio)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "Gantt", "project management", and "executive alignment".</t>
+          <t>The candidate meets the 3‑year minimum and location requirement, but the resume lacks core pharmaceutical marketing keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is missing pharma brand management terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Gantt View, project management, executive alignment, roadmap planning, OKRs, A/B testing</t>
+          <t>pharmaceutical brand management, marketing strategy, promotional materials, fieldwork with sales team, CMEs and conference participation, market dynamics analysis, regulatory compliance</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1805,29 +1748,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SPADTEK SOLUTIONS</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Network Services</t>
+          <t>Product Manager, Customer Support API Platform</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1838,22 +1781,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any networking-specific terms such as LBaaS, FWaaS, or DDI.</t>
+          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any API or integration platform experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Load Balancers as a Service (LBaaS), Firewalls as a Service (FWaaS), DDI as a Service (DDIaaS), DHCP, IP Address Management (IPAM), DNS, network service roadmap, service standardization, self‑service onboarding</t>
+          <t>API design, microservices, cloud platform, developer engagement, API governance, security standards, platform roadmap</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1876,50 +1819,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cytiva</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Biosimilars</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations, but the resume lacks core biosimilars and cell culture terminology, resulting in low keyword overlap and poor domain alignment.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>biosimilars, cell culture media, pricing strategy, market intelligence, competitive analysis, technical slide creation, commercial enablement</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1933,59 +1876,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Comviva</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
+          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
+          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1999,59 +1942,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>Innova ESI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - GO/JC/4605/2026</t>
+          <t>Product Owner (Healthcare Domain)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years experience while the JD requires 12+ years, triggering a hard rule that forces both scores below 30; also missing key terms like 'data warehousing' and 'GTM strategy'.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key healthcare and Scrum-specific terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>data warehousing, ETL pipelines, business intelligence dashboards, GTM strategy, product strategy</t>
+          <t>Scrum, Product Owner, SOX compliance, Release Train Engineer, Scaled Agile Framework, backlog grooming, healthcare domain</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2065,59 +2008,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MSD</t>
+          <t>Albemarle Corporation</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Ruminant</t>
+          <t>Data Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core data‑product keywords.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+          <t>data governance, data quality, enterprise reporting, cloud‑native analytics, SQL, Snowflake, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2131,7 +2074,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2140,78 +2083,210 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Accelya</t>
+          <t>Blue Spire Inc</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Specialist - Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules apply because the JD requires 10+ years and senior level, while the candidate has only 4 years; therefore both scores are forced below 30, with the biggest keyword gap being lack of Amazon Connect/LLM specific terms.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Amazon Connect, Amazon Lex, Large Language Models (LLMs), IVR, call containment, first contact resolution (FCR), AWS, product roadmap</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>MSD</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Ruminant</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Innova ESI</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner / Capability Manager</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>The JD mandates 6+ years of Product Owner experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of NDC or airline‑specific workflow experience.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>NDC, airline industry experience, platform/API solutions, SAFe, API integration, release management, OKRs, RICE prioritization</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. The most important keyword gap is the lack of explicit "Scrum" and "Product Owner" terminology.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Scrum, Product Owner, SOX compliance, Release Train Engineer, Scaled Agile Framework (SAFe), AS400, claim adjudication</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Apply</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -2229,6 +2304,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-23
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>WisdomAI</t>
+          <t>Autofleet</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -583,22 +583,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is a close match, so hard rules pass. The resume contains most core SaaS and Agile keywords but lacks several JD‑specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,24 +616,24 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aerchain</t>
+          <t>Superleap AI CRM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -651,22 +651,22 @@
         <v>4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and title seniority is appropriate, but the resume lacks several procurement‑specific terms and AI‑prototyping methodology keywords, lowering the ATS score. The strongest gap is the absence of explicit procurement experience.</t>
+          <t>The candidate meets the 4-year experience requirement and title level is acceptable, yielding solid ATS and fit scores; the most important keyword gap is the lack of ARR/MRR/churn metrics.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>procurement, AI prototyping, OKRs, RICE prioritization, customer NPS</t>
+          <t>ARR, MRR, churn, roadmap planning, OKRs, market trends analysis</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,24 +684,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Empower India</t>
+          <t>WisdomAI</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -717,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience and seniority requirements, but lacks several JD-specific keywords such as A/B testing and product roadmap, lowering the ATS score; the domain shift from SaaS/enterprise tools to financial services creates a moderate fit gap.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Usability testing, Customer research, Product roadmap, Compliance, Key performance indicators (KPIs), OKRs, Product strategy</t>
+          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Chevron</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific terms like roadmap, OKRs, and integration, lowering the ATS score; domain alignment is moderate but not a direct energy‑wells focus.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the seniority level, but lacks several specific JD terms such as scrum master and change control. The most important gap is the absence of explicit Scrum Master / change control experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, KPIs, integration with IT systems, digital platform governance, release management, value‑based prioritization</t>
+          <t>scrum master, change control procedures, mockups, flowcharts, process diagrams, project schedule, business acumen</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -823,52 +821,50 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Google Operations Center</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Applied AI and Engineering</t>
+          <t>Product Manager II - AI PM</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume lacks several JD‑specific terms such as LLMs, go‑to‑market, and ranking metrics, lowering the ATS score, while the strong GenAI and SaaS experience drives a solid fit score.</t>
+          <t>The candidate meets the 2+ years requirement and has relevant GenAI and SaaS experience, but the resume lacks several JD-specific AI tooling keywords, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>large language models (LLM), go‑to‑market strategy, ranking quality metrics, A/B testing, OKRs, user research, activation funnel, experiment design</t>
+          <t>Cursor, Claude Code, Replit, n8n, MCPs, AI agents, tool calling, LLM evaluation, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,29 +882,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>eReleGo Technologies Pvt Ltd (ETPL)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Finance Product Owner Associate</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,24 +913,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules but lacks several finance‑specific keywords (e.g., Confluence, dashboards, GL reporting) and domain experience, lowering both scores.</t>
+          <t>The resume meets the 3‑year minimum and title level, but misses several JD‑specific terms such as GTM strategy, product demos, and PRDs, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Confluence, financial reporting dashboards, General Ledger (GL) integration, exception management workflow, data modeling and aggregation</t>
+          <t>GTM strategy, product demos, deal closure support, PRD (Product Requirement Document), market trends analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,57 +950,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EchorTech</t>
+          <t>Applied Materials India</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior title triggers hard rules; most JD keywords are present but key terms like "product roadmap", "API integration" and "PRD" are missing.</t>
+          <t>The candidate meets the 4-year experience requirement and has no senior title conflict, but the resume lacks several core JD keywords (e.g., Python, product roadmap, supply chain), lowering the ATS score while still showing good overall fit.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>API integration, product roadmap, PRD (Product Requirements Document), product analytics tool (e.g., Mixpanel), OKRs or RICE prioritization</t>
+          <t>Python, product roadmap, supply chain, manufacturing operations, data pipelines, scalable architecture, OKRs, quantitative opportunity sizing</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1016,38 +1012,38 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Empower India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1063,12 +1059,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
+          <t>The resume meets the basic experience and seniority requirements, but lacks several JD-specific keywords such as A/B testing and product roadmap, lowering the ATS score; the domain shift from SaaS/enterprise tools to financial services creates a moderate fit gap.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
+          <t>A/B testing, Usability testing, Customer research, Product roadmap, Compliance, Key performance indicators (KPIs), OKRs, Product strategy</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,59 +1078,61 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kanerika Inc</t>
+          <t>Chevron</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>64</v>
-      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific terms like roadmap, OKRs, and integration, lowering the ATS score; domain alignment is moderate but not a direct energy‑wells focus.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
+          <t>product roadmap, OKRs, KPIs, integration with IT systems, digital platform governance, release management, value‑based prioritization</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,7 +1146,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1157,78 +1155,612 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>SAYZO</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the years and title requirements, but lacks many core JD keywords (e.g., GA4, Mixpanel, A/B testing), lowering the ATS score; the biggest gap is the absence of explicit growth‑experiment terminology.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, GA4, Mixpanel, Amplitude, Growth loops, PLG, CAC, LTV, Cohort analysis, Dashboard (GA4/Amplitude)</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Codeft Digital</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 2‑year minimum and has a matching title, but lacks the specific tool Zoho Projects mentioned in the JD, creating the biggest keyword gap.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Zoho Projects, A/B testing, OKRs, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>EchorTech</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior title triggers hard rules; most JD keywords are present but key terms like "product roadmap", "API integration" and "PRD" are missing.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>API integration, product roadmap, PRD (Product Requirements Document), product analytics tool (e.g., Mixpanel), OKRs or RICE prioritization</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>StarRez, Inc.</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager II</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>FBS Product Owner III- Guidewire</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Kanerika Inc</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TriNet</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>Qualys</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Associate Product Manager</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="2" t="n">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1244,6 +1776,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1255,7 +1795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1361,12 +1901,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Philips</t>
+          <t>Bytebeam</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, G&amp;B Digital Products, PHDSI</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1387,12 +1927,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core JD terms such as product roadmap, go‑to‑market, business case, and KPI tracking, lowering the ATS score; the biggest keyword gap is the absence of any mention of a product roadmap.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many JD-specific terms like fleet, telematics, OTA updates, resulting in a moderate ATS score and only partial domain fit.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, go-to-market strategy, business case development, KPIs (adoption, engagement, funnel performance), claims strategy, regulatory compliance, consumer insights, launch readiness, market readiness</t>
+          <t>fleet owners, telemetry, remote diagnostics, OTA updates, IoT, telematics, customer advisory board, OKRs, guardrail, A/B testing</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1415,24 +1955,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Jupiter</t>
+          <t>Zepto</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Unsecured Lending</t>
+          <t>Associate Product Manager – Planning</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1442,25 +1982,25 @@
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks many core JD keywords such as Python, pandas, forecasting and inventory‑planning terms, lowering the ATS score; the biggest gap is the absence of Python/pandas experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
+          <t>Python, pandas, numpy, forecasting, inventory management, root‑cause analysis, dashboards, SQL window functions, data visualization libraries</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1478,17 +2018,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1544,7 +2084,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1554,19 +2094,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Freight Tiger</t>
+          <t>Jupiter</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager- Unsecured Lending</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1576,7 +2116,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>55</v>
@@ -1589,12 +2129,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum and no senior title). The resume contains many generic product management keywords but lacks logistics‑specific terms such as freight invoicing, ERP integration, and payments, leading to a moderate ATS score and only a tangential domain fit.</t>
+          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>freight invoicing, payment reconciliation, ERP integration (SAP, Oracle, Tally), B2B payments workflow, logistics platform scalability, predictive AI models, anomaly detection, NPS tracking, financial integrations (banks, NBFCs, payment gateways)</t>
+          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1612,29 +2152,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pharmed Limited</t>
+          <t>Freight Tiger</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1644,25 +2184,25 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
+          <t>Hard rules pass (4 years meets the 2‑year minimum and no senior title). The resume contains many generic product management keywords but lacks logistics‑specific terms such as freight invoicing, ERP integration, and payments, leading to a moderate ATS score and only a tangential domain fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
+          <t>freight invoicing, payment reconciliation, ERP integration (SAP, Oracle, Tally), B2B payments workflow, logistics platform scalability, predictive AI models, anomaly detection, NPS tracking, financial integrations (banks, NBFCs, payment gateways)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1680,17 +2220,17 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1702,7 +2242,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Pharmaceuticals (Gynae Portfolio)</t>
+          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1712,25 +2252,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and location requirement, but the resume lacks core pharmaceutical marketing keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is missing pharma brand management terminology.</t>
+          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>pharmaceutical brand management, marketing strategy, promotional materials, fieldwork with sales team, CMEs and conference participation, market dynamics analysis, regulatory compliance</t>
+          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1748,7 +2288,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1758,7 +2298,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1814,7 +2354,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1824,14 +2364,14 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Comviva</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1847,22 +2387,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>27</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
+          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1880,29 +2420,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Comviva</t>
+          <t>IGEL Technology</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Bangalore</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1916,19 +2456,19 @@
         <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
+          <t>The JD requires 6+ years of enterprise product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of explicit analytics/observability experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
+          <t>analytics platform, observability, endpoint telemetry, cloud/SaaS offering, AI-driven insights</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1951,12 +2491,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1968,7 +2508,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Healthcare Domain)</t>
+          <t>Product Owner – PBM / Pharmacy Benefits</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1982,19 +2522,19 @@
         <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key healthcare and Scrum-specific terminology.</t>
+          <t>The JD requires 5+ years of experience while the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core pharmacy‑benefits terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Scrum, Product Owner, SOX compliance, Release Train Engineer, Scaled Agile Framework, backlog grooming, healthcare domain</t>
+          <t>Pharmacy Benefits Management (PBM), Rx formulary management, Drug data analysis, MS Access, Stakeholder presentations / release notes</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2017,29 +2557,29 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Albemarle Corporation</t>
+          <t>Publicis Sapient</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Data Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -2048,19 +2588,19 @@
         <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core data‑product keywords.</t>
+          <t>The JD demands 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks core domain keywords like 'Equity Derivatives' and 'Capital Markets'.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>data governance, data quality, enterprise reporting, cloud‑native analytics, SQL, Snowflake, OKRs, RICE prioritization</t>
+          <t>Equity Derivatives, Capital Markets, Banking, Financial Services, process mapping, risk management, project plan, milestones</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2083,24 +2623,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Blue Spire Inc</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - HR Technology</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2109,24 +2649,26 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules apply because the JD requires 10+ years and senior level, while the candidate has only 4 years; therefore both scores are forced below 30, with the biggest keyword gap being lack of Amazon Connect/LLM specific terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Amazon Connect, Amazon Lex, Large Language Models (LLMs), IVR, call containment, first contact resolution (FCR), AWS, product roadmap</t>
+          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2149,50 +2691,50 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>MSD</t>
+          <t>Blue Spire Inc</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Ruminant</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+          <t>Hard rules apply because the JD requires 10+ years and senior level, while the candidate has only 4 years; therefore both scores are forced below 30, with the biggest keyword gap being lack of Amazon Connect/LLM specific terms.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+          <t>Amazon Connect, Amazon Lex, Large Language Models (LLMs), IVR, call containment, first contact resolution (FCR), AWS, product roadmap</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2206,87 +2748,219 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Innova ESI</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Capability Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>MSD</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Ruminant</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>FBS Agile Product Manager III- Guidewire</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. The most important keyword gap is the lack of explicit "Scrum" and "Product Owner" terminology.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Scrum, Product Owner, SOX compliance, Release Train Engineer, Scaled Agile Framework (SAFe), AS400, claim adjudication</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
+      <c r="H17" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any Guidewire or Rally experience.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Guidewire, Rally, Cloud, Lean business case, Nonfunctional Requirements (NFRs), Agile Release Train (ART), Program Kanban, Enterprise vision roadmap</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2306,6 +2980,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-24
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Autofleet</t>
+          <t>Versatile Club Employer of Record</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -593,12 +593,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is a close match, so hard rules pass. The resume contains most core SaaS and Agile keywords but lacks several JD‑specific tools and frameworks.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflicts, so hard rules pass; the resume covers most core JD keywords but lacks explicit mentions of product roadmap, PRD, backlog grooming and analytics tools.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>product roadmap, PRD, backlog grooming, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,19 +621,19 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Superleap AI CRM</t>
+          <t>Smart Food Safe</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -647,26 +647,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title level is acceptable, yielding solid ATS and fit scores; the most important keyword gap is the lack of ARR/MRR/churn metrics.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>ARR, MRR, churn, roadmap planning, OKRs, market trends analysis</t>
+          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,24 +687,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>WisdomAI</t>
+          <t>Onsurity</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,24 +713,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
+          <t>The resume meets the years and title requirements, but lacks several JD‑specific tools and processes (e.g., Mixpanel/Amplitude, PRDs, competitor tracking), lowering the ATS score; domain mismatch with healthcare benefits reduces the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
+          <t>Mixpanel, Amplitude, Google Analytics, PRD, competitor analysis, marketing coordination, sales coordination</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,17 +750,17 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -826,19 +826,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>eReleGo Technologies Pvt Ltd (ETPL)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - AI PM</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,7 +847,9 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
@@ -859,12 +861,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2+ years requirement and has relevant GenAI and SaaS experience, but the resume lacks several JD-specific AI tooling keywords, lowering the ATS score.</t>
+          <t>The resume meets the 3‑year minimum and title level, but misses several JD‑specific terms such as GTM strategy, product demos, and PRDs, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Cursor, Claude Code, Replit, n8n, MCPs, AI agents, tool calling, LLM evaluation, OKRs</t>
+          <t>GTM strategy, product demos, deal closure support, PRD (Product Requirement Document), market trends analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,7 +884,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -892,19 +894,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>eReleGo Technologies Pvt Ltd (ETPL)</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II - AI PM</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -913,9 +915,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
@@ -927,12 +927,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title level, but misses several JD‑specific terms such as GTM strategy, product demos, and PRDs, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+          <t>The candidate meets the 2+ years requirement and has relevant GenAI and SaaS experience, but the resume lacks several JD-specific AI tooling keywords, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>GTM strategy, product demos, deal closure support, PRD (Product Requirement Document), market trends analysis</t>
+          <t>Cursor, Claude Code, Replit, n8n, MCPs, AI agents, tool calling, LLM evaluation, OKRs</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -960,19 +960,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Applied Materials India</t>
+          <t>Asymmetric Labs</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Associate Product Manager(Technical)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -981,24 +981,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and has no senior title conflict, but the resume lacks several core JD keywords (e.g., Python, product roadmap, supply chain), lowering the ATS score while still showing good overall fit.</t>
+          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Python, product roadmap, supply chain, manufacturing operations, data pipelines, scalable architecture, OKRs, quantitative opportunity sizing</t>
+          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1021,24 +1023,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Empower India</t>
+          <t>Accenture in India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1047,24 +1049,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience and seniority requirements, but lacks several JD-specific keywords such as A/B testing and product roadmap, lowering the ATS score; the domain shift from SaaS/enterprise tools to financial services creates a moderate fit gap.</t>
+          <t>The resume meets the 3‑year minimum and title level, but lacks several core JD terms (e.g., Personal Insurance, product backlog) resulting in a moderate ATS score; domain mismatch with insurance lowers the fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Usability testing, Customer research, Product roadmap, Compliance, Key performance indicators (KPIs), OKRs, Product strategy</t>
+          <t>Personal Insurance, product backlog, roadmap, human‑centered design, feedback loops</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,92 +1086,90 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chevron</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner</t>
+          <t>Applied AI Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and contains most of the JD keywords, but lacks several specific tools and frameworks; the biggest gap is the absence of OKR/metrics terminology.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific terms like roadmap, OKRs, and integration, lowering the ATS score; domain alignment is moderate but not a direct energy‑wells focus.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, OKRs, KPIs, integration with IT systems, digital platform governance, release management, value‑based prioritization</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SAYZO</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1177,30 +1179,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years and title requirements, but lacks many core JD keywords (e.g., GA4, Mixpanel, A/B testing), lowering the ATS score; the biggest gap is the absence of explicit growth‑experiment terminology.</t>
+          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, GA4, Mixpanel, Amplitude, Growth loops, PLG, CAC, LTV, Cohort analysis, Dashboard (GA4/Amplitude)</t>
+          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1223,24 +1223,24 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Codeft Digital</t>
+          <t>StarRez, Inc.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1249,26 +1249,24 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H12" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has a matching title, but lacks the specific tool Zoho Projects mentioned in the JD, creating the biggest keyword gap.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Zoho Projects, A/B testing, OKRs, RICE prioritization, NPS improvement</t>
+          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,7 +1284,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1296,19 +1294,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EchorTech</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1317,26 +1315,24 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior title triggers hard rules; most JD keywords are present but key terms like "product roadmap", "API integration" and "PRD" are missing.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>API integration, product roadmap, PRD (Product Requirements Document), product analytics tool (e.g., Mixpanel), OKRs or RICE prioritization</t>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1354,29 +1350,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>StarRez, Inc.</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>FBS Product Owner III- Guidewire</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1387,22 +1383,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
+          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1420,7 +1416,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1430,19 +1426,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>TriNet</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1456,19 +1452,19 @@
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1486,55 +1482,55 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>FBS Product Owner III- Guidewire</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
+          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,219 +1544,21 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Kanerika Inc</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but lacks several enterprise‑focused keywords such as privacy and data‑governance, lowering the ATS score; the strongest gap is the absence of privacy/compliance terminology.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>privacy, data governance, risk compliance, AI governance, API integration, personas, permissions, product roadmap, OKRs</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TriNet</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Qualys</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -1781,9 +1579,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1795,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1950,7 +1745,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -1960,7 +1755,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2018,7 +1813,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -2028,19 +1823,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GE Vernova</t>
+          <t>Rippling</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Manager, Payroll Integrations</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2051,22 +1846,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title or explicit 5+ year requirement), but the resume lacks many JD-specific terms and the title does not align closely, lowering the ATS score; the biggest keyword gap is the absence of program‑management terminology like NPI/CTQ.</t>
+          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>NPI (New Product Introduction), CTQ (Critical to Quality), budget management, program management, dashboards, metrics reporting, OKRs, cross‑functional program coordination</t>
+          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2084,29 +1879,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Jupiter</t>
+          <t>GE Vernova</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Unsecured Lending</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2115,26 +1910,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>55</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and has relevant product management experience, but the resume lacks many fintech lending-specific keywords and domain experience, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title or explicit 5+ year requirement), but the resume lacks many JD-specific terms and the title does not align closely, lowering the ATS score; the biggest keyword gap is the absence of program‑management terminology like NPI/CTQ.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>underwriting, KYC, RBI Digital Lending Guidelines, loan origination, risk compliance, personal loans, salary advances, approval rate, NPA, ROA</t>
+          <t>NPI (New Product Introduction), CTQ (Critical to Quality), budget management, program management, dashboards, metrics reporting, OKRs, cross‑functional program coordination</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2157,52 +1950,52 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Freight Tiger</t>
+          <t>Peak XV Partners</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Founding Product Manager | Early-Stage AI Cyber-Sec Portfolio Company</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum and no senior title). The resume contains many generic product management keywords but lacks logistics‑specific terms such as freight invoicing, ERP integration, and payments, leading to a moderate ATS score and only a tangential domain fit.</t>
+          <t>The resume meets the years requirement and title level, but lacks many core cyber‑security and early‑stage startup keywords, resulting in a modest ATS score and only moderate overall fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>freight invoicing, payment reconciliation, ERP integration (SAP, Oracle, Tally), B2B payments workflow, logistics platform scalability, predictive AI models, anomaly detection, NPS tracking, financial integrations (banks, NBFCs, payment gateways)</t>
+          <t>cybersecurity, go-to-market, roadmap, founding product manager, startup, product strategy, design direction, technical product development</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2220,29 +2013,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Pharmed Limited</t>
+          <t>Societe Generale Global Solution Centre</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
+          <t>Product Owner-MS Proxy PO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2251,26 +2044,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many Microsoft 365 specific keywords, resulting in a low ATS score; the biggest gap is the absence of any mention of Teams, Exchange, OneDrive or SharePoint.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
+          <t>Microsoft Teams, Exchange Online, OneDrive for Business, SharePoint Online, Azure integration, O365 licensing and governance, backlog grooming, sprint planning</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2293,24 +2084,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Cashfree</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Customer Support API Platform</t>
+          <t>Product Manager- 2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2319,24 +2110,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any API or integration platform experience.</t>
+          <t>The candidate meets the 3‑year minimum (4 years experience) so hard rules do not apply, but the resume lacks most payment‑specific keywords and domain experience, resulting in a low ATS score and only a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>API design, microservices, cloud platform, developer engagement, API governance, security standards, platform roadmap</t>
+          <t>UPI, merchant acquiring, payment gateway, API integration, NPCI guidelines, transaction processing, payment regulations, refund workflow, FinTech, customer insights</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2354,29 +2147,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Comviva</t>
+          <t>Pharmed Limited</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2385,24 +2178,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
+          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
+          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2420,7 +2215,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2430,45 +2225,45 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>IGEL Technology</t>
+          <t>Moneyview</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Bangalore</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 6+ years of enterprise product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of explicit analytics/observability experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most fintech‑specific keywords such as lending, loan origination, RBI/AML compliance, and Python/BigQuery, resulting in a low ATS match; the biggest gap is the absence of any fintech or lending domain experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>analytics platform, observability, endpoint telemetry, cloud/SaaS offering, AI-driven insights</t>
+          <t>Fintech, Lending, Credit product, Loan origination, Underwriting, RBI regulations, KYC/AML compliance, Python, BigQuery, AI/ML workflow</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2491,12 +2286,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2303,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – PBM / Pharmacy Benefits</t>
+          <t>Product Owner(healthcare domain)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2519,22 +2314,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience while the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks core pharmacy‑benefits terminology.</t>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any PBM/pharmacy or Rx domain terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy Benefits Management (PBM), Rx formulary management, Drug data analysis, MS Access, Stakeholder presentations / release notes</t>
+          <t>PBM experience, pharmacy domain knowledge, Rx formulary management, project management methodology (requirements, design, test, implementation), MS Excel advanced data analysis</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2557,50 +2352,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Publicis Sapient</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Customer Support API Platform</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks core domain keywords like 'Equity Derivatives' and 'Capital Markets'.</t>
+          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any API or integration platform experience.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Equity Derivatives, Capital Markets, Banking, Financial Services, process mapping, risk management, project plan, milestones</t>
+          <t>API design, microservices, cloud platform, developer engagement, API governance, security standards, platform roadmap</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2618,57 +2413,55 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>Comviva</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - HR Technology</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="G13" s="2" t="n">
-        <v>27</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
+          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
+          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2682,38 +2475,38 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Blue Spire Inc</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Snr Product manager - Customer Platforms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -2729,12 +2522,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules apply because the JD requires 10+ years and senior level, while the candidate has only 4 years; therefore both scores are forced below 30, with the biggest keyword gap being lack of Amazon Connect/LLM specific terms.</t>
+          <t>The JD title includes 'Snr', triggering the senior-role hard rule, so both scores must be below 30; the resume lacks several key VOC platform keywords.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Amazon Connect, Amazon Lex, Large Language Models (LLMs), IVR, call containment, first contact resolution (FCR), AWS, product roadmap</t>
+          <t>Medallia, MMX, voice of the customer (VOC), OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2748,33 +2541,33 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Owner - Digital Lab Platform</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2785,22 +2578,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
+          <t>The resume meets the experience requirement (4 years) and title seniority rules, but it lacks many JD‑specific terms (lab, data governance, UAT, training, roadmap) resulting in a modest ATS score and only a moderate fit.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
+          <t>lab execution systems, data governance, enterprise architecture, user acceptance testing (UAT), training materials, roadmap planning, backlog prioritization, process development</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2823,50 +2616,50 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MSD</t>
+          <t>Reckitt</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Ruminant</t>
+          <t>IT&amp;D Product Manager, P2P and Strategic Purchasing</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+          <t>Hard rules pass, but the resume lacks many procurement‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of Source‑to‑Pay and procurement terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+          <t>Source-to-Pay, procurement strategy, contracting lifecycle, KPIs and adoption metrics, roadmap ownership</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2880,87 +2673,353 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - HR Technology</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>JPMorganChase</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>MSD</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Ruminant</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Worldpay</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Digital Products, Payments) - Pune – 7+ years Exp</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 7+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key payment‑portal terms like 'payout tracking' and 'reconciliation' are missing.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>payout tracking, payment status tracking, dispute management, merchant self‑service, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>Capgemini</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>FBS Agile Product Manager III- Guidewire</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any Guidewire or Rally experience.</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Guidewire, Rally, Cloud, Lean business case, Nonfunctional Requirements (NFRs), Agile Release Train (ART), Program Kanban, Enterprise vision roadmap</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2982,6 +3041,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-25
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versatile Club Employer of Record</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Ground Transport)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,24 +581,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F2" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflicts, so hard rules pass; the resume covers most core JD keywords but lacks explicit mentions of product roadmap, PRD, backlog grooming and analytics tools.</t>
+          <t>The candidate meets the 4-year requirement and has a closely aligned title, yielding a solid ATS score despite missing several JD-specific tools and frameworks; the strongest keyword gap is the lack of A/B testing/OKR experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, PRD, backlog grooming, A/B testing, Mixpanel, NPS improvement</t>
+          <t>A/B testing, OKRs, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,19 +623,19 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Smart Food Safe</t>
+          <t>Superleap AI CRM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -649,22 +651,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
+          <t>The candidate meets the 4-year experience requirement and title level is acceptable, yielding solid ATS and fit scores; the most important keyword gap is the lack of ARR/MRR/churn metrics.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
+          <t>ARR, MRR, churn, roadmap planning, OKRs, market trends analysis</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Onsurity</t>
+          <t>Smart Food Safe</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -713,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years and title requirements, but lacks several JD‑specific tools and processes (e.g., Mixpanel/Amplitude, PRDs, competitor tracking), lowering the ATS score; domain mismatch with healthcare benefits reduces the fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, Google Analytics, PRD, competitor analysis, marketing coordination, sales coordination</t>
+          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Mouser</t>
+          <t>Onsurity</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,24 +781,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the seniority level, but lacks several specific JD terms such as scrum master and change control. The most important gap is the absence of explicit Scrum Master / change control experience.</t>
+          <t>The resume meets the years and title requirements, but lacks several JD‑specific tools and processes (e.g., Mixpanel/Amplitude, PRDs, competitor tracking), lowering the ATS score; domain mismatch with healthcare benefits reduces the fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>scrum master, change control procedures, mockups, flowcharts, process diagrams, project schedule, business acumen</t>
+          <t>Mixpanel, Amplitude, Google Analytics, PRD, competitor analysis, marketing coordination, sales coordination</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +818,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>eReleGo Technologies Pvt Ltd (ETPL)</t>
+          <t>Blitz</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,22 +853,22 @@
         <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title level, but misses several JD‑specific terms such as GTM strategy, product demos, and PRDs, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, so hard rules do not penalize. Strong overlap on core product management keywords but missing key JD terms like A/B testing and roadmap planning lowers the ATS score. Domain experience is solid in SaaS and enterprise tools but not directly in same‑day delivery logistics, resulting in a moderate fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>GTM strategy, product demos, deal closure support, PRD (Product Requirement Document), market trends analysis</t>
+          <t>A/B testing, product metrics, roadmap planning, PRD (Product Requirement Document), analytics tools (e.g., Mixpanel), experiment design</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -884,17 +886,17 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -960,19 +962,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Asymmetric Labs</t>
+          <t>eReleGo Technologies Pvt Ltd (ETPL)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(Technical)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -982,25 +984,25 @@
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
+          <t>The resume meets the 3‑year minimum and title level, but misses several JD‑specific terms such as GTM strategy, product demos, and PRDs, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
+          <t>GTM strategy, product demos, deal closure support, PRD (Product Requirement Document), market trends analysis</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,29 +1020,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Accenture in India</t>
+          <t>SuperKalam (YC W23)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Founding Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1056,19 +1058,19 @@
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title level, but lacks several core JD terms (e.g., Personal Insurance, product backlog) resulting in a moderate ATS score; domain mismatch with insurance lowers the fit score.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks several JD‑specific tools and growth‑focused terms, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Personal Insurance, product backlog, roadmap, human‑centered design, feedback loops</t>
+          <t>PostHog, A/B testing, growth experiments, vibe coding, product‑led growth, conversion rate optimization, user activation metrics, structured communication</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1091,50 +1093,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Applied Materials India</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Applied AI Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains most of the JD keywords, but lacks several specific tools and frameworks; the biggest gap is the absence of OKR/metrics terminology.</t>
+          <t>The candidate meets the 4-year experience requirement and has no senior title conflict, but the resume lacks several core JD keywords (e.g., Python, product roadmap, supply chain), lowering the ATS score while still showing good overall fit.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>Python, product roadmap, supply chain, manufacturing operations, data pipelines, scalable architecture, OKRs, quantitative opportunity sizing</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,59 +1150,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Techdome</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager AI</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
+          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,7 +1216,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1223,50 +1225,52 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>StarRez, Inc.</t>
+          <t>Olyv</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title level, but the resume lacks several fintech‑specific terms from the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>LMS, LOS, collections module, risk mitigation, product roadmap, automation workflows, integration, FinTech lending</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1280,38 +1284,38 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager - Assisted Service</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1320,19 +1324,19 @@
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI keywords but lacks several marketplace‑specific terms, lowering the ATS score; the biggest gap is the absence of financial‑services and risk‑management language.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
+          <t>Financial Services, Risk Management, Trust &amp; Safety, AI‑powered decision flows, Customer Support tools, Marketplace dynamics, Two‑sided platform, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,59 +1350,61 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Asymmetric Labs</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FBS Product Owner III- Guidewire</t>
+          <t>Associate Product Manager(Technical)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+          <t>The resume meets the hard rules, but only about half of the JD's specific technical keywords (e.g., React, Python, AI coding tools) appear, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well with the role, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
+          <t>React, Python, AI coding tools (Cursor, Claude Code, Replit), experiment design and A/B testing, success metrics definition</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1412,38 +1418,38 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager III, Technical, Amazon Fulfillment Technologies (AFT)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -1459,12 +1465,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). ATS score is moderate due to strong keyword overlap on tools and methodologies but missing many fulfillment‑specific terms. Fit score is lower because the candidate's domain (SaaS, travel, FMCG) only tangentially aligns with Amazon Fulfillment routing and mansort.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>Routing, Mansort, SCOT, Delivery Estimate Accuracy, self‑healing, scalable architecture, operations safety, A/B testing, Snowflake, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1478,28 +1484,28 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Qualys</t>
+          <t>Abracon</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1509,56 +1515,850 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F16" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Years of experience meet the 3‑year minimum and the title aligns, so hard rules pass; however the resume lacks key JD terms like go‑to‑market, revenue growth, and profitability, lowering the ATS score. Domain mismatch between hardware components and the candidate's SaaS/GenAI focus reduces the fit score.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>go-to-market strategy, revenue growth, profitability analysis, sales enablement, customer support, end-of-life management</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Ralph Lauren</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager-2</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, SQL, Power BI, Agile) but misses several JD‑specific terms like KPIs, dashboards, and data‑product metrics, lowering the ATS score. Domain fit is moderate; the candidate excels in SaaS and GenAI but lacks direct data‑product analytics experience.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Applied AI Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and contains most of the JD keywords, but lacks several specific tools and frameworks; the biggest gap is the absence of OKR/metrics terminology.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Franklin Templeton</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Techdome</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>StarRez, Inc.</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Anaqua</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
+      <c r="H22" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but lacks several JD-specific terms like product backlog and AI automation agents, leading to a moderate ATS score. Domain alignment is good with SaaS and enterprise experience.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>product backlog, backlog refinement, roadmap prioritization, intellectual property management, AI automation agents</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Amgen</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Data Assets Platform</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many relevant terms but misses several core JD keywords such as roadmap, governance, and UAT, limiting the ATS score. The strongest keyword gap is the lack of explicit 'roadmap' and 'governance' language.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>roadmap, governance, UAT, release readiness, metrics, data platform, backlog, product vision</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TriNet</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Backbase</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core JD terms such as workflow automation and AI agents, lowering the ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a decent fit.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>workflow automation, AI agents, data connectors, MVP definition, competitive positioning, real-time data integration, OKRs</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>tripstack</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Virtual Interlining</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title is a close match, but the resume lacks several JD‑specific terms such as API, payments, and virtual interlining, lowering the ATS score. Domain experience in travel tech and SaaS is strong, giving a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>API integration, payments processing, fraud prevention, pricing optimization, virtual interlining, B2B SaaS platform, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>MaxIQ</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns, but the resume lacks several JD‑specific terms such as product roadmap and analytics, lowering the ATS score; overall domain and skill fit are strong.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Product Roadmap, Analytics/Reporting, Scalability, Sales Enablement, Product Marketing, Competitive Landscape, Metrics measurement</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Copeland</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1579,6 +2379,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1590,7 +2402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1696,7 +2508,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bytebeam</t>
+          <t>xpat.money</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1706,28 +2518,30 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F2" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many JD-specific terms like fleet, telematics, OTA updates, resulting in a moderate ATS score and only partial domain fit.</t>
+          <t>The resume meets the years requirement (4 years vs 1‑3 years) and seniority constraints, but lacks key fintech and growth‑focused keywords, lowering both scores.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>fleet owners, telemetry, remote diagnostics, OTA updates, IoT, telematics, customer advisory board, OKRs, guardrail, A/B testing</t>
+          <t>Fintech, Payments, Product Metrics, User Funnel Analysis, Growth Activation, PRD, A/B testing</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1745,29 +2559,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Zepto</t>
+          <t>Qure.ai</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager – Planning</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1780,22 +2594,22 @@
         <v>3</v>
       </c>
       <c r="F3" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks many core JD keywords such as Python, pandas, forecasting and inventory‑planning terms, lowering the ATS score; the biggest gap is the absence of Python/pandas experience.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum). The resume contains many Agile and GenAI terms but lacks healthcare‑specific deployment and regulatory keywords, lowering the ATS score; the biggest gap is the absence of clinical/IT deployment terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Python, pandas, numpy, forecasting, inventory management, root‑cause analysis, dashboards, SQL window functions, data visualization libraries</t>
+          <t>clinical stakeholder management, IT integration and deployment, post‑deployment stabilization, guardrails for AI workflows, US market regulatory compliance, FDA clearance experience</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1813,29 +2627,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Rippling</t>
+          <t>Bytebeam</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Payroll Integrations</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1849,19 +2663,19 @@
         <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many JD-specific terms like fleet, telematics, OTA updates, resulting in a moderate ATS score and only partial domain fit.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
+          <t>fleet owners, telemetry, remote diagnostics, OTA updates, IoT, telematics, customer advisory board, OKRs, guardrail, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1879,29 +2693,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GE Vernova</t>
+          <t>Zepto</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Associate Product Manager – Planning</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1910,24 +2724,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title or explicit 5+ year requirement), but the resume lacks many JD-specific terms and the title does not align closely, lowering the ATS score; the biggest keyword gap is the absence of program‑management terminology like NPI/CTQ.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks many core JD keywords such as Python, pandas, forecasting and inventory‑planning terms, lowering the ATS score; the biggest gap is the absence of Python/pandas experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>NPI (New Product Introduction), CTQ (Critical to Quality), budget management, program management, dashboards, metrics reporting, OKRs, cross‑functional program coordination</t>
+          <t>Python, pandas, numpy, forecasting, inventory management, root‑cause analysis, dashboards, SQL window functions, data visualization libraries</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1945,57 +2761,55 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Peak XV Partners</t>
+          <t>FIS</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Founding Product Manager | Early-Stage AI Cyber-Sec Portfolio Company</t>
+          <t>Technical Product Owner - Sales Technology &amp; AI</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>53</v>
-      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years requirement and title level, but lacks many core cyber‑security and early‑stage startup keywords, resulting in a modest ATS score and only moderate overall fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many JD-specific platform and tool keywords, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate job fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>cybersecurity, go-to-market, roadmap, founding product manager, startup, product strategy, design direction, technical product development</t>
+          <t>Seismic, Responsive, LinkedIn Sales Navigator, SSO configuration, vendor management, renewal intelligence dashboards, AI agent configuration</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2018,24 +2832,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Societe Generale Global Solution Centre</t>
+          <t>Rippling</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner-MS Proxy PO</t>
+          <t>Product Manager, Payroll Integrations</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2046,22 +2860,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many Microsoft 365 specific keywords, resulting in a low ATS score; the biggest gap is the absence of any mention of Teams, Exchange, OneDrive or SharePoint.</t>
+          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Teams, Exchange Online, OneDrive for Business, SharePoint Online, Azure integration, O365 licensing and governance, backlog grooming, sprint planning</t>
+          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2079,29 +2893,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Cashfree</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- 2</t>
+          <t>Product Manager -Platform</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2110,26 +2924,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (4 years experience) so hard rules do not apply, but the resume lacks most payment‑specific keywords and domain experience, resulting in a low ATS score and only a moderate job‑fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with JD-specific terms like access‑control, API, and HLDs; the most important gap is the lack of platform‑security keywords. Fit score reflects some relevance (GenAI, enterprise SaaS) but a domain mismatch with cybersecurity platform responsibilities.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>UPI, merchant acquiring, payment gateway, API integration, NPCI guidelines, transaction processing, payment regulations, refund workflow, FinTech, customer insights</t>
+          <t>access control, permissioning, API, high‑level design (HLD), prototype, proof of concept, multi‑tenant, developer platform, MCP</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2152,24 +2964,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Pharmed Limited</t>
+          <t>UST</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Assistant Product Manager - Pharmaceuticals (Ortho Portfolio)</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2178,26 +2990,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
         <v>48</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and location requirements, but the resume lacks many pharma‑specific marketing keywords and domain experience, leading to low ATS and fit scores; the biggest gap is the absence of pharmaceutical brand management terminology.</t>
+          <t>Hard rules are satisfied, but the resume lacks many manufacturing and GxP-specific keywords required by the JD, leading to a low ATS score; the biggest gap is the absence of pharma/GxP terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>pharmaceutical brand management, marketing strategy development, promotional material creation, fieldwork with sales team, market insights gathering, competitive activity tracking, conference and CME participation, presentation skills</t>
+          <t>GxP regulations, GMP, GAMP 5, 21 CFR Part 11, CSV, manufacturing operations, product roadmaps, backlog management, change management, discovery workshops</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2215,29 +3025,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Moneyview</t>
+          <t>AppsForBharat</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2248,22 +3058,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most fintech‑specific keywords such as lending, loan origination, RBI/AML compliance, and Python/BigQuery, resulting in a low ATS match; the biggest gap is the absence of any fintech or lending domain experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is low due to missing core JD keywords like SEO, web analytics, and growth frameworks; title is one level below the target. Fit score is moderate because product management skills transfer but the domain (faith‑tech web consumer) differs from the candidate's B2B SaaS and travel tech background.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Fintech, Lending, Credit product, Loan origination, Underwriting, RBI regulations, KYC/AML compliance, Python, BigQuery, AI/ML workflow</t>
+          <t>SEO, Web analytics (e.g., Mixpanel, Google Analytics), A/B testing, Growth metrics (MAU, NPS), P&amp;L ownership, OKRs, Retention and monetization strategy</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2281,29 +3091,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Innova ESI</t>
+          <t>Cashfree</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner(healthcare domain)</t>
+          <t>Product Manager- 2</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2312,24 +3122,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any PBM/pharmacy or Rx domain terminology.</t>
+          <t>The candidate meets the 3‑year minimum (4 years experience) so hard rules do not apply, but the resume lacks most payment‑specific keywords and domain experience, resulting in a low ATS score and only a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>PBM experience, pharmacy domain knowledge, Rx formulary management, project management methodology (requirements, design, test, implementation), MS Excel advanced data analysis</t>
+          <t>UPI, merchant acquiring, payment gateway, API integration, NPCI guidelines, transaction processing, payment regulations, refund workflow, FinTech, customer insights</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2347,7 +3159,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2357,19 +3169,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Customer Support API Platform</t>
+          <t>Product Manager (Data Governance Platform, Metadata Management, Data Stewardship, Access Management) (6-12 years)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2380,22 +3192,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any API or integration platform experience.</t>
+          <t>The resume meets basic hard rules but lacks many core data governance keywords, resulting in a modest ATS score; the biggest gap is missing data governance and metadata management terms.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>API design, microservices, cloud platform, developer engagement, API governance, security standards, platform roadmap</t>
+          <t>data catalog, metadata management, data lineage, data quality, access management, stewardship, data governance framework, Snowflake, OKRs</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2413,29 +3225,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Comviva</t>
+          <t>CogniVed Solutions</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager – OpenShift</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2449,19 +3261,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9‑14 years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any mention of model registry, versioning, or drift detection.</t>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any OpenShift or container platform terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>model registry, versioning, drift detection, real‑time model scoring, agent authoring tools, workflow builder, decision orchestration engine</t>
+          <t>OpenShift, container platforms, cloud‑native technologies, on‑premise cloud, platform KPIs / SLIs / SLOs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2479,55 +3291,57 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Zaggle</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Snr Product manager - Customer Platforms</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'Snr', triggering the senior-role hard rule, so both scores must be below 30; the resume lacks several key VOC platform keywords.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum). The resume contains many relevant terms but misses several core fintech and P2P-specific keywords, lowering the ATS score; the biggest gap is the lack of procure‑to‑pay and payments terminology.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Medallia, MMX, voice of the customer (VOC), OKRs, NPS improvement</t>
+          <t>Procure-to-Pay, FinTech payments integration, Client onboarding, Renewals management, OKRs, RICE prioritization, A/B testing, NPS improvement, Snowflake</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2541,7 +3355,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -2550,12 +3364,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2611,7 +3425,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2621,7 +3435,7 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2677,7 +3491,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -2687,19 +3501,19 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>AVEVA</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - HR Technology</t>
+          <t>Product Owner, Electrical Engineering Software</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2708,26 +3522,24 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
+          <t>Hard rules pass, but the resume lacks core electrical engineering and CAD terminology required by the JD, resulting in very low keyword overlap and poor domain fit.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
+          <t>electrical engineering requirements, single-line diagrams, schematic and wiring diagrams, cable schedules, IEC/BS/IEEE standards, CAD‑based design workflow, panel drawings</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2745,29 +3557,29 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager - HR Technology</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2776,24 +3588,26 @@
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
+          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2816,50 +3630,50 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MSD</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Ruminant</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2873,59 +3687,59 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Worldpay</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Digital Products, Payments) - Pune – 7+ years Exp</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key payment‑portal terms like 'payout tracking' and 'reconciliation' are missing.</t>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>payout tracking, payment status tracking, dispute management, merchant self‑service, regulatory compliance</t>
+          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2939,59 +3753,59 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Talentmatics</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>FBS Agile Product Manager III- Guidewire</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G21" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H21" s="2" t="n">
-        <v>26</v>
-      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any Guidewire or Rally experience.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of CRM/SalesTech or revenue intelligence experience.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Guidewire, Rally, Cloud, Lean business case, Nonfunctional Requirements (NFRs), Agile Release Train (ART), Program Kanban, Enterprise vision roadmap</t>
+          <t>CRM, SalesTech, Revenue Intelligence, customer acquisition metrics (e.g., NPS, MAU growth), A/B testing, OKRs, Mixpanel, predictive analytics</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3009,17 +3823,347 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Worldpay</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Digital Products, Payments) - Pune – 7+ years Exp</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 7+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key payment‑portal terms like 'payout tracking' and 'reconciliation' are missing.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>payout tracking, payment status tracking, dispute management, merchant self‑service, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Global Payments Inc.</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Digital Products, Payments) - Pune – 7+ years Exp</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 7+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. The most important keyword gap is the lack of any payments‑specific terminology such as 'payout tracking' or 'reconciliation'.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>payout tracking, payment status tracking, dispute management, merchant self‑service, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>FBS Agile Product Manager III- Guidewire</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any Guidewire or Rally experience.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Guidewire, Rally, Cloud, Lean business case, Nonfunctional Requirements (NFRs), Agile Release Train (ART), Program Kanban, Enterprise vision roadmap</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>HSBC</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Snr Product manager - Customer Platforms</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The JD title includes 'Snr', triggering the senior-role hard rule, so both scores must be below 30; the resume lacks several key VOC platform keywords.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Medallia, MMX, voice of the customer (VOC), OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Syneos Health</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Product Manager (Salesforce)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Serilingampalli, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because core marketing product keywords like Salesforce, MarTech, ABM, lead capture, and campaign management are missing. Fit score is low due to domain mismatch—candidate’s experience is in SaaS and GenAI, not B2B marketing platforms.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce, MarTech, ABM, lead capture, campaign management, attribution, marketing platform integration, demand generation</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -3045,6 +4189,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-09-29
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>dentsu</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Ground Transport)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,9 +647,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
@@ -661,12 +659,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year requirement and has a closely aligned title, yielding a solid ATS score despite missing several JD-specific tools and frameworks; the strongest keyword gap is the lack of A/B testing/OKR experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core keywords but lacks several JD‑specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, Snowflake, NPS improvement</t>
+          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Blitz</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,26 +713,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>68</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>74</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, so hard rules do not penalize. Strong overlap on core product management keywords but missing key JD terms like A/B testing and roadmap planning lowers the ATS score. Domain experience is solid in SaaS and enterprise tools but not directly in same‑day delivery logistics, resulting in a moderate fit score.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the seniority level, but lacks several specific JD terms such as scrum master and change control. The most important gap is the absence of explicit Scrum Master / change control experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, product metrics, roadmap planning, PRD (Product Requirement Document), analytics tools (e.g., Mixpanel), experiment design</t>
+          <t>scrum master, change control procedures, mockups, flowcharts, process diagrams, project schedule, business acumen</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +748,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - SaaS- 4 to 6 Years</t>
+          <t>Product Manager, Glean Protect (Security &amp; Governance)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,26 +779,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume matches most core keywords and the required experience level, but lacks several specific tool and pricing/monetization terms from the JD, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several core JD terms like LLM, security, and governance, lowering the ATS score. Domain and skill overlap are solid but not a perfect match for the security/governance focus.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, REST APIs, Pricing strategy, API monetization, Confluence, Looker Studio, Tableau, Customer discovery</t>
+          <t>LLM, APIs, security governance, knowledge management, OKRs, A/B testing, enterprise search</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,29 +814,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Recruiterflow</t>
+          <t>Kadence</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager – Website Growth</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,24 +845,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, correct seniority and location). The resume covers many core keywords but misses several JD‑specific terms like product roadmap and quantitative analysis, limiting the ATS score. Overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several core website‑growth tools and e‑commerce terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product marketing, customer success, quantitative analysis, qualitative insights, user research, documentation, prototyping, UAT</t>
+          <t>Google Analytics 4, Google Search Console, Microsoft Clarity, Hotjar, A/B testing, Conversion Rate Optimization (CRO), Average Order Value (AOV), Customer Retention, E‑commerce, Website roadmap</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,34 +882,34 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L1</t>
+          <t>Global Product Manager, Antibody Solutions</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -922,19 +918,19 @@
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,29 +948,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SuperKalam (YC W23)</t>
+          <t>Bluevine</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Founding Product Manager</t>
+          <t>Product Manager II (Lending &amp; Credit)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -983,26 +979,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks several JD‑specific tools and growth‑focused terms, lowering the ATS score.</t>
+          <t>The resume meets the hard rules but lacks many fintech‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of payments/collections terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>PostHog, A/B testing, growth experiments, vibe coding, product‑led growth, conversion rate optimization, user activation metrics, structured communication</t>
+          <t>payments, collections, lending, capital markets, risk management, compliance, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1020,55 +1014,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Franklin Templeton</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager AI</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
+          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
+          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,38 +1076,38 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Glean Protect (Security &amp; Governance)</t>
+          <t>PRODUCT MANAGER L1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1122,19 +1116,19 @@
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several core JD terms like LLM, security, and governance, lowering the ATS score. Domain and skill overlap are solid but not a perfect match for the security/governance focus.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>LLM, APIs, security governance, knowledge management, OKRs, A/B testing, enterprise search</t>
+          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,7 +1142,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1157,97 +1151,95 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>OnArrival</t>
+          <t>State Street</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Flights)</t>
+          <t>Product Owner - Assistant Vice President</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard‑rule criteria (4 years experience, no senior title, no 5+ year requirement). It contains many relevant keywords but misses several core JD terms such as KPIs and roadmap, leading to a moderate ATS score. The candidate’s SaaS and GenAI background aligns reasonably well with the data‑centric product focus.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>KPIs, roadmap, release plan, risk management, dependency tracking, data visualization, dashboard, trade‑off decisions, performance metrics</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, but the resume lacks many JD‑specific keywords such as search, payments, and AI‑assisted prototyping, lowering the ATS score. Domain experience in travel tech and GenAI is strong, giving a solid fit score.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>search optimization, payment integration, post‑booking experience, A/B testing, success metrics (e.g., conversion rate, NPS), LLM evaluation and monitoring, OKRs or similar goal‑setting framework, edge‑case matrix, AI‑assisted prototyping</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>TriNet</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager III, Technical, Amazon Fulfillment Technologies (AFT)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -1263,12 +1255,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). ATS score is moderate due to strong keyword overlap on tools and methodologies but missing many fulfillment‑specific terms. Fit score is lower because the candidate's domain (SaaS, travel, FMCG) only tangentially aligns with Amazon Fulfillment routing and mansort.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Routing, Mansort, SCOT, Delivery Estimate Accuracy, self‑healing, scalable architecture, operations safety, A/B testing, Snowflake, OKRs</t>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1282,61 +1274,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Abracon</t>
+          <t>tripstack</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Years of experience meet the 3‑year minimum and the title aligns, so hard rules pass; however the resume lacks key JD terms like go‑to‑market, revenue growth, and profitability, lowering the ATS score. Domain mismatch between hardware components and the candidate's SaaS/GenAI focus reduces the fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant product and SaaS keywords but misses several operational and flight‑specific terms, lowering the ATS score; domain alignment is strong, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>go-to-market strategy, revenue growth, profitability analysis, sales enablement, customer support, end-of-life management</t>
+          <t>SLA adherence, incident management, root cause analysis (RCA), operational KPIs (uptime, latency, booking failure rate), API integration for flight content</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1350,483 +1340,21 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Franklin Templeton</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Capgemini</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>FBS Product Owner III</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because key tools and methodologies like OKRs, RICE, A/B testing, Mixpanel, Snowflake are missing; fit score is higher due to strong SaaS and GenAI experience aligning with the product owner role.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake, NPS improvement, Roadmap planning, Quality control metrics</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Anaqua</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but lacks several JD-specific terms like product backlog and AI automation agents, leading to a moderate ATS score. Domain alignment is good with SaaS and enterprise experience.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>product backlog, backlog refinement, roadmap prioritization, intellectual property management, AI automation agents</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Data Assets Platform</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many relevant terms but misses several core JD keywords such as roadmap, governance, and UAT, limiting the ATS score. The strongest keyword gap is the lack of explicit 'roadmap' and 'governance' language.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>roadmap, governance, UAT, release readiness, metrics, data platform, backlog, product vision</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>tripstack</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Virtual Interlining</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is a close match, but the resume lacks several JD‑specific terms such as API, payments, and virtual interlining, lowering the ATS score. Domain experience in travel tech and SaaS is strong, giving a solid fit score.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>API integration, payments processing, fraud prevention, pricing optimization, virtual interlining, B2B SaaS platform, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>MaxIQ</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns, but the resume lacks several JD‑specific terms such as product roadmap and analytics, lowering the ATS score; overall domain and skill fit are strong.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Product Roadmap, Analytics/Reporting, Scalability, Sales Enablement, Product Marketing, Competitive Landscape, Metrics measurement</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Copeland</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -1844,13 +1372,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1862,7 +1383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1968,12 +1489,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Modlix</t>
+          <t>Penguin Solutions</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI AdTech / MarTech</t>
+          <t>Software Product Manager, ClusterWareAI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1984,22 +1505,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many AdTech/MarTech specific terms and AI product metrics, lowering both scores; the biggest gap is missing keywords like "campaign management" and "LLM".</t>
+          <t>Hard rules are satisfied, but the resume lacks many core AI infrastructure and cluster management terms from the JD, lowering both ATS and fit scores; the biggest gap is missing keywords like "orchestration" and "cluster management".</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>campaign management, performance marketing, LLM, recommendation system, predictive model, GTM plan, MVP definition, product vision, KPIs, activation metrics</t>
+          <t>cluster management, orchestration, monitoring, distributed systems, cloud deployment, HPC, AI factory platform, automation, product roadmap, product vision</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2017,29 +1538,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Qure.ai</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-II, Amazon SEND</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2048,26 +1569,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 3‑year minimum). The resume contains many Agile and GenAI terms but lacks healthcare‑specific deployment and regulatory keywords, lowering the ATS score; the biggest gap is the absence of clinical/IT deployment terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but keyword overlap with the Amazon SEND JD is limited, especially around logistics, finance, and go‑to‑market concepts.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>clinical stakeholder management, IT integration and deployment, post‑deployment stabilization, guardrails for AI workflows, US market regulatory compliance, FDA clearance experience</t>
+          <t>go-to-market plan, PR/FAQs, finance collaboration, marketing partnership, cross‑border logistics, seller experience, usage analytics, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2085,29 +1604,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Penguin Solutions</t>
+          <t>RAK Ceramics</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Software Product Manager, ClusterWareAI</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2118,22 +1637,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks many core AI infrastructure and cluster management terms from the JD, lowering both ATS and fit scores; the biggest gap is missing keywords like "orchestration" and "cluster management".</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is low due to missing core domain keywords (sanitaryware, P&amp;L, route-to-retail, go-to-market, dealer enablement) and limited tool overlap. Fit score reflects transferable product skills but weak domain alignment with ceramics.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>cluster management, orchestration, monitoring, distributed systems, cloud deployment, HPC, AI factory platform, automation, product roadmap, product vision</t>
+          <t>P&amp;L ownership, route-to-retail, go-to-market execution, dealer enablement, sanitaryware/bathware/faucets portfolio, margin improvement, market insights, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2156,24 +1675,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Nykaa</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Platform</t>
+          <t>Product Manager II - Personalisation</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2184,22 +1703,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with JD-specific terms like access‑control, API, and HLDs; the most important gap is the lack of platform‑security keywords. Fit score reflects some relevance (GenAI, enterprise SaaS) but a domain mismatch with cybersecurity platform responsibilities.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>access control, permissioning, API, high‑level design (HLD), prototype, proof of concept, multi‑tenant, developer platform, MCP</t>
+          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2217,29 +1736,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Arbex</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Now, Amazon Now</t>
+          <t>Workday Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2250,22 +1769,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks most geospatial and location‑intelligence keywords required by the Amazon Now role, resulting in a low ATS score; the biggest gap is missing domain‑specific terms like "geospatial" and "location intelligence".</t>
+          <t>The resume lacks core HR‑specific keywords (Workday, HCM, Compensation, Benefits, Talent Acquisition) and the candidate's domain is SaaS/GenAI rather than HR tech, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>geospatial solutions, location intelligence, spatial analytics, dynamic mapping, address standardization, last-mile delivery, store network planning</t>
+          <t>Workday, HCM, Compensation, Benefits, Talent Acquisition, LOA, HRIS configuration, roadmap management, stakeholder engagement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2283,24 +1802,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Radiometer</t>
+          <t>Schneider Electric</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2310,28 +1829,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume contains few of the marketing‑focused keywords from the JD, resulting in a low ATS match; the biggest gap is the lack of diagnostic/marketing terminology.</t>
+          <t>The JD is for a senior Product Manager role; the candidate is an Associate Product Manager, triggering the senior‑title hard rule, so both scores must be below 30. The resume also lacks several core JD keywords such as "go‑to‑market", "SAFe", and "product increment".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Immunoassay, brand awareness, market surveys, sales enablement, advertising and promotions, global marketing, artwork collateral, customer success metrics</t>
+          <t>go-to-market strategy, Scaled Agile Framework (SAFe), Product Increment (PI) planning, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2349,55 +1868,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Wells Fargo</t>
+          <t>Infineon Technologies</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner: Markets Repo and Securities Lending Platform (VP)</t>
+          <t>Product Manager — Developer Platform (GitHub)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The job title includes 'VP', triggering a hard rule that forces both scores below 30 regardless of experience or keyword match; the resume lacks several core repo and securities‑lending terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any GitHub‑specific experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>collateral optimization, repo trading lifecycle, securities lending, inventory utilization, risk management tools</t>
+          <t>GitHub repository hygiene, SDK lifecycle management, developer portal, open‑source community building, instrumentation and analytics</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2415,57 +1934,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Zaggle</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Securities Services - Data &amp; AI Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 3‑year minimum). The resume contains many relevant terms but misses several core fintech and P2P-specific keywords, lowering the ATS score; the biggest gap is the lack of procure‑to‑pay and payments terminology.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any data‑lake or cloud platform mentions (e.g., Databricks, Hadoop, Spark).</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Procure-to-Pay, FinTech payments integration, Client onboarding, Renewals management, OKRs, RICE prioritization, A/B testing, NPS improvement, Snowflake</t>
+          <t>Databricks, Hadoop, Spark, AWS, Azure, data lake, metadata management, AI/ML model deployment, financial data</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2479,59 +1996,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AVEVA</t>
+          <t>thinkbridge</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Electrical Engineering Software</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core electrical engineering and CAD terminology required by the JD, resulting in very low keyword overlap and poor domain fit.</t>
+          <t>The resume meets the hard rules but contains limited JD-specific keywords and lacks explicit location match, resulting in a modest ATS score; the biggest gap is missing workflow‑mapping and discovery terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>electrical engineering requirements, single-line diagrams, schematic and wiring diagrams, cable schedules, IEC/BS/IEEE standards, CAD‑based design workflow, panel drawings</t>
+          <t>discovery sessions, workflow mapping, process automation, OKRs, RICE prioritization, business process modeling, automation developer collaboration, project manager coordination</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2545,59 +2062,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Creospan Private Limited</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner (Capital Markets+Agile environment)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
+          <t>The resume meets the hard rules but lacks many finance‑specific keywords and domain experience, lowering both ATS and fit scores; the most important gap is the absence of custody/trade settlement terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>Custody, Trade Settlement, Asset Servicing, SWIFT 15022, ISO 20022, Financial product lifecycle, Regulatory compliance, Risk reduction, Market and competitor analysis</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2611,59 +2128,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Techno-Comp Computer Services Pvt. Ltd.</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Core Platform and Infrastructure)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years (12‑18 years) of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of healthcare domain terminology.</t>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of OTA, vehicle‑to‑cloud pipelines, or embedded automotive systems.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>healthcare provider workflows, clinical operations, revenue cycle, global product team collaboration, backlog management templates</t>
+          <t>OTA updates, vehicle-to-cloud pipeline, embedded automotive systems, API design for cloud services, security compliance (e.g., ISO 26262), scalable infrastructure, remote diagnostics, fleet management platform</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2677,38 +2194,38 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ZettaMine Labs Pvt. Ltd.</t>
+          <t>Creospan Private Limited</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>[CQC6VPWC] Data Product Manager - Reltio MDM</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -2717,19 +2234,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 9-12 years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks the mandatory keyword 'Reltio MDM'.</t>
+          <t>Hard rule triggered: JD requires 8-10 years total experience (greater than candidate's 4 years), so both scores must be below 30; the most important keyword gap is lack of explicit trade lifecycle and post‑trade workflow terms.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Reltio MDM, data governance, data quality, master data management, SQL data validation</t>
+          <t>Trade Lifecycle, post‑trade workflows, SWIFT 15022, ISO 2022, Custody Operations</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2743,33 +2260,33 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Global Payments Inc.</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Digital Products, Payments) - Pune – 7+ years Exp</t>
+          <t>Vice President - Technology Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2783,19 +2300,19 @@
         <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. The most important keyword gap is the lack of any payments‑specific terminology such as 'payout tracking' or 'reconciliation'.</t>
+          <t>The JD title includes VP, triggering a hard rule that forces both scores below 30; the resume lacks senior‑level title and many JD‑specific keywords.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>payout tracking, payment status tracking, dispute management, merchant self‑service, regulatory compliance</t>
+          <t>Backlog ownership, Agile ceremonies, Risk and control systems, Compliance, Stakeholder partnership</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2813,149 +2330,17 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Citi</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Vice President - Technology Product Owner</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The JD title includes VP, triggering a hard rule that forces both scores below 30; the resume lacks senior‑level title and many JD‑specific keywords.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Backlog ownership, Agile ceremonies, Risk and control systems, Compliance, Stakeholder partnership</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Syneos Health</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Marketing Product Manager (Salesforce)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Serilingampalli, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because core marketing product keywords like Salesforce, MarTech, ABM, lead capture, and campaign management are missing. Fit score is low due to domain mismatch—candidate’s experience is in SaaS and GenAI, not B2B marketing platforms.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Salesforce, MarTech, ABM, lead capture, campaign management, attribution, marketing platform integration, demand generation</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -2974,8 +2359,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-01
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -694,30 +694,28 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PwC Acceleration Center India</t>
+          <t>dentsu</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
         <v>78</v>
       </c>
@@ -729,12 +727,12 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but a few key JD terms are missing, lowering the ATS score slightly; the strongest gap is the lack of explicit go‑to‑market/commercialization language.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core keywords but lacks several JD‑specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>go‑to‑market strategy, commercialization, OKRs, A/B testing, Snowflake</t>
+          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,24 +750,24 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Cite AI</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -785,22 +783,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Flick TV</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Connectors</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product and AI keywords but lacks connector‑specific terms, lowering the ATS score; domain alignment is strong, giving a higher fit score.</t>
+          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API, custom connector, Indexing API, LLM, Enterprise Graph, OKRs, A/B testing, Snowflake</t>
+          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -889,29 +887,29 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific</t>
+          <t>Cite AI</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager, Antibody Solutions</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -920,19 +918,19 @@
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
+          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
+          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,55 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Franklin Templeton</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager, Connectors</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product and AI keywords but lacks connector‑specific terms, lowering the ATS score; domain alignment is strong, giving a higher fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
+          <t>API, custom connector, Indexing API, LLM, Enterprise Graph, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1012,59 +1010,59 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L1</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1078,38 +1076,38 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Flutter Entertainment India</t>
+          <t>Atos</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner</t>
+          <t>AI platforms &amp; Agentic solutions Product Manager - ServiceNow (Global role)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1118,19 +1116,19 @@
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, SQL, Agile, stakeholder management) but lacks several data‑product specific terms, lowering the ATS score. The biggest gap is the absence of explicit data‑platform and lean methodology keywords.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks ServiceNow-specific terms and senior-level phrasing, and the title is two levels below the senior role.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Data Platform, Lean methodology, OKRs, Data Squad, A/B testing, Snowflake</t>
+          <t>ServiceNow, AI platforms, Agentic AI, Human-centered design, OKRs, GTM strategy, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1144,7 +1142,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1153,50 +1151,52 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>greytHR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F11" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1210,59 +1210,61 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>UST</t>
+          <t>Swish</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many JD keywords (Agile, stakeholder management, AI/GenAI, Jira) but lacks domain‑specific terms, lowering the fit score.</t>
+          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>clinical trial platform, regulatory compliance, workflow orchestration, product roadmap, MVP definition, AI Copilot, predictive analytics</t>
+          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1276,7 +1278,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1285,29 +1287,29 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>tripstack</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Global Product Manager, Antibody Solutions</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1316,19 +1318,19 @@
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant product and SaaS keywords but misses several operational and flight‑specific terms, lowering the ATS score; domain alignment is strong, giving a solid fit score.</t>
+          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>SLA adherence, incident management, root cause analysis (RCA), operational KPIs (uptime, latency, booking failure rate), API integration for flight content</t>
+          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1342,87 +1344,683 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Zeta</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager II</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Franklin Templeton</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LiveRamp</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT MANAGER L1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Backbase</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>(Agentic) Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core AI‑agent terminology from the JD, lowering the ATS score, while the candidate's GenAI and enterprise SaaS background gives a decent fit.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>LLM, inference latency, enterprise‑grade compliance, AI agents, data connectors, durable processes, cross‑pillar integration, customer discovery, roadmap definition</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Flutter Entertainment India</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Data Product Owner</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, SQL, Agile, stakeholder management) but lacks several data‑product specific terms, lowering the ATS score. The biggest gap is the absence of explicit data‑platform and lean methodology keywords.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Data Platform, Lean methodology, OKRs, Data Squad, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TriNet</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>UST</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager II</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many JD keywords (Agile, stakeholder management, AI/GenAI, Jira) but lacks domain‑specific terms, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>clinical trial platform, regulatory compliance, workflow orchestration, product roadmap, MVP definition, AI Copilot, predictive analytics</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>tripstack</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant product and SaaS keywords but misses several operational and flight‑specific terms, lowering the ATS score; domain alignment is strong, giving a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>SLA adherence, incident management, root cause analysis (RCA), operational KPIs (uptime, latency, booking failure rate), API integration for flight content</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>Zywave</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Product Owner</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core API and security keywords, lowering the ATS score, while the overall SaaS and enterprise experience gives a decent fit.</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>REST APIs, OAuth, SSO, API governance, data modeling, security compliance, BI reporting tools (e.g., Tableau), OKRs</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -1441,6 +2039,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1452,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1607,7 +2214,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -1617,19 +2224,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PhonePe</t>
+          <t>super.money</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, HR</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1640,22 +2247,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, but it lacks many HR‑specific keywords and domain experience, resulting in a low ATS match and only moderate overall fit.</t>
+          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass, but the resume lacks many JD‑specific tools and fintech/e‑commerce terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>HR systems, employee lifecycle, performance management, compensation, learning &amp; upskilling, API design, event‑driven architecture, product analytics, predictive modeling, telemetry</t>
+          <t>Mixpanel, Amplitude, A/B testing, funnel analysis, cohort tracking, BNPL, EMI-on-UPI, merchant onboarding, catalogue management, North Star metrics</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1678,24 +2285,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Lam Research</t>
+          <t>Tesco Bengaluru</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1704,26 +2311,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Years of experience meet the 3‑year minimum, but the resume lacks many core spares‑lifecycle keywords, resulting in a modest ATS score and a low fit due to domain mismatch.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management, Obsolescence Management, Last Time Buy, Bridge Buy, Engineering Change Management, Configuration Management, Spare Parts Forecasting, Supply Chain Coordination</t>
+          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1746,24 +2351,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Reo.Dev</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Founding Team (Growth)</t>
+          <t>Product Manager-II, Amazon SEND</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1774,22 +2379,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>50</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is low due to missing many growth‑specific keywords such as experimentation and funnel instrumentation. Fit score is moderate because the candidate has strong SaaS and GenAI experience but limited direct growth‑product work.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but keyword overlap with the Amazon SEND JD is limited, especially around logistics, finance, and go‑to‑market concepts.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>experimentation framework, A/B testing, funnel instrumentation, pricing levers, qualification logic, landing pages, lifecycle messaging, PMM collaboration, demand generation</t>
+          <t>go-to-market plan, PR/FAQs, finance collaboration, marketing partnership, cross‑border logistics, seller experience, usage analytics, A/B testing</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1807,29 +2412,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-II, Amazon SEND</t>
+          <t>Product Manager-Customer Contact Experience Services</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1840,22 +2445,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but keyword overlap with the Amazon SEND JD is limited, especially around logistics, finance, and go‑to‑market concepts.</t>
+          <t>No hard rule violations, but the resume lacks many core contact‑center and Genesys‑specific terms, resulting in a low ATS score; the biggest gap is the absence of any mention of Genesys Cloud CX or contact‑center operations.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>go-to-market plan, PR/FAQs, finance collaboration, marketing partnership, cross‑border logistics, seller experience, usage analytics, A/B testing</t>
+          <t>Genesys Cloud CX, contact center, service performance, incident management, business continuity, disaster recovery, supplier licensing management, privacy compliance, product roadmap, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1873,29 +2478,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>PlaySimple Games</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (MR Scanner Software)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1906,22 +2511,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>45</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
+          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
+          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1944,24 +2549,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Arbex</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Workday Product Owner</t>
+          <t>Product Owner (MR Scanner Software)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1972,22 +2577,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>41</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core HR‑specific keywords (Workday, HCM, Compensation, Benefits, Talent Acquisition) and the candidate's domain is SaaS/GenAI rather than HR tech, leading to low ATS and fit scores.</t>
+          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Workday, HCM, Compensation, Benefits, Talent Acquisition, LOA, HRIS configuration, roadmap management, stakeholder engagement</t>
+          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2005,29 +2610,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Partner Engineering Test Company</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Matthias Test Jobs 2 Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2038,22 +2643,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement, but the resume lacks iOS‑specific keywords and tools, resulting in a low ATS score; the biggest gap is the absence of iOS platform experience.</t>
+          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>iOS app development, App Store deployment, iOS design guidelines, User engagement metrics (e.g., MAU, DAU), A/B testing</t>
+          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2076,24 +2681,24 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Applied Materials India</t>
+          <t>Multi Recruit</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (SAP RTR)</t>
+          <t>Product Owner – Trade Finance</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2104,22 +2709,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of SAP FI/CO experience, but the candidate has only 4+ years overall product experience, triggering the hard rule; consequently both scores are kept below 30. The resume also lacks any SAP‑related terminology.</t>
+          <t>The resume lacks core trade‑finance terminology and specific JD keywords, resulting in a low ATS match; domain mismatch further reduces the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, FI/CO, RTR, PTP, SAP enhancement, SAP integration</t>
+          <t>Import/Export LC, Bank Guarantees (BG/SBLC), SWIFT MT/MX messaging, Functional Specification Document (FSD), Business Requirements Document (BRD), Supply Chain Finance (SCF), ICC Trade Finance guidelines (UCP, URDG, ISBP), Trade Finance journey wireframes/prototypes</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2137,55 +2742,55 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>FBS - Product Owner IV- Data Delivery</t>
+          <t>Product Owner (MR Scanner)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any data‑delivery or data‑governance terms.</t>
+          <t>The resume lacks many domain‑specific terms required for an MR scanner product role, resulting in low keyword overlap and poor fit; the biggest gap is the absence of medical imaging and MRI‑related terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Data Delivery, Data Governance, Data Modeling, Data Profiling, Data Architecture</t>
+          <t>Diagnostic Imaging, MRI physics, Medical device regulations, SAFe Agile, Risk Management, PI Planning, Product Owner, Safety compliance</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2199,7 +2804,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2208,50 +2813,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Entain India</t>
+          <t>Arbex</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Workday Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no explicit 5+ year requirement). ATS score is moderate due to missing many JD-specific keywords like backend APIs, OKRs, CRM, payment systems, and security/scalability. Fit score is decent because of strong SaaS and enterprise product experience, but domain mismatch with sports gaming platform.</t>
+          <t>The resume lacks core HR‑specific keywords (Workday, HCM, Compensation, Benefits, Talent Acquisition) and the candidate's domain is SaaS/GenAI rather than HR tech, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>backend APIs, OKRs, CRM, payment systems, security and scalability</t>
+          <t>Workday, HCM, Compensation, Benefits, Talent Acquisition, LOA, HRIS configuration, roadmap management, stakeholder engagement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2265,59 +2870,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Business Banking -SMB Client &amp; Frontline Experiences (Engage &amp; Deepen)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
+          <t>Hard rules pass, but the resume lacks many banking‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is the absence of risk/compliance and banker workflow terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
+          <t>banker workflow experience, risk and compliance controls, client onboarding and engagement metrics, product roadmap and OKRs, cross‑product engagement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2331,7 +2936,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -2340,50 +2945,50 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Japheth LLP</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Central Bank Digital Currency</t>
+          <t>FBS - Product Owner IV- Data Delivery</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many CBDC‑specific terms and fintech regulatory keywords, resulting in a modest ATS match and limited domain fit.</t>
+          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any data‑delivery or data‑governance terms.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Central Bank Digital Currency (CBDC), Regulatory compliance, Product backlog management, Product vision definition, Competitive analysis, Market research in financial services, Stakeholder engagement for financial products</t>
+          <t>Data Delivery, Data Governance, Data Modeling, Data Profiling, Data Architecture</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2397,11 +3002,11 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -2411,14 +3016,14 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Japheth LLP</t>
+          <t>Entain India</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -2434,22 +3039,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks key fintech and payment system keywords required by the JD, lowering the ATS score; the candidate's SaaS and GenAI experience is only partially relevant to the fintech domain.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no explicit 5+ year requirement). ATS score is moderate due to missing many JD-specific keywords like backend APIs, OKRs, CRM, payment systems, and security/scalability. Fit score is decent because of strong SaaS and enterprise product experience, but domain mismatch with sports gaming platform.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>UPI, IMPS, payment systems, UML, markdown, CBDC, go-to-market strategy, fintech industry trends</t>
+          <t>backend APIs, OKRs, CRM, payment systems, security and scalability</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2467,29 +3072,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Japheth LLP</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Business Analyst - CBDC</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2500,22 +3105,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>46</v>
-      </c>
       <c r="H16" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core fintech and CBDC keywords, resulting in low ATS and fit scores; the biggest gap is the absence of any CBDC‑related experience.</t>
+          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Central Bank Digital Currency (CBDC), UPI, IMPS, User Acceptance Testing, Product Roadmap, Financial Services, Compliance, Market Trends Analysis</t>
+          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2538,24 +3143,24 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Sibros</t>
+          <t>Japheth LLP</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Core Platform and Infrastructure)</t>
+          <t>Product Owner - Central Bank Digital Currency</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2566,22 +3171,22 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of OTA, vehicle‑to‑cloud pipelines, or embedded automotive systems.</t>
+          <t>Hard rules pass, but the resume lacks many CBDC‑specific terms and fintech regulatory keywords, resulting in a modest ATS match and limited domain fit.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>OTA updates, vehicle-to-cloud pipeline, embedded automotive systems, API design for cloud services, security compliance (e.g., ISO 26262), scalable infrastructure, remote diagnostics, fleet management platform</t>
+          <t>Central Bank Digital Currency (CBDC), Regulatory compliance, Product backlog management, Product vision definition, Competitive analysis, Market research in financial services, Stakeholder engagement for financial products</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2599,17 +3204,149 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Japheth LLP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks key fintech and payment system keywords required by the JD, lowering the ATS score; the candidate's SaaS and GenAI experience is only partially relevant to the fintech domain.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>UPI, IMPS, payment systems, UML, markdown, CBDC, go-to-market strategy, fintech industry trends</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Sibros</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Core Platform and Infrastructure)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of OTA, vehicle‑to‑cloud pipelines, or embedded automotive systems.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>OTA updates, vehicle-to-cloud pipeline, embedded automotive systems, API design for cloud services, security compliance (e.g., ISO 26262), scalable infrastructure, remote diagnostics, fleet management platform</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -2631,6 +3368,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-02
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,9 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" s="2" t="n">
         <v>78</v>
       </c>
@@ -616,7 +618,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,7 +628,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -648,7 +650,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
@@ -694,19 +696,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>dentsu</t>
+          <t>peopleHum</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -727,12 +729,12 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core keywords but lacks several JD‑specific tools and frameworks.</t>
+          <t>The resume meets the hard rules and includes most required keywords, but lacks explicit mentions of roadmap planning, PRDs, and structured customer interview processes.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, RICE prioritization, NPS improvement</t>
+          <t>roadmap, PRD, customer interviews, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +752,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Kaufman Rossin</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Hybrid Scrum Master &amp; Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,24 +783,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>The resume meets the 4‑year experience rule and contains most core ATS keywords (Agile, sprint ceremonies, Jira, user stories, epics, acceptance criteria, stakeholder management), but misses several role‑specific terms such as Scrum Master and Product Owner.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>Scrum Master, Product Owner, backlog grooming, US‑based IT stakeholder, IT product lifecycle, Sprint backlog, Kanban</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,24 +820,24 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Flick TV</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -847,24 +851,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,24 +888,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Cite AI</t>
+          <t>Flick TV</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -913,24 +919,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
+          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
+          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,29 +956,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Oxeva.ai</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Connectors</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -981,22 +989,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product and AI keywords but lacks connector‑specific terms, lowering the ATS score; domain alignment is strong, giving a higher fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core terms like program management, KPI definition, and explicit roadmap/vision language.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>API, custom connector, Indexing API, LLM, Enterprise Graph, OKRs, A/B testing, Snowflake</t>
+          <t>program management, KPIs, roadmap development, ethical AI considerations, user research / stakeholder interviews, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1022,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>The Career Company | India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,24 +1053,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>The candidate meets the 4‑year requirement and has relevant GenAI and SaaS experience, but the resume lacks several core GenAI terms (LLMs, embeddings, agents, fine‑tuning, specific cloud providers) reducing the ATS keyword density.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>LLMs, Embeddings, Agents/Tool Calling, Fine‑tuning, OpenAI, Azure OpenAI, AWS Bedrock</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,29 +1090,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Atos</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>AI platforms &amp; Agentic solutions Product Manager - ServiceNow (Global role)</t>
+          <t>Technical Product Manager - Marketplace</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1111,24 +1121,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks ServiceNow-specific terms and senior-level phrasing, and the title is two levels below the senior role.</t>
+          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, AI platforms, Agentic AI, Human-centered design, OKRs, GTM strategy, NPS improvement, A/B testing, Snowflake</t>
+          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1146,29 +1158,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>greytHR</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager, Amazon Now</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1178,25 +1190,25 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
+          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
+          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,29 +1226,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Swish</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1246,25 +1258,25 @@
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1282,55 +1294,57 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager, Antibody Solutions</t>
+          <t>Technical Product Manager - Experimentation</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
+          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,29 +1362,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Zeta</t>
+          <t>greytHR</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1380,25 +1394,25 @@
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>61</v>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
+          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1416,55 +1430,57 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Franklin Templeton</t>
+          <t>Swish</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F15" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains several key terms but misses core AI governance and adoption language, lowering the ATS score. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Responsible AI, bias mitigation, privacy and security compliance, model lifecycle management, adoption metrics</t>
+          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1478,28 +1494,28 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>LiveRamp</t>
+          <t>Meraki Labs</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1509,28 +1525,28 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1544,59 +1560,61 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L1</t>
+          <t>AI Product Manager I / II - Talent Forge</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F17" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H17" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority is appropriate, but several JD‑specific terms are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of RFP/pre‑sales processes.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>RFP, pre‑sales coordination, product vision, roadmap creation, product architecture, DevOps collaboration, user acceptance testing, impact analysis, dashboard reporting</t>
+          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1610,59 +1628,61 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Backbase</t>
+          <t>Infineon Technologies</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>(Agentic) Product Manager</t>
+          <t>Product Owner Digital Product Experience</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core AI‑agent terminology from the JD, lowering the ATS score, while the candidate's GenAI and enterprise SaaS background gives a decent fit.</t>
+          <t>The candidate meets the years requirement and has relevant Agile and stakeholder management experience, but lacks many e‑commerce specific keywords from the JD, leading to a moderate ATS score and a modest fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>LLM, inference latency, enterprise‑grade compliance, AI agents, data connectors, durable processes, cross‑pillar integration, customer discovery, roadmap definition</t>
+          <t>e-commerce, product catalog, conversion optimization, web analytics, A/B testing, search experience, customer journey mapping, product backlog grooming</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1676,33 +1696,33 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Flutter Entertainment India</t>
+          <t>Global HealthX</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1711,24 +1731,26 @@
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G19" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H19" s="2" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, SQL, Agile, stakeholder management) but lacks several data‑product specific terms, lowering the ATS score. The biggest gap is the absence of explicit data‑platform and lean methodology keywords.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Data Platform, Lean methodology, OKRs, Data Squad, A/B testing, Snowflake</t>
+          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1746,29 +1768,29 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Manager (AI)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1777,24 +1799,26 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1812,55 +1836,57 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UST</t>
+          <t>LiveRamp</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F21" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G21" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H21" s="2" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many JD keywords (Agile, stakeholder management, AI/GenAI, Jira) but lacks domain‑specific terms, lowering the fit score.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>clinical trial platform, regulatory compliance, workflow orchestration, product roadmap, MVP definition, AI Copilot, predictive analytics</t>
+          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1874,7 +1900,7 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
@@ -1883,50 +1909,50 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>tripstack</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many relevant product and SaaS keywords but misses several operational and flight‑specific terms, lowering the ATS score; domain alignment is strong, giving a solid fit score.</t>
+          <t>The resume meets the hard rules (4 years experience, appropriate title) and contains many relevant product management keywords, but lacks domain-specific terms for pharmaceutical reference standards, lowering the fit score; the biggest gap is missing forecasting/financial modeling keywords.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>SLA adherence, incident management, root cause analysis (RCA), operational KPIs (uptime, latency, booking failure rate), API integration for flight content</t>
+          <t>forecasting, financial modeling, portfolio management, regulatory compliance, reference standards</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1940,38 +1966,38 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Zywave</t>
+          <t>Flutter Entertainment India</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Data Product Owner</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -1980,47 +2006,179 @@
         <v>68</v>
       </c>
       <c r="G23" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, SQL, Agile, stakeholder management) but lacks several data‑product specific terms, lowering the ATS score. The biggest gap is the absence of explicit data‑platform and lean methodology keywords.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Data Platform, Lean methodology, OKRs, Data Squad, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Zywave</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G24" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core API and security keywords, lowering the ATS score, while the overall SaaS and enterprise experience gives a decent fit.</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>REST APIs, OAuth, SSO, API governance, data modeling, security compliance, BI reporting tools (e.g., Tableau), OKRs</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Owner</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -2048,6 +2206,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2059,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2165,12 +2325,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Glomo</t>
+          <t>super.money</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager / Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2179,24 +2339,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>55</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>60</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>57</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title and location). The resume lacks many sales‑focused keywords required by the JD, lowering the ATS score, while the candidate’s SaaS and enterprise product experience gives a moderate fit.</t>
+          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass, but the resume lacks many JD‑specific tools and fintech/e‑commerce terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>sales discovery calls, demo presentations, merchant onboarding, compliance integration, PRD, roadmap prioritization, IFSCA, FEMA/LRS, risk management</t>
+          <t>Mixpanel, Amplitude, A/B testing, funnel analysis, cohort tracking, BNPL, EMI-on-UPI, merchant onboarding, catalogue management, North Star metrics</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2214,29 +2376,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>super.money</t>
+          <t>Glomo</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager / Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2245,24 +2407,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass, but the resume lacks many JD‑specific tools and fintech/e‑commerce terms, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title and location). The resume lacks many sales‑focused keywords required by the JD, lowering the ATS score, while the candidate’s SaaS and enterprise product experience gives a moderate fit.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, A/B testing, funnel analysis, cohort tracking, BNPL, EMI-on-UPI, merchant onboarding, catalogue management, North Star metrics</t>
+          <t>sales discovery calls, demo presentations, merchant onboarding, compliance integration, PRD, roadmap prioritization, IFSCA, FEMA/LRS, risk management</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2280,29 +2444,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tesco Bengaluru</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, HR</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2311,24 +2475,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
+          <t>The resume meets the 4‑year experience requirement, but it lacks many HR‑specific keywords and domain experience, resulting in a low ATS match and only moderate overall fit.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
+          <t>HR systems, employee lifecycle, performance management, compensation, learning &amp; upskilling, API design, event‑driven architecture, product analytics, predictive modeling, telemetry</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2346,29 +2512,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Lam Research</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-II, Amazon SEND</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2377,24 +2543,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but keyword overlap with the Amazon SEND JD is limited, especially around logistics, finance, and go‑to‑market concepts.</t>
+          <t>Years of experience meet the 3‑year minimum, but the resume lacks many core spares‑lifecycle keywords, resulting in a modest ATS score and a low fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>go-to-market plan, PR/FAQs, finance collaboration, marketing partnership, cross‑border logistics, seller experience, usage analytics, A/B testing</t>
+          <t>Product Lifecycle Management, Obsolescence Management, Last Time Buy, Bridge Buy, Engineering Change Management, Configuration Management, Spare Parts Forecasting, Supply Chain Coordination</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2412,17 +2580,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2646,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -2488,45 +2656,45 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PlaySimple Games</t>
+          <t>insightsoftware</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner – Regulatory Solutions</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core game‑related keywords and mobile‑consumer product experience, resulting in low ATS and fit scores; the biggest gap is missing mobile game and user acquisition terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but lacks many regulatory‑finance specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of regulatory reporting terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>mobile games, user acquisition, growth strategy, game feature specs, key performance indicators (KPIs), A/B testing, user retention</t>
+          <t>Regulatory reporting, ESG reporting, Solvency II, Compliance filing, Financial filing disclosures, User story creation for regulatory workflows, Stakeholder management with finance/compliance teams, Data governance for regulatory data</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2540,59 +2708,61 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (MR Scanner Software)</t>
+          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many domain‑specific terms from the JD (e.g., MRI, SAFe, medical device regulations), resulting in low keyword overlap and a poor fit for the imaging product owner role.</t>
+          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SAFe Agile, MRI physics, medical device regulations, diagnostic imaging, risk management, PI planning, product feature definition, requirement engineering</t>
+          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2606,28 +2776,28 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>Entain India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -2637,28 +2807,28 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no explicit 5+ year requirement). ATS score is moderate due to missing many JD-specific keywords like backend APIs, OKRs, CRM, payment systems, and security/scalability. Fit score is decent because of strong SaaS and enterprise product experience, but domain mismatch with sports gaming platform.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
+          <t>backend APIs, OKRs, CRM, payment systems, security and scalability</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2672,59 +2842,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Multi Recruit</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Trade Finance</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core trade‑finance terminology and specific JD keywords, resulting in a low ATS match; domain mismatch further reduces the fit score.</t>
+          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Import/Export LC, Bank Guarantees (BG/SBLC), SWIFT MT/MX messaging, Functional Specification Document (FSD), Business Requirements Document (BRD), Supply Chain Finance (SCF), ICC Trade Finance guidelines (UCP, URDG, ISBP), Trade Finance journey wireframes/prototypes</t>
+          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2738,59 +2908,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Siemens Healthineers</t>
+          <t>Japheth LLP</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (MR Scanner)</t>
+          <t>Product Owner - Central Bank Digital Currency</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many domain‑specific terms required for an MR scanner product role, resulting in low keyword overlap and poor fit; the biggest gap is the absence of medical imaging and MRI‑related terminology.</t>
+          <t>Hard rules pass, but the resume lacks many CBDC‑specific terms and fintech regulatory keywords, resulting in a modest ATS match and limited domain fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Diagnostic Imaging, MRI physics, Medical device regulations, SAFe Agile, Risk Management, PI Planning, Product Owner, Safety compliance</t>
+          <t>Central Bank Digital Currency (CBDC), Regulatory compliance, Product backlog management, Product vision definition, Competitive analysis, Market research in financial services, Stakeholder engagement for financial products</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2804,59 +2974,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Arbex</t>
+          <t>Japheth LLP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Workday Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core HR‑specific keywords (Workday, HCM, Compensation, Benefits, Talent Acquisition) and the candidate's domain is SaaS/GenAI rather than HR tech, leading to low ATS and fit scores.</t>
+          <t>Hard rules pass, but the resume lacks key fintech and payment system keywords required by the JD, lowering the ATS score; the candidate's SaaS and GenAI experience is only partially relevant to the fintech domain.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Workday, HCM, Compensation, Benefits, Talent Acquisition, LOA, HRIS configuration, roadmap management, stakeholder engagement</t>
+          <t>UPI, IMPS, payment systems, UML, markdown, CBDC, go-to-market strategy, fintech industry trends</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2870,483 +3040,21 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>JPMorganChase</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Business Banking -SMB Client &amp; Frontline Experiences (Engage &amp; Deepen)</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many banking‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is the absence of risk/compliance and banker workflow terminology.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>banker workflow experience, risk and compliance controls, client onboarding and engagement metrics, product roadmap and OKRs, cross‑product engagement</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Capgemini</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>FBS - Product Owner IV- Data Delivery</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any data‑delivery or data‑governance terms.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Data Delivery, Data Governance, Data Modeling, Data Profiling, Data Architecture</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Entain India</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no explicit 5+ year requirement). ATS score is moderate due to missing many JD-specific keywords like backend APIs, OKRs, CRM, payment systems, and security/scalability. Fit score is decent because of strong SaaS and enterprise product experience, but domain mismatch with sports gaming platform.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>backend APIs, OKRs, CRM, payment systems, security and scalability</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Japheth LLP</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Central Bank Digital Currency</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many CBDC‑specific terms and fintech regulatory keywords, resulting in a modest ATS match and limited domain fit.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Central Bank Digital Currency (CBDC), Regulatory compliance, Product backlog management, Product vision definition, Competitive analysis, Market research in financial services, Stakeholder engagement for financial products</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Japheth LLP</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks key fintech and payment system keywords required by the JD, lowering the ATS score; the candidate's SaaS and GenAI experience is only partially relevant to the fintech domain.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>UPI, IMPS, payment systems, UML, markdown, CBDC, go-to-market strategy, fintech industry trends</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Sibros</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager (Core Platform and Infrastructure)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of OTA, vehicle‑to‑cloud pipelines, or embedded automotive systems.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>OTA updates, vehicle-to-cloud pipeline, embedded automotive systems, API design for cloud services, security compliance (e.g., ISO 26262), scalable infrastructure, remote diagnostics, fleet management platform</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -3363,13 +3071,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-03
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Versatile Club Employer of Record</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>81</v>
-      </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflicts, so hard rules pass; the resume covers most core JD keywords but lacks explicit mentions of product roadmap, PRD, backlog grooming and analytics tools.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, PRD, backlog grooming, A/B testing, Mixpanel, NPS improvement</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -623,24 +623,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>Flick TV</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-4 to 6 Years</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,26 +649,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years and title requirements and contains many JD keywords, but lacks several specific analytics and API tools and pricing terminology.</t>
+          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, REST APIs, pricing strategy, API monetization, customer discovery, product-market fit</t>
+          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -691,24 +689,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>peopleHum</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Manager - Marketplace</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,24 +715,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and includes most required keywords, but lacks explicit mentions of roadmap planning, PRDs, and structured customer interview processes.</t>
+          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>roadmap, PRD, customer interviews, OKRs, A/B testing</t>
+          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +752,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Kaufman Rossin</t>
+          <t>LH2 AI Labs</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Hybrid Scrum Master &amp; Product Owner</t>
+          <t>Founding Product Manager - Data Marketplace</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,26 +783,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience rule and contains most core ATS keywords (Agile, sprint ceremonies, Jira, user stories, epics, acceptance criteria, stakeholder management), but misses several role‑specific terms such as Scrum Master and Product Owner.</t>
+          <t>The candidate meets the 4‑year experience requirement and location, but the JD lacks specific keywords, resulting in a moderate ATS match; the most notable gap is the absence of marketplace‑specific terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Scrum Master, Product Owner, backlog grooming, US‑based IT stakeholder, IT product lifecycle, Sprint backlog, Kanban</t>
+          <t>Data marketplace, Two‑sided platform, OKRs, A/B testing, User research, Metrics/KPIs, API strategy</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,29 +818,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Manager - Experimentation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -852,25 +850,25 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -888,24 +886,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Flick TV</t>
+          <t>Swish</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -920,25 +918,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
+          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
+          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -966,19 +964,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Oxeva.ai</t>
+          <t>Meraki Labs</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -989,22 +987,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core terms like program management, KPI definition, and explicit roadmap/vision language.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>program management, KPIs, roadmap development, ethical AI considerations, user research / stakeholder interviews, A/B testing, OKRs</t>
+          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1022,29 +1020,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>The Career Company | India</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AI Product Manager I / II - Talent Forge</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1054,25 +1052,25 @@
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and has relevant GenAI and SaaS experience, but the resume lacks several core GenAI terms (LLMs, embeddings, agents, fine‑tuning, specific cloud providers) reducing the ATS keyword density.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>LLMs, Embeddings, Agents/Tool Calling, Fine‑tuning, OpenAI, Azure OpenAI, AWS Bedrock</t>
+          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1100,24 +1098,24 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Global HealthX</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Marketplace</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1125,22 +1123,22 @@
         <v>3</v>
       </c>
       <c r="F10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H10" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1154,61 +1152,61 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>LiveRamp</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Now</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>78</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>72</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
+          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1222,61 +1220,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>USP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume matches many ATS keywords but lacks several core JD terms like forecasting and financial modeling, lowering the ATS score. Domain mismatch (pharma reference standards vs SaaS/GenAI) reduces the fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>forecasting, financial modeling, prioritization framework, OKRs, market research analysis</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1290,38 +1286,38 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Experimentation</t>
+          <t>Product Manager (AI &amp; Software Delivery)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1339,12 +1335,12 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title rule is triggered; however the resume lacks several core JD tools and methodologies, lowering the ATS score. The strongest keyword gap is the absence of Azure DevOps/Waterfall and LLM‑related terms.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
+          <t>Azure DevOps, Waterfall, Scrum/Kanban, LLM integration, Chatbots, AI agents, Change control, Risk management, Trello, Asana</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1358,61 +1354,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>greytHR</t>
+          <t>Improzo</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Associate Product Manager (APM)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
+          <t>The candidate meets the 4-year experience requirement and title alignment, but the JD lacks many specific keywords present in the resume, leading to a moderate ATS score; the strongest gap is the absence of explicit JD tools like Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
+          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, PLG, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1426,44 +1420,42 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Swish</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
         <v>68</v>
       </c>
@@ -1475,12 +1467,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
+          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1494,691 +1486,21 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Meraki Labs</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Eightfold AI</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>AI Product Manager I / II - Talent Forge</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Infineon Technologies</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner Digital Product Experience</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru East, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the years requirement and has relevant Agile and stakeholder management experience, but lacks many e‑commerce specific keywords from the JD, leading to a moderate ATS score and a modest fit score due to domain mismatch.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>e-commerce, product catalog, conversion optimization, web analytics, A/B testing, search experience, customer journey mapping, product backlog grooming</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Global HealthX</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager (AI)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>LiveRamp</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>US Pharmacopeia</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, appropriate title) and contains many relevant product management keywords, but lacks domain-specific terms for pharmaceutical reference standards, lowering the fit score; the biggest gap is missing forecasting/financial modeling keywords.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>forecasting, financial modeling, portfolio management, regulatory compliance, reference standards</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Flutter Entertainment India</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Data Product Owner</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, SQL, Agile, stakeholder management) but lacks several data‑product specific terms, lowering the ATS score. The biggest gap is the absence of explicit data‑platform and lean methodology keywords.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Data Platform, Lean methodology, OKRs, Data Squad, A/B testing, Snowflake</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Zywave</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core API and security keywords, lowering the ATS score, while the overall SaaS and enterprise experience gives a decent fit.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>REST APIs, OAuth, SSO, API governance, data modeling, security compliance, BI reporting tools (e.g., Tableau), OKRs</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -2198,16 +1520,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2219,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2386,19 +1698,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Glomo</t>
+          <t>Zixflow</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager / Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2407,26 +1719,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>57</v>
-      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title and location). The resume lacks many sales‑focused keywords required by the JD, lowering the ATS score, while the candidate’s SaaS and enterprise product experience gives a moderate fit.</t>
+          <t>The resume meets the 4-year experience requirement and has no senior title conflict, but the job description provides no concrete keywords, resulting in a low ATS match; the strongest gap is the absence of typical product metrics and tooling keywords.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>sales discovery calls, demo presentations, merchant onboarding, compliance integration, PRD, roadmap prioritization, IFSCA, FEMA/LRS, risk management</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2444,57 +1754,55 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PhonePe</t>
+          <t>Yulu</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, HR</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Bengaluru Area</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>51</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, but it lacks many HR‑specific keywords and domain experience, resulting in a low ATS match and only moderate overall fit.</t>
+          <t>No explicit years requirement or senior title triggers hard rules, but the resume lacks many JD-specific keywords, lowering the ATS score; the strongest gap is the absence of common product management frameworks and metrics.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>HR systems, employee lifecycle, performance management, compensation, learning &amp; upskilling, API design, event‑driven architecture, product analytics, predictive modeling, telemetry</t>
+          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, User research &amp; testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2512,34 +1820,34 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Lam Research</t>
+          <t>Skillz</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Manager, Engagement</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Bengaluru Area</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -2547,22 +1855,22 @@
         <v>3</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Years of experience meet the 3‑year minimum, but the resume lacks many core spares‑lifecycle keywords, resulting in a modest ATS score and a low fit due to domain mismatch.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). ATS score is low due to missing core gaming and mobile product keywords; the biggest gap is the lack of any gaming‑related terminology. Fit score reflects decent product skills but limited domain relevance to mobile esports.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management, Obsolescence Management, Last Time Buy, Bridge Buy, Engineering Change Management, Configuration Management, Spare Parts Forecasting, Supply Chain Coordination</t>
+          <t>mobile gaming, player engagement metrics, A/B testing, OKRs, user retention, growth hacking, live ops, game telemetry, in‑app monetization</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2585,12 +1893,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -2656,24 +1964,24 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>insightsoftware</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Regulatory Solutions</t>
+          <t>Product Manager - Business Banking -SMB Client &amp; Frontline Experiences (Engage &amp; Deepen)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -2682,19 +1990,19 @@
         <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but lacks many regulatory‑finance specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of regulatory reporting terminology.</t>
+          <t>Hard rules pass, but the resume lacks many banking‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is the absence of risk/compliance and banker workflow terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Regulatory reporting, ESG reporting, Solvency II, Compliance filing, Financial filing disclosures, User story creation for regulatory workflows, Stakeholder management with finance/compliance teams, Data governance for regulatory data</t>
+          <t>banker workflow experience, risk and compliance controls, client onboarding and engagement metrics, product roadmap and OKRs, cross‑product engagement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2712,17 +2020,17 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -2790,19 +2098,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Entain India</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2813,22 +2121,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>59</v>
-      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no explicit 5+ year requirement). ATS score is moderate due to missing many JD-specific keywords like backend APIs, OKRs, CRM, payment systems, and security/scalability. Fit score is decent because of strong SaaS and enterprise product experience, but domain mismatch with sports gaming platform.</t>
+          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>backend APIs, OKRs, CRM, payment systems, security and scalability</t>
+          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2846,7 +2154,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2856,205 +2164,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Japheth LLP</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Central Bank Digital Currency</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many CBDC‑specific terms and fintech regulatory keywords, resulting in a modest ATS match and limited domain fit.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Central Bank Digital Currency (CBDC), Regulatory compliance, Product backlog management, Product vision definition, Competitive analysis, Market research in financial services, Stakeholder engagement for financial products</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Japheth LLP</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks key fintech and payment system keywords required by the JD, lowering the ATS score; the candidate's SaaS and GenAI experience is only partially relevant to the fintech domain.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>UPI, IMPS, payment systems, UML, markdown, CBDC, go-to-market strategy, fintech industry trends</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -3068,9 +2178,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-04
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Meraki Labs</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Founding Product Manager - myRico</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,26 +581,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers most core JD keywords but misses explicit terms like "customer obsession" and "product judgment".</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>customer obsession, product judgment, OKRs, prototype, workflow automation, A/B testing</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,24 +616,24 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Flick TV</t>
+          <t>peopleHum</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -654,19 +652,19 @@
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1+ year requirement and title alignment, but lacks ecommerce/marketplace specific terminology, lowering the ATS score; the biggest keyword gap is the absence of ecommerce/marketplace language.</t>
+          <t>The resume meets the hard rules and includes most required keywords, but lacks explicit mentions of roadmap planning, PRDs, and structured customer interview processes.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>ecommerce, marketplace, A/B testing, OKRs, NPS improvement</t>
+          <t>roadmap, PRD, customer interviews, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Kaufman Rossin</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Marketplace</t>
+          <t>Hybrid Scrum Master &amp; Product Owner</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -716,25 +714,25 @@
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
+          <t>The resume meets the 4‑year experience rule and contains most core ATS keywords (Agile, sprint ceremonies, Jira, user stories, epics, acceptance criteria, stakeholder management), but misses several role‑specific terms such as Scrum Master and Product Owner.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>Scrum Master, Product Owner, backlog grooming, US‑based IT stakeholder, IT product lifecycle, Sprint backlog, Kanban</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LH2 AI Labs</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Founding Product Manager - Data Marketplace</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,24 +781,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and location, but the JD lacks specific keywords, resulting in a moderate ATS match; the most notable gap is the absence of marketplace‑specific terminology.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Data marketplace, Two‑sided platform, OKRs, A/B testing, User research, Metrics/KPIs, API strategy</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,17 +818,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Experimentation</t>
+          <t>Technical Product Manager - Marketplace</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -853,22 +853,22 @@
         <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
+          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
+          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -891,24 +891,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Swish</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager, Amazon Now</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -921,22 +921,22 @@
         <v>3</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title matches, but lacks several JD‑specific tools and methodologies, notably A/B testing and Mixpanel, lowering the ATS score; the biggest keyword gap is the absence of experimentation/A‑B testing experience.</t>
+          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Metabase, logistics, food delivery, experiment design, delivery time estimation</t>
+          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,24 +954,24 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Meraki Labs</t>
+          <t>The Career Company | India</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -985,24 +985,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
+          <t>The candidate meets the 4‑year requirement and has relevant GenAI and SaaS experience, but the resume lacks several core GenAI terms (LLMs, embeddings, agents, fine‑tuning, specific cloud providers) reducing the ATS keyword density.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
+          <t>LLMs, Embeddings, Agents/Tool Calling, Fine‑tuning, OpenAI, Azure OpenAI, AWS Bedrock</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1030,19 +1032,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Eightfold AI</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager I / II - Talent Forge</t>
+          <t>Technical Product Manager - Experimentation</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1058,19 +1060,19 @@
         <v>58</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
+          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1088,24 +1090,24 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Global HealthX</t>
+          <t>Meraki Labs</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1115,30 +1117,28 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H10" s="2" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
+          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1166,47 +1166,45 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>LiveRamp</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Global Product Manager, Antibody Solutions</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1220,59 +1218,61 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>USP</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
+          <t>AI Product Manager I / II - Talent Forge</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume matches many ATS keywords but lacks several core JD terms like forecasting and financial modeling, lowering the ATS score. Domain mismatch (pharma reference standards vs SaaS/GenAI) reduces the fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>forecasting, financial modeling, prioritization framework, OKRs, market research analysis</t>
+          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1295,52 +1295,50 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Techdome</t>
+          <t>Ericsson</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (AI &amp; Software Delivery)</t>
+          <t>IT Product Owner - Intelligent Service Management</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>58</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title rule is triggered; however the resume lacks several core JD tools and methodologies, lowering the ATS score. The strongest keyword gap is the absence of Azure DevOps/Waterfall and LLM‑related terms.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant tools (Jira, SQL, Agile) but lacks several core JD terms such as OKRs, financial planning, and service‑management governance, limiting the ATS match.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, Waterfall, Scrum/Kanban, LLM integration, Chatbots, AI agents, Change control, Risk management, Trello, Asana</t>
+          <t>OKRs, financial planning, budget forecasting, regulatory compliance, service management / ITSM, governance meetings, product line strategy, autonomous AI operations</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1354,59 +1352,61 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Improzo</t>
+          <t>Infineon Technologies</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (APM)</t>
+          <t>Product Owner Digital Product Experience</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title alignment, but the JD lacks many specific keywords present in the resume, leading to a moderate ATS score; the strongest gap is the absence of explicit JD tools like Mixpanel or A/B testing.</t>
+          <t>The candidate meets the years requirement and has relevant Agile and stakeholder management experience, but lacks many e‑commerce specific keywords from the JD, leading to a moderate ATS score and a modest fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, PLG, NPS improvement, MAU growth</t>
+          <t>e-commerce, product catalog, conversion optimization, web analytics, A/B testing, search experience, customer journey mapping, product backlog grooming</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1420,87 +1420,425 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager, Private Brands</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 3+ year requirement and matches the Bengaluru location, so hard rules do not penalize it; however, key private‑brand specific terms like inventory management and catalog initiatives are missing, lowering the ATS score. The strongest keyword gap is the lack of any mention of inventory/forecasting or supply‑chain work.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>inventory management, forecasting, supply chain optimization, catalog management, marketplace analytics, A/B testing, OKRs, customer NPS, growth metrics</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Global HealthX</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Amgen</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager (AI)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>USP</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume matches many ATS keywords but lacks several core JD terms like forecasting and financial modeling, lowering the ATS score. Domain mismatch (pharma reference standards vs SaaS/GenAI) reduces the fit score.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>forecasting, financial modeling, prioritization framework, OKRs, market research analysis</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Techdome</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (AI &amp; Software Delivery)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title rule is triggered; however the resume lacks several core JD tools and methodologies, lowering the ATS score. The strongest keyword gap is the absence of Azure DevOps/Waterfall and LLM‑related terms.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Azure DevOps, Waterfall, Scrum/Kanban, LLM integration, Chatbots, AI agents, Change control, Risk management, Trello, Asana</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Barclays</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Technical Product Owner</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Apply</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
@@ -1520,6 +1858,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1531,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1637,12 +1980,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>super.money</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Robotics</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1652,25 +1995,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass, but the resume lacks many JD‑specific tools and fintech/e‑commerce terms, lowering both scores.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass, but the resume contains few of the robotics‑focused keywords from the JD, leading to a low ATS score; the biggest gap is the lack of any mention of physical AI data collection or robotics.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, A/B testing, funnel analysis, cohort tracking, BNPL, EMI-on-UPI, merchant onboarding, catalogue management, North Star metrics</t>
+          <t>physical AI data collection, robotics, task assignment, metadata management, quality review workflows, teleoperation, foundation model, RFP, go-to-market messaging</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1688,29 +2031,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Zixflow</t>
+          <t>Agratas – A Tata Enterprise</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - Pack Technology</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1721,22 +2064,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and has no senior title conflict, but the job description provides no concrete keywords, resulting in a low ATS match; the strongest gap is the absence of typical product metrics and tooling keywords.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the battery‑pack specific keywords required by the JD, resulting in low ATS and fit scores; the most important gap is the absence of any Battery Management System or hardware integration terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization</t>
+          <t>Battery Management System (BMS), energy density, SCRUM, KPIs (cost, reliability, safety), hardware integration, manufacturability, cost optimization, battery pack architecture</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1754,55 +2097,57 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yulu</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Greater Bengaluru Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>No explicit years requirement or senior title triggers hard rules, but the resume lacks many JD-specific keywords, lowering the ATS score; the strongest gap is the absence of common product management frameworks and metrics.</t>
+          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, User research &amp; testing</t>
+          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1816,355 +2161,21 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Skillz</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Engagement</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Greater Bengaluru Area</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). ATS score is low due to missing core gaming and mobile product keywords; the biggest gap is the lack of any gaming‑related terminology. Fit score reflects decent product skills but limited domain relevance to mobile esports.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>mobile gaming, player engagement metrics, A/B testing, OKRs, user retention, growth hacking, live ops, game telemetry, in‑app monetization</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>EY</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager-Customer Contact Experience Services</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>No hard rule violations, but the resume lacks many core contact‑center and Genesys‑specific terms, resulting in a low ATS score; the biggest gap is the absence of any mention of Genesys Cloud CX or contact‑center operations.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Genesys Cloud CX, contact center, service performance, incident management, business continuity, disaster recovery, supplier licensing management, privacy compliance, product roadmap, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>JPMorganChase</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Business Banking -SMB Client &amp; Frontline Experiences (Engage &amp; Deepen)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many banking‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is the absence of risk/compliance and banker workflow terminology.</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>banker workflow experience, risk and compliance controls, client onboarding and engagement metrics, product roadmap and OKRs, cross‑product engagement</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules but lacks many core product‑owner keywords and the payments/cards domain experience, resulting in a moderate ATS score and low fit score; the biggest gap is missing Scrum and metrics terminology.</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Scrum, adoption rates, usage patterns, customer satisfaction (NPS), revenue generation, metrics tracking, OKRs</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
@@ -2173,11 +2184,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-05
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>peopleHum</t>
+          <t>Accion Labs</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,22 +649,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and includes most required keywords, but lacks explicit mentions of roadmap planning, PRDs, and structured customer interview processes.</t>
+          <t>The resume meets the hard rules and aligns well with the product manager role, but several key JD terms (APIs, Cloud, Python, LLMs, Integration, Distributed Systems) are missing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>roadmap, PRD, customer interviews, OKRs, A/B testing</t>
+          <t>APIs, Cloud, Python, LLMs, Integration, Distributed Systems</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Kaufman Rossin</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Hybrid Scrum Master &amp; Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,22 +717,22 @@
         <v>4</v>
       </c>
       <c r="F4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>82</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience rule and contains most core ATS keywords (Agile, sprint ceremonies, Jira, user stories, epics, acceptance criteria, stakeholder management), but misses several role‑specific terms such as Scrum Master and Product Owner.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Scrum Master, Product Owner, backlog grooming, US‑based IT stakeholder, IT product lifecycle, Sprint backlog, Kanban</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>Bright Money</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - AI and Agentic</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -782,25 +782,25 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and location, so hard rules pass; however the resume lacks several fintech‑specific terms (LLM, credit‑card, marketplace) reducing the ATS match.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
+          <t>LLM, AI money assistant, credit card product, FinTech, Marketplace dynamics, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,29 +818,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Marketplace</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,26 +849,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and has a relevant title, so hard rules do not penalize the scores; the main ATS gap is missing marketplace‑specific terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many Agile and product delivery terms but lacks several JD‑specific data‑product keywords, lowering the ATS score; the main gap is missing explicit customer‑segmentation and data‑governance terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Marketplace dynamics, Two‑sided platform, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>customer segmentation, personalisation, insight datasets, data governance, analytics collaboration, data science partnership, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,29 +884,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Narayana Health</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Now</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -918,25 +916,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,57 +952,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>The Career Company | India</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Global Product Manager, Antibody Solutions</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and has relevant GenAI and SaaS experience, but the resume lacks several core GenAI terms (LLMs, embeddings, agents, fine‑tuning, specific cloud providers) reducing the ATS keyword density.</t>
+          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>LLMs, Embeddings, Agents/Tool Calling, Fine‑tuning, OpenAI, Azure OpenAI, AWS Bedrock</t>
+          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1022,29 +1018,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Tesco Bengaluru</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Experimentation</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1053,26 +1049,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
         <v>58</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title does not violate seniority rules, but the resume lacks several JD‑specific keywords (e.g., API gateway, real‑time data governance). This lowers the ATS score while the strong travel‑tech and GenAI background yields a solid fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume lacks several JD-specific data product terms such as segmentation and governance, lowering the ATS score, while the candidate's GenAI and SaaS background gives a moderate fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>API gateway, real-time data processing, data governance, A/B testing, NPS improvement, Marketplace dynamics, two-sided platform, OKRs, RICE prioritization</t>
+          <t>customer segmentation, audience filters, insights datasets, data governance, stakeholder interviews, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1090,55 +1084,57 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Meraki Labs</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (AI &amp; Software Delivery)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to limited overlap with JD-specific terminology and only partial title alignment. Fit score is higher because the candidate's GenAI and enterprise SaaS experience aligns well with the AI‑teammate product vision.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title rule is triggered; however the resume lacks several core JD tools and methodologies, lowering the ATS score. The strongest keyword gap is the absence of Azure DevOps/Waterfall and LLM‑related terms.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>customer obsession, product judgment, AI teammate, workflow automation, prototype, user research, OKRs, A/B testing, NPS improvement</t>
+          <t>Azure DevOps, Waterfall, Scrum/Kanban, LLM integration, Chatbots, AI agents, Change control, Risk management, Trello, Asana</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1152,693 +1148,21 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Thermo Fisher Scientific</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Global Product Manager, Antibody Solutions</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru East, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>No hard rule violations; the resume contains many generic product management terms but lacks several JD‑specific keywords and domain experience in life‑sciences, leading to a moderate ATS score and a lower fit score.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Voice of Customer (VOC), Strategic marketing, Product roadmap ownership, Matrixed organization collaboration, Go‑to‑market strategy</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Eightfold AI</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>AI Product Manager I / II - Talent Forge</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks many JD-specific terms such as cloud platforms and talent‑tech jargon, lowering the ATS score, while the candidate's GenAI and SaaS experience gives a moderate job‑fit.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Azure, AWS, API design, headless architecture, OKRs, A/B testing, NPS improvement, talent acquisition, PLG</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Ericsson</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>IT Product Owner - Intelligent Service Management</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant tools (Jira, SQL, Agile) but lacks several core JD terms such as OKRs, financial planning, and service‑management governance, limiting the ATS match.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, financial planning, budget forecasting, regulatory compliance, service management / ITSM, governance meetings, product line strategy, autonomous AI operations</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Infineon Technologies</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner Digital Product Experience</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru East, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the years requirement and has relevant Agile and stakeholder management experience, but lacks many e‑commerce specific keywords from the JD, leading to a moderate ATS score and a modest fit score due to domain mismatch.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>e-commerce, product catalog, conversion optimization, web analytics, A/B testing, search experience, customer journey mapping, product backlog grooming</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Private Brands</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 3+ year requirement and matches the Bengaluru location, so hard rules do not penalize it; however, key private‑brand specific terms like inventory management and catalog initiatives are missing, lowering the ATS score. The strongest keyword gap is the lack of any mention of inventory/forecasting or supply‑chain work.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>inventory management, forecasting, supply chain optimization, catalog management, marketplace analytics, A/B testing, OKRs, customer NPS, growth metrics</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Global HealthX</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but the resume lacks several JD‑specific keywords, lowering the ATS score; the biggest gap is the absence of explicit experiment/metrics terminology.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, OKRs, NPS improvement, user research interviews, experiment framework, healthcare domain experience</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager (AI)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>USP</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager/Product Manager (Reference Standards)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume matches many ATS keywords but lacks several core JD terms like forecasting and financial modeling, lowering the ATS score. Domain mismatch (pharma reference standards vs SaaS/GenAI) reduces the fit score.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>forecasting, financial modeling, prioritization framework, OKRs, market research analysis</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Techdome</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager (AI &amp; Software Delivery)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title rule is triggered; however the resume lacks several core JD tools and methodologies, lowering the ATS score. The strongest keyword gap is the absence of Azure DevOps/Waterfall and LLM‑related terms.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Azure DevOps, Waterfall, Scrum/Kanban, LLM integration, Chatbots, AI agents, Change control, Risk management, Trello, Asana</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -1853,16 +1177,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1874,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1980,12 +1294,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Pice®</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Robotics</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1998,22 +1312,22 @@
         <v>2</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass, but the resume contains few of the robotics‑focused keywords from the JD, leading to a low ATS score; the biggest gap is the lack of any mention of physical AI data collection or robotics.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass, but the resume lacks many core lending‑product keywords (e.g., KYC, credit, disbursal, APIs) and location details, limiting the ATS score. The strongest gap is the absence of credit‑lending terminology.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>physical AI data collection, robotics, task assignment, metadata management, quality review workflows, teleoperation, foundation model, RFP, go-to-market messaging</t>
+          <t>KYC, credit, disbursal, APIs, funnel metrics, compliance, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2031,29 +1345,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Agratas – A Tata Enterprise</t>
+          <t>Snapmint</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Pack Technology</t>
+          <t>Product Manager - Seller Experience</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2062,24 +1376,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the battery‑pack specific keywords required by the JD, resulting in low ATS and fit scores; the most important gap is the absence of any Battery Management System or hardware integration terminology.</t>
+          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass; however the resume lacks many seller‑experience specific keywords from the JD, lowering the ATS score. The biggest gap is missing marketplace‑seller terminology like "seller onboarding" and "catalog management".</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Battery Management System (BMS), energy density, SCRUM, KPIs (cost, reliability, safety), hardware integration, manufacturability, cost optimization, battery pack architecture</t>
+          <t>seller onboarding, catalog management, pricing and promotions, KYC verification, seller performance dashboards, self‑service tools, marketplace dynamics, order management</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2097,34 +1413,34 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Bright Money</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
+          <t>Product Manager - Credit Card</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -2132,22 +1448,22 @@
         <v>3</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). The resume lacks core fintech and credit‑card terminology, lowering both scores; the biggest gap is missing credit‑card/financial‑services keywords.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
+          <t>credit card, risk management, credit underwriting, financial services marketplace, A/B testing, product metrics, growth funnel, roadmap planning, KYC/AML compliance</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2161,21 +1477,355 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TELUS Digital</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Robotics</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass, but the resume contains few of the robotics‑focused keywords from the JD, leading to a low ATS score; the biggest gap is the lack of any mention of physical AI data collection or robotics.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>physical AI data collection, robotics, task assignment, metadata management, quality review workflows, teleoperation, foundation model, RFP, go-to-market messaging</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Namma Yatri</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore Urban, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title), but the resume contains few of the specific mobility platform keywords from the JD, leading to a low ATS score; the biggest gap is missing terms like Beckn Protocol and ONDC.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Beckn Protocol, ONDC network, API design and integration, A/B testing, OKRs, Marketplace dynamics, Two-sided platform, NPS improvement, Growth metrics (MAU, retention)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Agratas – A Tata Enterprise</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Pack Technology</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the battery‑pack specific keywords required by the JD, resulting in low ATS and fit scores; the most important gap is the absence of any Battery Management System or hardware integration terminology.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Battery Management System (BMS), energy density, SCRUM, KPIs (cost, reliability, safety), hardware integration, manufacturability, cost optimization, battery pack architecture</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Opella</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Data Product Owner - SAP HUB</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks many SAP‑specific terms and data‑hub experience, leading to a moderate ATS score and a low fit score due to domain mismatch.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Data extraction, Unified data model, Data privacy, SOX compliance, Regulatory compliance, Cybersecurity requirements, SLA management, Test case execution</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EMotorad</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager- Business Systems and Operations</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement, but lacks many ERP and manufacturing-specific terms and the location does not match Pune, resulting in moderate ATS and fit scores; the biggest keyword gap is the absence of ERPNext/Frappe experience.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext, Frappe, production planning, inventory management, order-to-cash, procurement, workflow automation, supply chain, manufacturing operations, OKRs</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -2184,6 +1834,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-07
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Meraki Labs</t>
+          <t>YourDOST</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Founding Product Manager - myRico</t>
+          <t>Associate Product Manager/ Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,24 +581,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers most core JD keywords but misses explicit terms like "customer obsession" and "product judgment".</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches the Associate Product Manager level, yielding solid ATS and fit scores; the biggest keyword gap is the lack of explicit mention of "no‑code tools" and formal "PRD" creation.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>customer obsession, product judgment, OKRs, prototype, workflow automation, A/B testing</t>
+          <t>no-code tools, product analytics tools, PRD, competition analysis, market analysis, OKRs</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,29 +618,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Confidential Careers</t>
+          <t>Smart Food Safe</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -648,25 +650,25 @@
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑4 year requirement and title level, but the resume lacks several exact JD terms such as API and post‑launch iteration, lowering the ATS score. Overall fit is strong due to relevant SaaS and GenAI experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>API design, post‑launch iteration, technical design discussions, AI tools usage, ruthless prioritization</t>
+          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +686,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>Revantage, A Blackstone Portfolio Company</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -716,25 +718,25 @@
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
+          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +754,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -784,7 +786,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>78</v>
@@ -797,12 +799,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; it contains many JD keywords but lacks ecommerce‑specific terms, lowering the fit.</t>
+          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>ecommerce, API documentation, A/B testing, OKRs, NPS improvement, data pipeline, SQL reporting</t>
+          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,24 +827,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,9 +853,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
@@ -865,12 +865,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because the resume contains many relevant product management terms but lacks several common JD keywords; fit score is higher due to strong SaaS and GenAI experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -888,34 +888,34 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Lucidity</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -924,19 +924,19 @@
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides few concrete keywords, resulting in moderate ATS keyword coverage; the strongest gap is the lack of explicit OKR or A/B testing experience.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, User segmentation, Roadmap planning, KPIs tracking</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,29 +954,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Bright Money</t>
+          <t>Infinity Learn</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI and Agentic</t>
+          <t>Growth Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -985,26 +985,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and location, so hard rules pass; however the resume lacks several fintech‑specific terms (LLM, credit‑card, marketplace) reducing the ATS match.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the target role, but the JD lacks many specific keywords resulting in moderate ATS coverage; the biggest gap is the absence of explicit growth‑focused metrics and tools.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>LLM, AI money assistant, credit card product, FinTech, Marketplace dynamics, A/B testing, OKRs, NPS improvement</t>
+          <t>A/B testing, OKRs, Growth metrics (e.g., MAU, NPS), Mixpanel or Amplitude, PLG strategy</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1022,29 +1020,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Notified</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, AIRX</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1053,26 +1051,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as backlog refinement and product roadmap, lowering the ATS score.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks specific keywords, leading to moderate ATS confidence; the most notable gap is the absence of explicit product‑metrics and experimentation terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>backlog refinement, product roadmap, product marketing, customer success, investor relations, public relations</t>
+          <t>OKRs, A/B testing, Product metrics, User research, Roadmap planning, Stakeholder alignment frameworks (e.g., RICE), Growth metrics (MAU, NPS), Data instrumentation (Mixpanel, Amplitude)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1090,24 +1086,24 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1126,19 +1122,19 @@
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many Agile and product delivery terms but lacks several JD‑specific data‑product keywords, lowering the ATS score; the main gap is missing explicit customer‑segmentation and data‑governance terminology.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>customer segmentation, personalisation, insight datasets, data governance, analytics collaboration, data science partnership, A/B testing, OKRs</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1156,24 +1152,24 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1183,30 +1179,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1229,24 +1223,24 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>Bright Money</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Consumer App Experience)</t>
+          <t>Product Manager - AI and Agentic</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1255,24 +1249,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is low due to limited overlap with JD-specific terms like consumer native apps and insurance, while fit score is higher because the candidate's travel‑tech and SaaS background aligns well with Booking.com's consumer travel product domain.</t>
+          <t>The candidate meets the 4‑year experience requirement and location, so hard rules pass; however the resume lacks several fintech‑specific terms (LLM, credit‑card, marketplace) reducing the ATS match.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>consumer-facing native applications, e-commerce, A/B testing, OKRs, NPS improvement, post‑book insurance experience, regulated insurance, two‑sided marketplace</t>
+          <t>LLM, AI money assistant, credit card product, FinTech, Marketplace dynamics, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1295,24 +1291,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Tesco Bengaluru</t>
+          <t>Notified</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1323,22 +1319,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume lacks several JD-specific data product terms such as segmentation and governance, lowering the ATS score, while the candidate's GenAI and SaaS background gives a moderate fit.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as backlog refinement and product roadmap, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>customer segmentation, audience filters, insights datasets, data governance, stakeholder interviews, A/B testing, Snowflake</t>
+          <t>backlog refinement, product roadmap, product marketing, customer success, investor relations, public relations</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1356,57 +1352,55 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>AppBroda</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Agentic, Customer Engagement</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; however the resume lacks several JD‑specific terms such as LLMs and internal tooling, lowering the ATS score. The strongest keyword gap is the absence of "Large Language Models".</t>
+          <t>The candidate meets the 4‑year experience requirement and the role is not senior, so hard rules pass; however, the job description provides no concrete keywords, resulting in moderate keyword coverage and a few gaps.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Large Language Models (LLMs), AI‑motivated chat tools, Enterprise Business Intelligence (BI), internal tooling, cross‑functional collaboration with sellers, analysts, and operations</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1420,38 +1414,38 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>LiveRamp</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -1460,19 +1454,19 @@
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many Agile and product delivery terms but lacks several JD‑specific data‑product keywords, lowering the ATS score; the main gap is missing explicit customer‑segmentation and data‑governance terminology.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+          <t>customer segmentation, personalisation, insight datasets, data governance, analytics collaboration, data science partnership, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1486,38 +1480,38 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Narayana Health</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager (AI)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1528,19 +1522,19 @@
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1554,7 +1548,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1563,35 +1557,33 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Zynga</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
@@ -1603,12 +1595,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords but lacks gaming‑specific terms, lowering the ATS score. The biggest gap is the absence of mobile gaming and player‑centric metrics.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>mobile gaming, A/B testing, user acquisition, KPIs, OKRs, Mixpanel, player engagement metrics, live ops</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1622,28 +1614,28 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Northern Trust</t>
+          <t>Tesco Bengaluru</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1653,56 +1645,720 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="H18" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title). The resume lacks several JD-specific data product terms such as segmentation and governance, lowering the ATS score, while the candidate's GenAI and SaaS background gives a moderate fit.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>customer segmentation, audience filters, insights datasets, data governance, stakeholder interviews, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>MSN Laboratories</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the basic experience and location criteria and aligns well with the product manager role, but it lacks several common PM keywords that many ATS parsers expect, lowering the ATS score; the strongest gap is the absence of explicit methodology terms like OKRs or A/B testing.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ThinkWise Consulting LLP</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager / Business Analyst</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit keywords, leading to moderate ATS confidence; the strongest gap is the absence of common product analytics and prioritization terms.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>LiveRamp</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager, Agentic, Customer Engagement</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; however the resume lacks several JD‑specific terms such as LLMs and internal tooling, lowering the ATS score. The strongest keyword gap is the absence of "Large Language Models".</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Large Language Models (LLMs), AI‑motivated chat tools, Enterprise Business Intelligence (BI), internal tooling, cross‑functional collaboration with sellers, analysts, and operations</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Amgen</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager (AI)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TriNet</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Autodesk</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (Data Ingestion &amp; Delivery)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune/Pimpri-Chinchwad Area</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns closely with the target role, but the job description provides few concrete keywords, resulting in moderate ATS keyword coverage; the most notable gap is the absence of explicit data‑ingestion and delivery terminology.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Data ingestion pipelines, ETL processes, Data delivery APIs, SQL performance tuning, A/B testing, OKRs</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>AskTalos</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager – B2B SaaS</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the resume lacks several core SaaS and product‑management keywords from the JD, lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ORMAE</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the generic JD provides few concrete keywords, leading to moderate ATS confidence and a solid but not outstanding fit.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking (e.g., MAU, NPS), Product analytics tools (e.g., Mixpanel, Amplitude)</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Northern Trust</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>The resume meets the hard rules (4 years experience, correct title) and contains many core product management keywords, but lacks several JD-specific terms such as Azure DevOps, SAFe, and financial‑services context, limiting the ATS score. The most important keyword gap is the absence of Azure DevOps/SAFe experience.</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Azure DevOps, SAFe, Microsoft Copilot, financial services, wealth management, product roadmaps, release planning</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -1725,6 +2381,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1736,7 +2402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1903,7 +2569,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -1971,7 +2637,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2039,19 +2705,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bright Money</t>
+          <t>1% Club</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Credit Card</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2060,26 +2726,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). The resume lacks core fintech and credit‑card terminology, lowering both scores; the biggest gap is missing credit‑card/financial‑services keywords.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many typical product manager keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience gives a decent fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>credit card, risk management, credit underwriting, financial services marketplace, A/B testing, product metrics, growth funnel, roadmap planning, KYC/AML compliance</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product-led growth (PLG)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2097,55 +2761,57 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Namma Yatri</t>
+          <t>Bright Money</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Credit Card</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title), but the resume contains few of the specific mobility platform keywords from the JD, leading to a low ATS score; the biggest gap is missing terms like Beckn Protocol and ONDC.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). The resume lacks core fintech and credit‑card terminology, lowering both scores; the biggest gap is missing credit‑card/financial‑services keywords.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Beckn Protocol, ONDC network, API design and integration, A/B testing, OKRs, Marketplace dynamics, Two-sided platform, NPS improvement, Growth metrics (MAU, retention)</t>
+          <t>credit card, risk management, credit underwriting, financial services marketplace, A/B testing, product metrics, growth funnel, roadmap planning, KYC/AML compliance</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2173,45 +2839,47 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Opella</t>
+          <t>geidea</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner - SAP HUB</t>
+          <t>CP Product Owner</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many SAP‑specific terms and data‑hub experience, leading to a moderate ATS score and a low fit score due to domain mismatch.</t>
+          <t>Hard rules are satisfied, but the resume contains few of the payment‑specific keywords and tools required by the JD, leading to a low ATS score; the biggest gap is the lack of any card‑payment or fintech terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SAP, Data extraction, Unified data model, Data privacy, SOX compliance, Regulatory compliance, Cybersecurity requirements, SLA management, Test case execution</t>
+          <t>card payment flows (authorization, clearing, settlement), EMV, ISO 8583, UAT (User Acceptance Testing), Confluence, partner integration delivery, SOPs, release notes, KPIs such as approval rates and transaction volumes</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2225,38 +2893,38 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Namma Yatri</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -2265,19 +2933,19 @@
         <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title), but the resume contains few of the specific mobility platform keywords from the JD, leading to a low ATS score; the biggest gap is missing terms like Beckn Protocol and ONDC.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>Beckn Protocol, ONDC network, API design and integration, A/B testing, OKRs, Marketplace dynamics, Two-sided platform, NPS improvement, Growth metrics (MAU, retention)</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2291,61 +2959,61 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>EMotorad</t>
+          <t>Bhaktilok</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Business Systems and Operations</t>
+          <t>Product Manager / Associate Product Manager — Growth &amp; Monetization</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, but lacks many ERP and manufacturing-specific terms and the location does not match Pune, resulting in moderate ATS and fit scores; the biggest keyword gap is the absence of ERPNext/Frappe experience.</t>
+          <t>Hard rules pass, but the resume misses many core JD keywords (e.g., Mixpanel, subscription pricing experiments) and lacks consumer‑app/payment experience, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>ERPNext, Frappe, production planning, inventory management, order-to-cash, procurement, workflow automation, supply chain, manufacturing operations, OKRs</t>
+          <t>Mixpanel, A/B testing, subscription growth, pricing experiments, UPI, autopay, Razorpay, Juspay, Hindi</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2359,87 +3027,487 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>Opella</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors Employment Changes Product Owner - VOIS</t>
+          <t>Data Product Owner - SAP HUB</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks many SAP‑specific terms and data‑hub experience, leading to a moderate ATS score and a low fit score due to domain mismatch.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>SAP, Data extraction, Unified data model, Data privacy, SOX compliance, Regulatory compliance, Cybersecurity requirements, SLA management, Test case execution</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Amgen</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Micron Technology</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>EMotorad</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager- Business Systems and Operations</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement, but lacks many ERP and manufacturing-specific terms and the location does not match Pune, resulting in moderate ATS and fit scores; the biggest keyword gap is the absence of ERPNext/Frappe experience.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>ERPNext, Frappe, production planning, inventory management, order-to-cash, procurement, workflow automation, supply chain, manufacturing operations, OKRs</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>UBS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Market Risk Exposure Platforms Integration</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience rule, but it lacks many core product‑manager keywords from the UBS risk‑platform JD and does not show location alignment, resulting in a low ATS pass likelihood; the biggest gap is the absence of risk‑domain terminology.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Market Risk, Risk Exposure, Integration, Financial Services, Regulatory compliance, OKRs, Product roadmap, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>VOIS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SAP SuccessFactors Employment Changes Product Owner - VOIS</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Hard rules pass, but the resume lacks core HR and SAP SuccessFactors keywords and the title does not align with Product Owner, resulting in low ATS and modest fit scores; the biggest gap is missing SAP SuccessFactors/HR lifecycle terminology.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>SAP SuccessFactors, Employee Central, HR lifecycle, employment changes, HR Business Partner</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>HARMAN India</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pimpri Chinchwad, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2454,6 +3522,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-08
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>YourDOST</t>
+          <t>Smart Food Safe</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager/ Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>81</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches the Associate Product Manager level, yielding solid ATS and fit scores; the biggest keyword gap is the lack of explicit mention of "no‑code tools" and formal "PRD" creation.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>no-code tools, product analytics tools, PRD, competition analysis, market analysis, OKRs</t>
+          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,29 +618,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Smart Food Safe</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,26 +649,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
+          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
+          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -686,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Revantage, A Blackstone Portfolio Company</t>
+          <t>Cite AI</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>76</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is solid due to strong keyword overlap (Jira, Agile, sprint ceremonies, GenAI) but missing core AI‑product terms like model drift and KPI tracking. Fit score is high because the candidate’s SaaS and GenAI experience aligns well with the AI‑powered product focus.</t>
+          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>model drift, bias mitigation, ethical considerations, KPIs, success metrics, product roadmap, OKRs, A/B testing</t>
+          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -754,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>Modlix</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager - AI / B2B SaaS/Martech</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -789,22 +785,22 @@
         <v>4</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
+          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -822,24 +818,24 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -849,7 +845,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -858,19 +854,19 @@
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because the resume contains many relevant product management terms but lacks several common JD keywords; fit score is higher due to strong SaaS and GenAI experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking, NPS improvement</t>
+          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -893,24 +889,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Lucidity</t>
+          <t>Precisely</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager - AI Platform</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -921,22 +917,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides few concrete keywords, resulting in moderate ATS keyword coverage; the strongest gap is the lack of explicit OKR or A/B testing experience.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is close enough to the target role, but the JD lacks explicit keywords, resulting in moderate ATS confidence; the biggest gap is the absence of common product management frameworks and analytics tools.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, User segmentation, Roadmap planning, KPIs tracking</t>
+          <t>OKRs, A/B testing, Metrics tracking (e.g., Mixpanel, Amplitude), Roadmap planning, User research / JTBD</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,29 +950,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Infinity Learn</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Growth Product Manager</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -985,24 +981,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title aligns with the target role, but the JD lacks many specific keywords resulting in moderate ATS coverage; the biggest gap is the absence of explicit growth‑focused metrics and tools.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Growth metrics (e.g., MAU, NPS), Mixpanel or Amplitude, PLG strategy</t>
+          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1025,24 +1023,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Notified</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AIRX</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1056,19 +1054,19 @@
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks specific keywords, leading to moderate ATS confidence; the most notable gap is the absence of explicit product‑metrics and experimentation terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as backlog refinement and product roadmap, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Product metrics, User research, Roadmap planning, Stakeholder alignment frameworks (e.g., RICE), Growth metrics (MAU, NPS), Data instrumentation (Mixpanel, Amplitude)</t>
+          <t>backlog refinement, product roadmap, product marketing, customer success, investor relations, public relations</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1086,24 +1084,24 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>JUSPAY</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1122,19 +1120,19 @@
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
+          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1157,50 +1155,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Product Platform</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1218,29 +1216,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Bright Money</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI and Agentic</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1249,26 +1247,24 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and location, so hard rules pass; however the resume lacks several fintech‑specific terms (LLM, credit‑card, marketplace) reducing the ATS match.</t>
+          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>LLM, AI money assistant, credit card product, FinTech, Marketplace dynamics, A/B testing, OKRs, NPS improvement</t>
+          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,29 +1282,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Notified</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Assisted Service</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1319,22 +1315,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as backlog refinement and product roadmap, lowering the ATS score.</t>
+          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>backlog refinement, product roadmap, product marketing, customer success, investor relations, public relations</t>
+          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,55 +1348,55 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>AppBroda</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the role is not senior, so hard rules pass; however, the job description provides no concrete keywords, resulting in moderate keyword coverage and a few gaps.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization</t>
+          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1414,7 +1410,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1423,29 +1419,29 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>LiveRamp</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -1454,19 +1450,19 @@
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many Agile and product delivery terms but lacks several JD‑specific data‑product keywords, lowering the ATS score; the main gap is missing explicit customer‑segmentation and data‑governance terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>customer segmentation, personalisation, insight datasets, data governance, analytics collaboration, data science partnership, A/B testing, OKRs</t>
+          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1480,61 +1476,61 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Agentic, Customer Engagement</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; however the resume lacks several JD‑specific terms such as LLMs and internal tooling, lowering the ATS score. The strongest keyword gap is the absence of "Large Language Models".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>Large Language Models (LLMs), AI‑motivated chat tools, Enterprise Business Intelligence (BI), internal tooling, cross‑functional collaboration with sellers, analysts, and operations</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,7 +1544,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1557,29 +1553,29 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Zynga</t>
+          <t>Dr. Reddy's Laboratories</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Manager - Enterprise Processes</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1588,21 +1584,17 @@
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords but lacks gaming‑specific terms, lowering the ATS score. The biggest gap is the absence of mobile gaming and player‑centric metrics.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>mobile gaming, A/B testing, user acquisition, KPIs, OKRs, Mixpanel, player engagement metrics, live ops</t>
-        </is>
-      </c>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the job description provides no specific keywords, limiting the ATS match.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -1614,7 +1606,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -1623,50 +1615,50 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Tesco Bengaluru</t>
+          <t>PDI Technologies</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner III</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume lacks several JD-specific data product terms such as segmentation and governance, lowering the ATS score, while the candidate's GenAI and SaaS background gives a moderate fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant product management terms, but the job description provides no concrete keywords, resulting in moderate ATS confidence and a decent fit based on domain experience.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>customer segmentation, audience filters, insights datasets, data governance, stakeholder interviews, A/B testing, Snowflake</t>
+          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, Stakeholder alignment frameworks (e.g., RICE, MoSCoW), Data analytics tools (e.g., Mixpanel, Amplitude), Product analytics, User research methodologies</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1680,28 +1672,28 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MSN Laboratories</t>
+          <t>TriNet</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1715,24 +1707,26 @@
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F19" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience and location criteria and aligns well with the product manager role, but it lacks several common PM keywords that many ATS parsers expect, lowering the ATS score; the strongest gap is the absence of explicit methodology terms like OKRs or A/B testing.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization, NPS improvement</t>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1755,50 +1749,52 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ThinkWise Consulting LLP</t>
+          <t>AskTalos</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager / Business Analyst</t>
+          <t>Technical Product Manager – B2B SaaS</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit keywords, leading to moderate ATS confidence; the strongest gap is the absence of common product analytics and prioritization terms.</t>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the resume lacks several core SaaS and product‑management keywords from the JD, lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1812,7 +1808,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -1826,24 +1822,24 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>LiveRamp</t>
+          <t>Northern Trust</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1852,19 +1848,19 @@
         <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+          <t>The resume meets the hard rules (4 years experience, correct title) and contains many core product management keywords, but lacks several JD-specific terms such as Azure DevOps, SAFe, and financial‑services context, limiting the ATS score. The most important keyword gap is the absence of Azure DevOps/SAFe experience.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+          <t>Azure DevOps, SAFe, Microsoft Copilot, financial services, wealth management, product roadmaps, release planning</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1878,64 +1874,64 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Rinf</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Agentic, Customer Engagement</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; however the resume lacks several JD‑specific terms such as LLMs and internal tooling, lowering the ATS score. The strongest keyword gap is the absence of "Large Language Models".</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Large Language Models (LLMs), AI‑motivated chat tools, Enterprise Business Intelligence (BI), internal tooling, cross‑functional collaboration with sellers, analysts, and operations</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1944,66 +1940,66 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Equiniti</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager (AI)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant AI/GenAI and SaaS experience, but the resume lacks several JD‑specific terms related to rapid discovery, prototyping, and data‑centric experimentation.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and the title aligns (Associate PM → PM). Strong overlap on core keywords, but a few JD‑specific tools/methodologies are absent.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>rapid discovery sprint, prototype development, pilot testing, user research, A/B testing, OKRs, Snowflake</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -2012,38 +2008,38 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Eightfold</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AI Product Manager I / II - Talent Forge</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -2051,27 +2047,27 @@
         <v>3</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The resume meets the 3‑year minimum and seniority constraints, and contains many core keywords (GenAI, RAG, Agile, Jira, SQL, Power BI, SaaS). The biggest gap is the lack of talent‑domain and cloud platform terms such as Azure/AWS.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>Azure, AWS, agentic AI, talent workflow, headless API, OKRs, A/B testing, Snowflake, NPS improvement, PLG</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2080,21 +2076,21 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2111,11 +2107,13 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pune/Pimpri-Chinchwad Area</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F25" s="2" t="n">
         <v>68</v>
       </c>
@@ -2137,7 +2135,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2146,11 +2144,11 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2160,24 +2158,24 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>Emerson</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager – B2B SaaS</t>
+          <t>Product Manager Ultrasonic Plastics</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -2186,24 +2184,24 @@
         <v>68</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the resume lacks several core SaaS and product‑management keywords from the JD, lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
+          <t>The resume meets the experience and seniority constraints, but lacks several core JD terms such as product roadmap, pricing strategy, and competitive analysis, lowering the ATS score; overall domain and skill alignment are solid, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
+          <t>product roadmap, pricing strategy, competitive analysis, voice of customer, stage‑gate process, go‑to‑market plan, cost optimization, product certification</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2212,7 +2210,7 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
@@ -2221,55 +2219,57 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ORMAE</t>
+          <t>Athisa Health</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F27" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the generic JD provides few concrete keywords, leading to moderate ATS confidence and a solid but not outstanding fit.</t>
+          <t>The resume meets the years and seniority requirements, but lacks many JD‑specific terms (e.g., therapist‑matching, client‑facing platform, success metrics), resulting in a moderate ATS score; overall fit is decent due to strong SaaS and GenAI experience but limited health‑tech domain exposure.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking (e.g., MAU, NPS), Product analytics tools (e.g., Mixpanel, Amplitude)</t>
+          <t>therapist-matching, client-facing platform, success metrics, lean documentation, operations workflow analysis, build vs buy evaluation, no-code/low-code platforms</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -2278,42 +2278,44 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Northern Trust</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F28" s="2" t="n">
         <v>68</v>
       </c>
@@ -2325,17 +2327,17 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, correct title) and contains many core product management keywords, but lacks several JD-specific terms such as Azure DevOps, SAFe, and financial‑services context, limiting the ATS score. The most important keyword gap is the absence of Azure DevOps/SAFe experience.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, SAFe, Microsoft Copilot, financial services, wealth management, product roadmaps, release planning</t>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -2344,21 +2346,223 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Narayana Health</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many generic product management keywords but lacks HR‑specific terms and compliance language, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Core HR, Roles &amp; Access, access governance, information security, data protection, KPIs, Tesco Flow methodology, OKRs, Jobs‑to‑be‑Done</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>SKU Digital</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title). The resume lacks key healthcare/RCM terminology, lowering both scores; the biggest gap is missing medical coding and claims processing keywords.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Revenue Cycle Management (RCM), medical coding, claims processing, ICD-10-CM, CPT, HCPCS, LLM, cloud-native platform, healthcare regulations</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2391,6 +2595,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2402,7 +2609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2522,9 +2729,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>55</v>
       </c>
@@ -2569,7 +2774,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2637,47 +2842,45 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Snapmint</t>
+          <t>GravityONE</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Seller Experience</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (4 years experience) and has no senior title, so hard rules pass; however the resume lacks many seller‑experience specific keywords from the JD, lowering the ATS score. The biggest gap is missing marketplace‑seller terminology like "seller onboarding" and "catalog management".</t>
+          <t>The resume meets the 4‑year experience requirement and contains relevant product management experience, but the job description provides no concrete keywords, resulting in low ATS keyword density; the biggest gap is the absence of typical PM framework terms.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>seller onboarding, catalog management, pricing and promotions, KYC verification, seller performance dashboards, self‑service tools, marketplace dynamics, order management</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking, Product analytics (e.g., Mixpanel), RICE prioritization, Customer segmentation</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2695,29 +2898,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1% Club</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II - Ads</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2726,24 +2929,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many typical product manager keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience gives a decent fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many fintech‑specific terms and ads‑product keywords, resulting in a modest ATS score and limited domain fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product-led growth (PLG)</t>
+          <t>Payments, Fintech, Ads platform, A/B testing, OKRs, API integration, Risk intelligence, NPS improvement, Revenue growth metrics</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2761,29 +2966,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bright Money</t>
+          <t>Bureau</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Credit Card</t>
+          <t>Product Manager (RASP)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2793,25 +2998,25 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 3‑year minimum and no senior title). The resume lacks core fintech and credit‑card terminology, lowering both scores; the biggest gap is missing credit‑card/financial‑services keywords.</t>
+          <t>The candidate meets the 4‑year requirement and seniority rules, but the resume lacks most security‑focused keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>credit card, risk management, credit underwriting, financial services marketplace, A/B testing, product metrics, growth funnel, roadmap planning, KYC/AML compliance</t>
+          <t>Android, iOS, mobile security, runtime application self‑protection (RASP), code obfuscation, anti‑tampering, MITM protection, SDK integration, Zero Trust framework</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2829,40 +3034,38 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>geidea</t>
+          <t>Thommidhi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CP Product Owner</t>
+          <t>Product Manager Intern</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Kolkata Area</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>45</v>
       </c>
@@ -2874,12 +3077,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume contains few of the payment‑specific keywords and tools required by the JD, leading to a low ATS score; the biggest gap is the lack of any card‑payment or fintech terminology.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific keywords and domain experience with creator platforms, leading to a modest ATS score and only moderate fit.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>card payment flows (authorization, clearing, settlement), EMV, ISO 8583, UAT (User Acceptance Testing), Confluence, partner integration delivery, SOPs, release notes, KPIs such as approval rates and transaction volumes</t>
+          <t>A/B testing, user interviews, spec writing, scope reduction, product discovery, prediction-to-outcome, early-stage product strategy</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2893,7 +3096,7 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -2902,50 +3105,50 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Namma Yatri</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Engineering Product Manager | 15+ Years</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title), but the resume contains few of the specific mobility platform keywords from the JD, leading to a low ATS score; the biggest gap is missing terms like Beckn Protocol and ONDC.</t>
+          <t>No hard rule violations; however, the job description provides few concrete keywords, resulting in limited keyword overlap and a modest ATS score. The most important gap is the absence of typical Cisco engineering product management terms.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Beckn Protocol, ONDC network, API design and integration, A/B testing, OKRs, Marketplace dynamics, Two-sided platform, NPS improvement, Growth metrics (MAU, retention)</t>
+          <t>Cloud infrastructure, Network automation, API strategy, Metrics and reporting (e.g., NPS, MAU), Roadmap planning</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2959,61 +3162,59 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bhaktilok</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager / Associate Product Manager — Growth &amp; Monetization</t>
+          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume misses many core JD keywords (e.g., Mixpanel, subscription pricing experiments) and lacks consumer‑app/payment experience, leading to low ATS and fit scores.</t>
+          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, subscription growth, pricing experiments, UPI, autopay, Razorpay, Juspay, Hindi</t>
+          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3027,7 +3228,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -3036,24 +3237,24 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Opella</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner - SAP HUB</t>
+          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3064,22 +3265,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many SAP‑specific terms and data‑hub experience, leading to a moderate ATS score and a low fit score due to domain mismatch.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP, Data extraction, Unified data model, Data privacy, SOX compliance, Regulatory compliance, Cybersecurity requirements, SLA management, Test case execution</t>
+          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3097,29 +3298,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Broadridge India</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3128,26 +3329,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
+          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
+          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3165,34 +3364,34 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Serrala</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Product Owner (SAP)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -3201,19 +3400,19 @@
         <v>45</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>No hard rule violations; however the JD provides virtually no keywords, resulting in low ATS keyword overlap. The biggest gap is the lack of SAP‑specific terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>SAP, product roadmap, OKRs, RICE prioritization, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3227,61 +3426,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EMotorad</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Business Systems and Operations</t>
+          <t>SAP SuccessFactors Employment Changes Product Owner - VOIS</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, but lacks many ERP and manufacturing-specific terms and the location does not match Pune, resulting in moderate ATS and fit scores; the biggest keyword gap is the absence of ERPNext/Frappe experience.</t>
+          <t>Hard rules pass, but the resume lacks core HR and SAP SuccessFactors keywords and the title does not align with Product Owner, resulting in low ATS and modest fit scores; the biggest gap is missing SAP SuccessFactors/HR lifecycle terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>ERPNext, Frappe, production planning, inventory management, order-to-cash, procurement, workflow automation, supply chain, manufacturing operations, OKRs</t>
+          <t>SAP SuccessFactors, Employee Central, HR lifecycle, employment changes, HR Business Partner</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3304,55 +3501,57 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>2070Health</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Market Risk Exposure Platforms Integration</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience rule, but it lacks many core product‑manager keywords from the UBS risk‑platform JD and does not show location alignment, resulting in a low ATS pass likelihood; the biggest gap is the absence of risk‑domain terminology.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Market Risk, Risk Exposure, Integration, Financial Services, Regulatory compliance, OKRs, Product roadmap, A/B testing, Snowflake</t>
+          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -3361,64 +3560,66 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>xponentiate</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors Employment Changes Product Owner - VOIS</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core HR and SAP SuccessFactors keywords and the title does not align with Product Owner, resulting in low ATS and modest fit scores; the biggest gap is missing SAP SuccessFactors/HR lifecycle terminology.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors, Employee Central, HR lifecycle, employment changes, HR Business Partner</t>
+          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -3427,64 +3628,66 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HARMAN India</t>
+          <t>Mergenomics</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Automotive Product Manager - (HW, SW, Mech, HUD/Display, GTM)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pimpri Chinchwad, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F16" s="2" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>45</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core automotive and hardware/software keywords required by the JD and does not demonstrate location alignment, resulting in a low ATS score; the candidate's SaaS and GenAI background only tangentially matches the automotive cockpit domain, leading to a modest fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to good keyword overlap on Agile, Jira, SaaS but missing many healthcare-specific terms; fit score is low because the candidate's domain experience does not align with RCM/medical coding.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>HUD, In-vehicle infotainment, OEM integration, TAM/SAM/SOM, MRD, PRD, platform reuse, system-level integration, make &amp; buy analysis</t>
+          <t>medical coding, claims processing, ICD-10-CM, CPT, HCPCS, revenue cycle management, healthcare regulations, go-to-market strategy, customer research</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -3502,12 +3705,78 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager – Procurement Technology – Contingency Workforce Management, VP</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>MH, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The JD’s corporate title includes "VP", triggering a hard rule that forces both scores below 30 despite the candidate’s 4 years of experience; the most important keyword gap is the absence of any procurement‑specific terminology such as "source‑to‑pay" or "IR35".</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>source-to-pay, IRIR35 compliance, procurement interoperability, vendor risk management, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Indeed, Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3528,6 +3797,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-09
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Smart Food Safe</t>
+          <t>InCred Financial Services</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers most JD keywords but lacks a few analytics and measurement terms, leading to a strong ATS score and a solid fit despite limited fintech domain exposure.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,29 +618,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>YourDOST</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager/ Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -654,19 +654,19 @@
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches the Associate Product Manager level, yielding solid ATS and fit scores; the biggest keyword gap is the lack of explicit mention of "no‑code tools" and formal "PRD" creation.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
+          <t>no-code tools, product analytics tools, PRD, competition analysis, market analysis, OKRs</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Cite AI</t>
+          <t>Smart Food Safe</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,24 +715,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
+          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,57 +752,57 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Modlix</t>
+          <t>myHQ by ANAROCK</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI / B2B SaaS/Martech</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
+          <t>The candidate meets the experience requirement (4 years) and seniority constraints, but the resume lacks several JD-specific tools and methodologies, lowering the ATS score; the strongest keyword gap is the absence of Mixpanel/Amplitude experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
+          <t>Mixpanel or Amplitude, A/B testing, No-code prototyping tools, User research and behavioral data analysis, Product dashboards and KPI monitoring</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -823,50 +825,52 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Cite AI</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many PM keywords but misses core JD terms like product roadmap and P&amp;L, lowering the ATS score; overall domain fit is good.</t>
+          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product P&amp;L, business case, product positioning, voice of customer, pricing strategy, product data integrity</t>
+          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -884,29 +888,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Precisely</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI Platform</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,24 +919,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is close enough to the target role, but the JD lacks explicit keywords, resulting in moderate ATS confidence; the biggest gap is the absence of common product management frameworks and analytics tools.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking (e.g., Mixpanel, Amplitude), Roadmap planning, User research / JTBD</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,29 +956,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>Modlix</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Product Manager - AI / B2B SaaS/Martech</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -982,25 +988,25 @@
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
+          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,24 +1024,24 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Notified</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1049,7 +1055,9 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
@@ -1061,12 +1069,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several core JD terms such as backlog refinement and product roadmap, lowering the ATS score.</t>
+          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>backlog refinement, product roadmap, product marketing, customer success, investor relations, public relations</t>
+          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1084,29 +1092,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JUSPAY</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1115,24 +1123,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
+          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1155,24 +1165,24 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Okta</t>
+          <t>JUSPAY</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Product Platform</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,24 +1191,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
+          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1221,19 +1233,19 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>greytHR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1249,22 +1261,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
+          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
+          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1287,24 +1299,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Assisted Service</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1313,24 +1325,26 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume misses several finance‑focused and eBay‑specific keywords, lowering the ATS score; the candidate's domain is SaaS/enterprise rather than marketplace financial services, creating a skills gap.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>financial services, payments, fraud detection, risk management, trust &amp; safety, marketplace dynamics, customer experience (CX), AI‑first, A/B testing</t>
+          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,55 +1362,57 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several JD‑specific terms such as service design and OKRs, lowering the ATS score; overall domain and skill alignment is strong.</t>
+          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>service design, OKRs, KPIs, A/B testing, Snowflake, Mixpanel, global partnership, roadmap development, data science insights</t>
+          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1410,59 +1426,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>LiveRamp</t>
+          <t>JAGGAER</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, AI Data &amp; Insight Products</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product and technical terms but misses several JD‑specific activation and data‑privacy keywords, lowering the ATS score. The candidate’s SaaS and GenAI experience aligns well with LiveRamp’s domain, giving a solid fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific tools and frameworks; overall fit is strong due to relevant SaaS and GenAI experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>campaign configuration, activation workflow, monitoring dashboards, data onboarding, privacy compliance, customer segmentation, product vision and roadmap</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1480,29 +1496,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Arcesium</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Agentic, Customer Engagement</t>
+          <t>Product Manager - Tax</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1511,26 +1527,24 @@
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; however the resume lacks several JD‑specific terms such as LLMs and internal tooling, lowering the ATS score. The strongest keyword gap is the absence of "Large Language Models".</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume lacks several JD‑specific tools and methodologies, lowering the ATS score; the strongest gap is the absence of common product analytics and prioritization terms.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Large Language Models (LLMs), AI‑motivated chat tools, Enterprise Business Intelligence (BI), internal tooling, cross‑functional collaboration with sellers, analysts, and operations</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,29 +1562,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reddy's Laboratories</t>
+          <t>TriNet</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Enterprise Processes</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1579,22 +1593,28 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the job description provides no specific keywords, limiting the ATS match.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -1615,52 +1635,48 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PDI Technologies</t>
+          <t>Anchanto</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner III</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant product management terms, but the job description provides no concrete keywords, resulting in moderate ATS confidence and a decent fit based on domain experience.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, Stakeholder alignment frameworks (e.g., RICE, MoSCoW), Data analytics tools (e.g., Mixpanel, Amplitude), Product analytics, User research methodologies</t>
-        </is>
-      </c>
+          <t>Hard rules pass; the candidate meets the experience level and title seniority. ATS score is moderate due to lack of explicit JD keywords, while fit score is high because of strong SaaS and GenAI product experience.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -1672,61 +1688,59 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>TIAA</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Owner role, but the resume lacks several JD-specific keywords, lowering the ATS score; overall domain and skill fit are strong.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1740,21 +1754,21 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -1822,19 +1836,19 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Northern Trust</t>
+          <t>Zywave</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1848,19 +1862,19 @@
         <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, correct title) and contains many core product management keywords, but lacks several JD-specific terms such as Azure DevOps, SAFe, and financial‑services context, limiting the ATS score. The most important keyword gap is the absence of Azure DevOps/SAFe experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core API and security keywords, lowering the ATS score, while the overall SaaS and enterprise experience gives a decent fit.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, SAFe, Microsoft Copilot, financial services, wealth management, product roadmaps, release planning</t>
+          <t>REST APIs, OAuth, SSO, API governance, data modeling, security compliance, BI reporting tools (e.g., Tableau), OKRs</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1878,60 +1892,62 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Rinf</t>
+          <t>Vena Solutions</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Integrations</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F22" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1940,7 +1956,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -1949,57 +1965,55 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Equiniti</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Compliance</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and the title aligns (Associate PM → PM). Strong overlap on core keywords, but a few JD‑specific tools/methodologies are absent.</t>
+          <t>The resume meets the 4‑year experience requirement and has no senior‑level title conflict, but it lacks many JD‑specific keywords (e.g., education platform names, compliance software, and specific GenAI tool mentions), limiting the ATS score. The strongest keyword gap is the absence of any named GenAI tools such as ChatGPT.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG</t>
+          <t>ChatGPT, Gemini, Claude, AppsAnywhere, Ithos, Regulatory compliance, Accreditation, AI/ML integration, OKRs</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -2008,7 +2022,7 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
@@ -2017,52 +2031,50 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Eightfold</t>
+          <t>Rinf</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager I / II - Talent Forge</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and seniority constraints, and contains many core keywords (GenAI, RAG, Agile, Jira, SQL, Power BI, SaaS). The biggest gap is the lack of talent‑domain and cloud platform terms such as Azure/AWS.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Azure, AWS, agentic AI, talent workflow, headless API, OKRs, A/B testing, Snowflake, NPS improvement, PLG</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2080,7 +2092,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2090,24 +2102,24 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Equiniti</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Data Ingestion &amp; Delivery)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>MH, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -2115,27 +2127,27 @@
         <v>3</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns closely with the target role, but the job description provides few concrete keywords, resulting in moderate ATS keyword coverage; the most notable gap is the absence of explicit data‑ingestion and delivery terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and the title aligns (Associate PM → PM). Strong overlap on core keywords, but a few JD‑specific tools/methodologies are absent.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Data ingestion pipelines, ETL processes, Data delivery APIs, SQL performance tuning, A/B testing, OKRs</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2148,17 +2160,17 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2224,47 +2236,47 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Athisa Health</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>67</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years and seniority requirements, but lacks many JD‑specific terms (e.g., therapist‑matching, client‑facing platform, success metrics), resulting in a moderate ATS score; overall fit is decent due to strong SaaS and GenAI experience but limited health‑tech domain exposure.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>therapist-matching, client-facing platform, success metrics, lean documentation, operations workflow analysis, build vs buy evaluation, no-code/low-code platforms</t>
+          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2282,17 +2294,17 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2360,14 +2372,14 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Narayana Health</t>
+          <t>Athisa Health</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2377,30 +2389,30 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks healthcare‑specific terminology, lowering both scores.</t>
+          <t>The resume meets the years and seniority requirements, but lacks many JD‑specific terms (e.g., therapist‑matching, client‑facing platform, success metrics), resulting in a moderate ATS score; overall fit is decent due to strong SaaS and GenAI experience but limited health‑tech domain exposure.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>clinical domain knowledge, healthcare regulations, HIPAA compliance, EHR integration, patient outcomes metrics, OKRs, A/B testing</t>
+          <t>therapist-matching, client-facing platform, success metrics, lean documentation, operations workflow analysis, build vs buy evaluation, no-code/low-code platforms</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2418,17 +2430,17 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2494,75 +2506,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>SKU Digital</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume lacks key healthcare/RCM terminology, lowering both scores; the biggest gap is missing medical coding and claims processing keywords.</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Revenue Cycle Management (RCM), medical coding, claims processing, ICD-10-CM, CPT, HCPCS, LLM, cloud-native platform, healthcare regulations</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2541,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2715,12 +2658,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Zepto</t>
+          <t>Bureau</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (RASP)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2729,24 +2672,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 2‑year minimum and no senior title). The resume lacks many supply‑chain and logistics keywords required by the JD, lowering the ATS score, while the candidate's SaaS and GenAI experience gives a moderate job‑fit.</t>
+          <t>The candidate meets the 4‑year requirement and seniority rules, but the resume lacks most security‑focused keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Warehouse Management System (WMS), Inventory Management, Order Management System (OMS), Transport Management System (TMS), GTM strategy, competitive analysis, supply chain, product metrics, OKRs</t>
+          <t>Android, iOS, mobile security, runtime application self‑protection (RASP), code obfuscation, anti‑tampering, MITM protection, SDK integration, Zero Trust framework</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2764,57 +2709,55 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>8byte</t>
+          <t>Thommidhi</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – FinTech</t>
+          <t>Product Manager Intern</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Kolkata Area</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title) but lacks many fintech‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of any financial‑technology or regulatory language.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific keywords and domain experience with creator platforms, leading to a modest ATS score and only moderate fit.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Financial technology, Regulatory compliance, Product Requirement Document (PRD), Roadmap, Platform‑scale engineering, Risk management, Institutional customers, Digital workflows, OKRs</t>
+          <t>A/B testing, user interviews, spec writing, scope reduction, product discovery, prediction-to-outcome, early-stage product strategy</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2828,28 +2771,28 @@
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GravityONE</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2859,28 +2802,28 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains relevant product management experience, but the job description provides no concrete keywords, resulting in low ATS keyword density; the biggest gap is the absence of typical PM framework terms.</t>
+          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics tracking, Product analytics (e.g., Mixpanel), RICE prioritization, Customer segmentation</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2894,61 +2837,61 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Ads</t>
+          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many fintech‑specific terms and ads‑product keywords, resulting in a modest ATS score and limited domain fit.</t>
+          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Payments, Fintech, Ads platform, A/B testing, OKRs, API integration, Risk intelligence, NPS improvement, Revenue growth metrics</t>
+          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2962,61 +2905,59 @@
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bureau</t>
+          <t>Broadridge India</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (RASP)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and seniority rules, but the resume lacks most security‑focused keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
+          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Android, iOS, mobile security, runtime application self‑protection (RASP), code obfuscation, anti‑tampering, MITM protection, SDK integration, Zero Trust framework</t>
+          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -3030,38 +2971,38 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Thommidhi</t>
+          <t>Serrala</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Intern</t>
+          <t>Product Owner (SAP)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Greater Kolkata Area</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -3070,19 +3011,19 @@
         <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific keywords and domain experience with creator platforms, leading to a modest ATS score and only moderate fit.</t>
+          <t>No hard rule violations; however the JD provides virtually no keywords, resulting in low ATS keyword overlap. The biggest gap is the lack of SAP‑specific terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user interviews, spec writing, scope reduction, product discovery, prediction-to-outcome, early-stage product strategy</t>
+          <t>SAP, product roadmap, OKRs, RICE prioritization, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -3096,11 +3037,11 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -3110,45 +3051,45 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Engineering Product Manager | 15+ Years</t>
+          <t>Product Manager - Industrial</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; however, the job description provides few concrete keywords, resulting in limited keyword overlap and a modest ATS score. The most important gap is the absence of typical Cisco engineering product management terms.</t>
+          <t>No hard rule violations; the resume shows 4 years experience and appropriate title, but the JD provides no concrete keywords, resulting in low keyword density. The biggest gap is the lack of typical product‑management methodology terms.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Cloud infrastructure, Network automation, API strategy, Metrics and reporting (e.g., NPS, MAU), Roadmap planning</t>
+          <t>OKRs, A/B testing, Product roadmap, User research, Metrics/KPIs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -3162,59 +3103,59 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
+          <t>Product Manager - Market Risk Exposure Platforms Integration</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>52</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
+          <t>The resume meets the 4‑year experience rule, but it lacks many core product‑manager keywords from the UBS risk‑platform JD and does not show location alignment, resulting in a low ATS pass likelihood; the biggest gap is the absence of risk‑domain terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
+          <t>Market Risk, Risk Exposure, Integration, Financial Services, Regulatory compliance, OKRs, Product roadmap, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3228,7 +3169,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -3237,29 +3178,29 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Zinnia</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SAP S4 Hana Product Manager – Procurement Transformation</t>
+          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -3275,12 +3216,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority rules, but it lacks core procurement and SAP S/4HANA terminology, resulting in a low ATS keyword match and limited domain fit.</t>
+          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, Procurement, Blueprinting workshops, Legacy system integration, Enterprise architecture, KPI tracking, Supply chain, Finance integration, Migration planning</t>
+          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3294,59 +3235,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Broadridge India</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
+          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
+          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3360,7 +3301,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -3369,50 +3310,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Serrala</t>
+          <t>BNY</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (SAP)</t>
+          <t>Vice President, POM Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune/Pimpri-Chinchwad Area</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; however the JD provides virtually no keywords, resulting in low ATS keyword overlap. The biggest gap is the lack of SAP‑specific terminology.</t>
+          <t>Hard rule 3 triggers because the target title contains 'VP', so both scores must be below 30 regardless of experience or keywords; the resume lacks senior‑level leadership keywords.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SAP, product roadmap, OKRs, RICE prioritization, A/B testing</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG strategy</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3430,60 +3371,62 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>2070Health</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors Employment Changes Product Owner - VOIS</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core HR and SAP SuccessFactors keywords and the title does not align with Product Owner, resulting in low ATS and modest fit scores; the biggest gap is missing SAP SuccessFactors/HR lifecycle terminology.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors, Employee Central, HR lifecycle, employment changes, HR Business Partner</t>
+          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -3492,28 +3435,28 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2070Health</t>
+          <t>xponentiate</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -3534,19 +3477,19 @@
         <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
+          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3574,19 +3517,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>xponentiate</t>
+          <t>Qonevo Technologies Private Limited</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3596,25 +3539,25 @@
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
+          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
+          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3637,52 +3580,50 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Mergenomics</t>
+          <t>Broadridge</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to good keyword overlap on Agile, Jira, SaaS but missing many healthcare-specific terms; fit score is low because the candidate's domain experience does not align with RCM/medical coding.</t>
+          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>medical coding, claims processing, ICD-10-CM, CPT, HCPCS, revenue cycle management, healthcare regulations, go-to-market strategy, customer research</t>
+          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3700,60 +3641,62 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Deutsche Bank</t>
+          <t>Magicmind Technologies</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Procurement Technology – Contingency Workforce Management, VP</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>MH, India</t>
+          <t>WB, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD’s corporate title includes "VP", triggering a hard rule that forces both scores below 30 despite the candidate’s 4 years of experience; the most important keyword gap is the absence of any procurement‑specific terminology such as "source‑to‑pay" or "IR35".</t>
+          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>source-to-pay, IRIR35 compliance, procurement interoperability, vendor risk management, regulatory compliance</t>
+          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -3766,17 +3709,17 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-10
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -628,19 +628,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>YourDOST</t>
+          <t>Tario</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager/ Product Manager</t>
+          <t>Product Manager - AI-Powered SaaS</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,24 +649,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>79</v>
-      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches the Associate Product Manager level, yielding solid ATS and fit scores; the biggest keyword gap is the lack of explicit mention of "no‑code tools" and formal "PRD" creation.</t>
+          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior‑level title triggers hard rules; the resume covers most core JD terms but lacks several specific keywords like "customer‑facing" and "prototype".</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>no-code tools, product analytics tools, PRD, competition analysis, market analysis, OKRs</t>
+          <t>customer-facing, prototype, A/B testing, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,24 +686,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Smart Food Safe</t>
+          <t>myHQ by ANAROCK</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -711,30 +713,30 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many JD keywords but misses core documentation terms and some cross‑functional collaboration items, leading to a solid but not perfect ATS score.</t>
+          <t>The candidate meets the experience requirement (4 years) and seniority constraints, but the resume lacks several JD-specific tools and methodologies, lowering the ATS score; the strongest keyword gap is the absence of Mixpanel/Amplitude experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>PRD, BRD, FRD, competitive analysis, customer discovery, product roadmap, product performance metrics, sales collaboration, marketing collaboration</t>
+          <t>Mixpanel or Amplitude, A/B testing, No-code prototyping tools, User research and behavioral data analysis, Product dashboards and KPI monitoring</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,39 +754,39 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>myHQ by ANAROCK</t>
+          <t>Cite AI</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
@@ -797,12 +799,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and seniority constraints, but the resume lacks several JD-specific tools and methodologies, lowering the ATS score; the strongest keyword gap is the absence of Mixpanel/Amplitude experience.</t>
+          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel or Amplitude, A/B testing, No-code prototyping tools, User research and behavioral data analysis, Product dashboards and KPI monitoring</t>
+          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,29 +822,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Cite AI</t>
+          <t>Modlix</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - AI / B2B SaaS/Martech</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -852,25 +854,25 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
+          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -888,29 +890,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -919,26 +921,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers many core keywords but misses several key tools and pricing/API monetization terms, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
+          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, API monetization, pricing strategy, customer discovery</t>
+          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -956,29 +956,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Modlix</t>
+          <t>Auric AI Labs</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI / B2B SaaS/Martech</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -987,26 +987,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
+          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1024,29 +1022,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1059,22 +1057,22 @@
         <v>3</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>69</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
+          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1092,29 +1090,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>JUSPAY</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1124,25 +1122,25 @@
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
+          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1165,19 +1163,19 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>JUSPAY</t>
+          <t>greytHR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1192,25 +1190,25 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
+          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
+          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1228,29 +1226,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>greytHR</t>
+          <t>Landmark Group</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1259,24 +1257,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="H12" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
+          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks several planning‑specific keywords (e.g., PRD, UAT, backlog grooming) reducing the ATS score; overall experience aligns reasonably with the role.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
+          <t>PRD, UAT planning and execution, backlog grooming, data pipelines, metrics tracking, recommendations engine, AI‑native workflow</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1294,29 +1294,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, IN P3P</t>
+          <t>Product Manager, Product Platform</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1326,25 +1326,25 @@
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
+          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1362,29 +1362,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1394,25 +1394,25 @@
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
+          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1435,50 +1435,52 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>JAGGAER</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI Data &amp; Insight Products</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific tools and frameworks; overall fit is strong due to relevant SaaS and GenAI experience.</t>
+          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
+          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1492,33 +1494,33 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Arcesium</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Tax</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1527,24 +1529,26 @@
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume lacks several JD‑specific tools and methodologies, lowering the ATS score; the strongest gap is the absence of common product analytics and prioritization terms.</t>
+          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1562,29 +1566,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>PDI Technologies</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner III</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1593,26 +1597,24 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant product management terms, but the job description provides no concrete keywords, resulting in moderate ATS confidence and a decent fit based on domain experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, Stakeholder alignment frameworks (e.g., RICE, MoSCoW), Data analytics tools (e.g., Mixpanel, Amplitude), Product analytics, User research methodologies</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1630,29 +1632,29 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Anchanto</t>
+          <t>Vena Solutions</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Integrations</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1663,20 +1665,24 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the candidate meets the experience level and title seniority. ATS score is moderate due to lack of explicit JD keywords, while fit score is high because of strong SaaS and GenAI product experience.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -1692,60 +1698,60 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TIAA</t>
+          <t>Rinf</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Owner role, but the resume lacks several JD-specific keywords, lowering the ATS score; overall domain and skill fit are strong.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -1754,7 +1760,7 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
@@ -1763,57 +1769,55 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AskTalos</t>
+          <t>Emerson</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager – B2B SaaS</t>
+          <t>Product Manager Ultrasonic Plastics</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the resume lacks several core SaaS and product‑management keywords from the JD, lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
+          <t>The resume meets the experience and seniority constraints, but lacks several core JD terms such as product roadmap, pricing strategy, and competitive analysis, lowering the ATS score; overall domain and skill alignment are solid, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Product‑led growth (PLG)</t>
+          <t>product roadmap, pricing strategy, competitive analysis, voice of customer, stage‑gate process, go‑to‑market plan, cost optimization, product certification</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -1822,7 +1826,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -1831,55 +1835,57 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Zywave</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F21" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume misses several core API and security keywords, lowering the ATS score, while the overall SaaS and enterprise experience gives a decent fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>REST APIs, OAuth, SSO, API governance, data modeling, security compliance, BI reporting tools (e.g., Tableau), OKRs</t>
+          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -1888,38 +1894,38 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Vena Solutions</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Integrations</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1927,27 +1933,27 @@
         <v>3</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1956,64 +1962,66 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>Knorr-Bremse</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Compliance</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F23" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G23" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="G23" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="H23" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑level title conflict, but it lacks many JD‑specific keywords (e.g., education platform names, compliance software, and specific GenAI tool mentions), limiting the ATS score. The strongest keyword gap is the absence of any named GenAI tools such as ChatGPT.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, Power BI, Agile, SQL) but lacks several trailer‑specific portfolio and change‑management terms, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>ChatGPT, Gemini, Claude, AppsAnywhere, Ithos, Regulatory compliance, Accreditation, AI/ML integration, OKRs</t>
+          <t>Change Request (CR) process, Portfolio optimization, VaVe pipeline, Phase‑in/phase‑out tracking, Supply chain coordination, Cost‑value engineering, Trailer product wiring, Ramp‑up monitoring</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -2022,64 +2030,66 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Rinf</t>
+          <t>Knorr-Bremse AG</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>Mulshi, Maharashtra, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F24" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because key JD terms like Power BI, Jira, Agile, stakeholder management appear, but many portfolio‑ and change‑management keywords are missing. Fit score is lower due to limited trailer/vehicle product experience.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
+          <t>portfolio optimization, change request (CR) process, VaVe pipeline, phase‑in / phase‑out tracking, cost optimization, Excel reporting, product lifecycle documentation</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2092,421 +2102,17 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Equiniti</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and the title aligns (Associate PM → PM). Strong overlap on core keywords, but a few JD‑specific tools/methodologies are absent.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Emerson</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager Ultrasonic Plastics</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>MH, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the experience and seniority constraints, but lacks several core JD terms such as product roadmap, pricing strategy, and competitive analysis, lowering the ATS score; overall domain and skill alignment are solid, giving a decent fit score.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, pricing strategy, competitive analysis, voice of customer, stage‑gate process, go‑to‑market plan, cost optimization, product certification</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Indeed, Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Amazon.com</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, IN P3P</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager II</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>TS, India</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Indeed, Linkedin</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Athisa Health</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>TS, India</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the years and seniority requirements, but lacks many JD‑specific terms (e.g., therapist‑matching, client‑facing platform, success metrics), resulting in a moderate ATS score; overall fit is decent due to strong SaaS and GenAI experience but limited health‑tech domain exposure.</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>therapist-matching, client-facing platform, success metrics, lean documentation, operations workflow analysis, build vs buy evaluation, no-code/low-code platforms</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Tesco</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many generic product management keywords but lacks HR‑specific terms and compliance language, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Core HR, Roles &amp; Access, access governance, information security, data protection, KPIs, Tesco Flow methodology, OKRs, Jobs‑to‑be‑Done</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -2535,12 +2141,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2552,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2719,45 +2319,45 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Thommidhi</t>
+          <t>Eli Lilly and Company</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Intern</t>
+          <t>Product Manager – Enterprise AI Operations &amp; Observability</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Greater Kolkata Area</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific keywords and domain experience with creator platforms, leading to a modest ATS score and only moderate fit.</t>
+          <t>No explicit years or seniority violations, but the JD provides virtually no keyword detail, resulting in a low ATS match; the candidate's GenAI and enterprise SaaS background aligns well with an Enterprise AI Operations role.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user interviews, spec writing, scope reduction, product discovery, prediction-to-outcome, early-stage product strategy</t>
+          <t>Observability, AI Operations, ML Ops, Metrics &amp; Monitoring, Alerting frameworks, Kubernetes, Prometheus, Grafana, Data pipeline orchestration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2771,33 +2371,33 @@
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Keka HR</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager – Finance &amp; Planning</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2811,21 +2411,17 @@
         <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
-        </is>
-      </c>
+          <t>No explicit hard rule violations, but the job description provides virtually no keywords, resulting in a low ATS match; the candidate's strong SaaS and GenAI background is the main fit factor.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2846,24 +2442,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager, Product Operations - Measurement &amp; Reporting</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2872,26 +2468,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum but lacks many JD‑specific measurement and reporting keywords and does not show location alignment, resulting in a low ATS score; the biggest gap is the absence of dashboard/KPI experience.</t>
+          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>KPIs, Dashboard, Scorecard, Product maturity assessment, Quantitative analysis, Qualitative feedback, Measurement framework, Analytics platform, Data instrumentation</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2909,17 +2503,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2579,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -3051,19 +2645,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Industrial</t>
+          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3074,22 +2668,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; the resume shows 4 years experience and appropriate title, but the JD provides no concrete keywords, resulting in low keyword density. The biggest gap is the lack of typical product‑management methodology terms.</t>
+          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Product roadmap, User research, Metrics/KPIs</t>
+          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -3107,17 +2701,17 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -3129,38 +2723,38 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Market Risk Exposure Platforms Integration</t>
+          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience rule, but it lacks many core product‑manager keywords from the UBS risk‑platform JD and does not show location alignment, resulting in a low ATS pass likelihood; the biggest gap is the absence of risk‑domain terminology.</t>
+          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Market Risk, Risk Exposure, Integration, Financial Services, Regulatory compliance, OKRs, Product roadmap, A/B testing, Snowflake</t>
+          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -3169,64 +2763,66 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Zinnia</t>
+          <t>2070Health</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Technical) - Identity &amp; Access Management</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks many core CIAM and security keywords required by the JD, resulting in a low ATS match and limited domain relevance.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OAuth 2.0, OpenID Connect, SAML, SCIM, MFA, RBAC, ABAC, CIAM, regulatory compliance, passwordless authentication</t>
+          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -3235,64 +2831,66 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>xponentiate</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
+          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -3301,7 +2899,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -3310,55 +2908,57 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BNY</t>
+          <t>Qonevo Technologies Private Limited</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Vice President, POM Product Owner</t>
+          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune/Pimpri-Chinchwad Area</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rule 3 triggers because the target title contains 'VP', so both scores must be below 30 regardless of experience or keywords; the resume lacks senior‑level leadership keywords.</t>
+          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG strategy</t>
+          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -3367,11 +2967,11 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -3381,47 +2981,45 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2070Health</t>
+          <t>Broadridge</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
+          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
+          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3444,29 +3042,29 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>xponentiate</t>
+          <t>Magicmind Technologies</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>WB, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -3474,22 +3072,22 @@
         <v>2</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
+          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
+          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3512,214 +3110,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Qonevo Technologies Private Limited</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Broadridge</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>TS, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Magicmind Technologies</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>WB, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -3738,9 +3134,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-11
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>InCred Financial Services</t>
+          <t>Tario</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - AI-Powered SaaS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume covers most JD keywords but lacks a few analytics and measurement terms, leading to a strong ATS score and a solid fit despite limited fintech domain exposure.</t>
+          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior‑level title triggers hard rules; the resume covers most core JD terms but lacks several specific keywords like "customer‑facing" and "prototype".</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>customer-facing, prototype, A/B testing, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,57 +618,55 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Tario</t>
+          <t>Michael Page</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI-Powered SaaS</t>
+          <t>Marketing: Product Manager | Bangalore</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Rural, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (has 4 years) and no senior‑level title triggers hard rules; the resume covers most core JD terms but lacks several specific keywords like "customer‑facing" and "prototype".</t>
+          <t>Hard rules are satisfied; the resume contains most core JD keywords (Power BI, Jira, Agile, stakeholder management) but lacks media‑specific terms, lowering the ATS score to the high‑70s. Domain mismatch with media/marketing reduces the fit score to the mid‑60s.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>customer-facing, prototype, A/B testing, OKRs, Mixpanel</t>
+          <t>Digital Asset Management (DAM), Content Governance, Media Technology, Marketing, A/B testing, OKRs, User NPS improvement</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -691,12 +689,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -764,19 +762,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Cite AI</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -786,25 +784,25 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and title alignment, but the resume lacks several JD-specific keywords such as visibility tracking and competitor benchmarking, lowering the ATS score. The strongest keyword gap is the absence of "visibility tracking".</t>
+          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>visibility tracking, competitor benchmarking, source analysis, product roadmap, AI search</t>
+          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -822,29 +820,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Modlix</t>
+          <t>Auric AI Labs</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI / B2B SaaS/Martech</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -853,26 +851,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, so hard rules pass. The resume covers many core keywords but misses several JD‑specific terms like product roadmap and GTM, limiting the ATS score.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, GTM strategy, CRM, marketing technology, analytics dashboards, A/B testing, OKRs</t>
+          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -890,29 +886,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -921,24 +917,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
+          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -956,24 +954,24 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Auric AI Labs</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -983,28 +981,30 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H8" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
+          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
+          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,129 +1018,127 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>Sanofi</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Product Owner Corporate</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks specific keywords, resulting in moderate ATS coverage; the most notable gap is the absence of explicit product‑management frameworks such as OKRs or A/B testing.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Roadmap planning, KPIs, User research, Metrics tracking, Product analytics (e.g., Mixpanel), RICE prioritization</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JUSPAY</t>
+          <t>Shras It Solutions</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title alignment, but the resume lacks several payment‑specific tools and technologies mentioned in the JD, lowering both scores.</t>
+          <t>The candidate meets the 2‑year minimum and has relevant SaaS experience, but the resume lacks several JD‑specific terms such as product discovery, roadmap definition, KPIs, and GCC client travel, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Payments, Purescript, Haskell, Sketch, Flinto, Tableau, Data science programming</t>
+          <t>product discovery, roadmap definition, KPIs, dashboards, GCC client travel, Bachelor's in Computer Science</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1154,38 +1152,38 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>greytHR</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1196,19 +1194,19 @@
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, but lacks many payroll‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of statutory/compliance language.</t>
+          <t>The resume meets the hard rules and contains many Agile and product management keywords, but lacks healthcare-specific terms, lowering the ATS score; the biggest gap is the missing healthcare domain language.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>statutory compliance, payroll processing, anomaly detection, AI‑driven compliance alerts, user personas, business process flows, customer success, global payroll</t>
+          <t>Healthcare claims administration, US healthcare experience, Backlog grooming, Definition of Ready, Definition of Done, Scrum ceremonies, AI-enabled requirements tools, HIPAA compliance</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1222,129 +1220,125 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Landmark Group</t>
+          <t>ModMed India</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum and title level, but the resume lacks several planning‑specific keywords (e.g., PRD, UAT, backlog grooming) reducing the ATS score; overall experience aligns reasonably with the role.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>PRD, UAT planning and execution, backlog grooming, data pipelines, metrics tracking, recommendations engine, AI‑native workflow</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Okta</t>
+          <t>TIAA</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Product Platform</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many relevant product management terms but misses several core identity‑security keywords from the JD, lowering the ATS score; the biggest gap is the lack of any mention of backup/recovery or identity management.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Owner role, but the resume lacks several JD-specific keywords, lowering the ATS score; overall domain and skill fit are strong.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>backup and recovery, self‑service recovery center, identity management, IT admin, resilience strategy, large‑scale enterprise scalability, product vision and roadmap, security compliance</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1358,61 +1352,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Atlas Copco Group</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, IN P3P</t>
+          <t>Product Owner - Digital Technology</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune/Pimpri-Chinchwad Area</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
+          <t>The candidate meets the 4‑year experience requirement and the role title does not contain senior‑level terms, so hard rules pass; however the resume lacks several typical product‑owner keywords such as roadmap and OKRs, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
+          <t>Product roadmap, OKRs, KPIs, Backlog grooming, A/B testing, User segmentation, Metrics dashboard</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1426,61 +1418,61 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Vena Solutions</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner, Integrations</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
+          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1494,7 +1486,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1503,35 +1495,33 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Techdome</t>
+          <t>Simpplr</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager - Product Discovery &amp; Strategy</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
@@ -1543,17 +1533,17 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core product and AI keywords but misses key discovery terms like market sizing and TAM, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
+          <t>market sizing, TAM/SAM analysis, pricing strategy, unit economics, customer interviews, low-code platform, employee engagement metrics, intranet product experience</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -1562,64 +1552,66 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PDI Technologies</t>
+          <t>Freshot Robotics - Food Automation</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner III</t>
+          <t>Project Coordinator (Scrum Master &amp; Product Owner)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H17" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant product management terms, but the job description provides no concrete keywords, resulting in moderate ATS confidence and a decent fit based on domain experience.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior‑level title conflict, but the resume lacks several core Scrum/PO terms (e.g., Scrum Master, Confluence, UAT) reducing the ATS score; overall experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, Stakeholder alignment frameworks (e.g., RICE, MoSCoW), Data analytics tools (e.g., Mixpanel, Amplitude), Product analytics, User research methodologies</t>
+          <t>Scrum Master, Scrum, Product Owner, Confluence, User Acceptance Testing (UAT), Backlog grooming, Roadmap, Pipeline</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1628,7 +1620,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -1637,55 +1629,57 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Vena Solutions</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Integrations</t>
+          <t>Product Manager, IN P3P</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1694,7 +1688,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -1703,50 +1697,52 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Rinf</t>
+          <t>Knorr-Bremse</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F19" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers most core product management keywords but misses several JD-specific tools and frameworks.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, Power BI, Agile, SQL) but lacks several trailer‑specific portfolio and change‑management terms, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, Roadmap planning, User research, Metrics tracking</t>
+          <t>Change Request (CR) process, Portfolio optimization, VaVe pipeline, Phase‑in/phase‑out tracking, Supply chain coordination, Cost‑value engineering, Trailer product wiring, Ramp‑up monitoring</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1764,60 +1760,62 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Emerson</t>
+          <t>Knorr-Bremse AG</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Ultrasonic Plastics</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>MH, India</t>
+          <t>Mulshi, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience and seniority constraints, but lacks several core JD terms such as product roadmap, pricing strategy, and competitive analysis, lowering the ATS score; overall domain and skill alignment are solid, giving a decent fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because key JD terms like Power BI, Jira, Agile, stakeholder management appear, but many portfolio‑ and change‑management keywords are missing. Fit score is lower due to limited trailer/vehicle product experience.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, pricing strategy, competitive analysis, voice of customer, stage‑gate process, go‑to‑market plan, cost optimization, product certification</t>
+          <t>portfolio optimization, change request (CR) process, VaVe pipeline, phase‑in / phase‑out tracking, cost optimization, Excel reporting, product lifecycle documentation</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -1830,289 +1828,17 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Amazon.com</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, IN P3P</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager II</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>TS, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Indeed, Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Knorr-Bremse</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager Trailer Business</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>MH, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, Power BI, Agile, SQL) but lacks several trailer‑specific portfolio and change‑management terms, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Change Request (CR) process, Portfolio optimization, VaVe pipeline, Phase‑in/phase‑out tracking, Supply chain coordination, Cost‑value engineering, Trailer product wiring, Ramp‑up monitoring</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Knorr-Bremse AG</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager Trailer Business</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Mulshi, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because key JD terms like Power BI, Jira, Agile, stakeholder management appear, but many portfolio‑ and change‑management keywords are missing. Fit score is lower due to limited trailer/vehicle product experience.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>portfolio optimization, change request (CR) process, VaVe pipeline, phase‑in / phase‑out tracking, cost optimization, Excel reporting, product lifecycle documentation</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -2137,10 +1863,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2152,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2258,40 +1980,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bureau</t>
+          <t>Eli Lilly and Company</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (RASP)</t>
+          <t>Product Manager – Enterprise AI Operations &amp; Observability</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement and seniority rules, but the resume lacks most security‑focused keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
+          <t>No explicit years or seniority violations, but the JD provides virtually no keyword detail, resulting in a low ATS match; the candidate's GenAI and enterprise SaaS background aligns well with an Enterprise AI Operations role.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Android, iOS, mobile security, runtime application self‑protection (RASP), code obfuscation, anti‑tampering, MITM protection, SDK integration, Zero Trust framework</t>
+          <t>Observability, AI Operations, ML Ops, Metrics &amp; Monitoring, Alerting frameworks, Kubernetes, Prometheus, Grafana, Data pipeline orchestration</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2305,38 +2025,38 @@
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Eli Lilly and Company</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Enterprise AI Operations &amp; Observability</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -2345,19 +2065,19 @@
         <v>38</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>No explicit years or seniority violations, but the JD provides virtually no keyword detail, resulting in a low ATS match; the candidate's GenAI and enterprise SaaS background aligns well with an Enterprise AI Operations role.</t>
+          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Observability, AI Operations, ML Ops, Metrics &amp; Monitoring, Alerting frameworks, Kubernetes, Prometheus, Grafana, Data pipeline orchestration</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2380,24 +2100,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Keka HR</t>
+          <t>Golden Opportunities</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Finance &amp; Planning</t>
+          <t>Product Manager - GO/JC/4605/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2408,20 +2128,24 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>No explicit hard rule violations, but the job description provides virtually no keywords, resulting in a low ATS match; the candidate's strong SaaS and GenAI background is the main fit factor.</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>The candidate has only 4 years experience while the JD requires 12+ years, triggering a hard rule that forces both scores below 30; also missing key terms like 'data warehousing' and 'GTM strategy'.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>data warehousing, ETL pipelines, business intelligence dashboards, GTM strategy, product strategy</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2437,29 +2161,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Broadridge India</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2470,22 +2194,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
+          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
+          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2503,55 +2227,55 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Broadridge India</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
+          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
+          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2565,7 +2289,7 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -2574,55 +2298,55 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Serrala</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (SAP)</t>
+          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; however the JD provides virtually no keywords, resulting in low ATS keyword overlap. The biggest gap is the lack of SAP‑specific terminology.</t>
+          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SAP, product roadmap, OKRs, RICE prioritization, A/B testing</t>
+          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -2631,64 +2355,66 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>Qonevo Technologies Private Limited</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
+          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
+          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
+          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -2697,7 +2423,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -2706,55 +2432,55 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Broadridge</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>MH, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
+          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
+          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -2767,34 +2493,34 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2070Health</t>
+          <t>Magicmind Technologies</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>WB, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -2802,22 +2528,22 @@
         <v>2</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core growth‑product keywords (e.g., A/B testing, SEO/SEM, CAC, CRM, WhatsApp) needed for a strong ATS match and the domain experience is only tangential to e‑pharmacy.</t>
+          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, SEO, SEM, CRM, CAC, WhatsApp, push notifications, SMS campaigns, event tracking</t>
+          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2840,24 +2566,24 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>xponentiate</t>
+          <t>NatWest Group</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Technical Product Manager, Agentic AI, VP</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2866,26 +2592,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many core e‑pharmacy growth keywords (A/B testing, CAC, CLV, SEO/SEM, referral loops, WhatsApp/push/SMS), resulting in a modest ATS score and only a moderate fit for the health‑care marketplace role.</t>
+          <t>The JD title includes "VP", triggering hard rule 3, so both scores must be below 30 regardless of experience or keyword overlap. The most important missing keyword is "machine learning".</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CAC (Customer Acquisition Cost), CLV (Customer Lifetime Value), SEO / SEM, Referral program, WhatsApp / push / SMS campaigns, Event tracking, Lifecycle marketing</t>
+          <t>machine learning, risk management, OKRs, A/B testing, product roadmap</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2903,219 +2627,17 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Qonevo Technologies Private Limited</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Broadridge</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>TS, India</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Magicmind Technologies</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>WB, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -3131,9 +2653,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-12
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -628,45 +628,47 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Michael Page</t>
+          <t>Fam</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Marketing: Product Manager | Bangalore</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Rural, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains most core JD keywords (Power BI, Jira, Agile, stakeholder management) but lacks media‑specific terms, lowering the ATS score to the high‑70s. Domain mismatch with media/marketing reduces the fit score to the mid‑60s.</t>
+          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Digital Asset Management (DAM), Content Governance, Media Technology, Marketing, A/B testing, OKRs, User NPS improvement</t>
+          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,24 +686,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>myHQ by ANAROCK</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -711,7 +713,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -719,22 +721,22 @@
         <v>2</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement (4 years) and seniority constraints, but the resume lacks several JD-specific tools and methodologies, lowering the ATS score; the strongest keyword gap is the absence of Mixpanel/Amplitude experience.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but it misses core JD terms like explicit KPI ownership and ROI focus, lowering the ATS score slightly.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel or Amplitude, A/B testing, No-code prototyping tools, User research and behavioral data analysis, Product dashboards and KPI monitoring</t>
+          <t>product KPIs, product vision and strategy, A/B testing, OKRs, ROI analysis</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +754,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Masai</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -787,22 +789,22 @@
         <v>3</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
+          <t>The candidate meets the 3‑year minimum and holds an Associate Product Manager title, but the resume lacks several JD‑specific tools and processes (e.g., Notion, Confluence, UAT, SOPs). Keyword density is moderate, leading to a solid but not high ATS score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
+          <t>Notion, Confluence, Google Sheets/Excel, User Acceptance Testing (UAT), Standard Operating Procedures (SOPs), Release notes, Process workflow documentation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,17 +822,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -896,19 +898,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>kim.cc</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, IN P3P</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,26 +919,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and eCommerce terms; the biggest gap is lack of VBA/financial technology keywords. Fit score is lower because the candidate's domain (travel SaaS, GenAI) only loosely aligns with Amazon's seller‑financial products.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management and GenAI terms but misses several JD-specific keywords like AI governance and experimentation, lowering the ATS score. The strongest keyword gap is the lack of any mention of AI governance/hallucination mitigation.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>VBA, financial technology, eCommerce, seller experience, cost/benefit analysis, business case development</t>
+          <t>AI governance, hallucination mitigation, A/B testing, platform analytics, experimentation methodology, OKRs, product success metrics, roadmap planning</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,57 +954,57 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Techdome</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - AI/ SaaS Products</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the resume lacks several core JD tools and methodologies, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, REST APIs, API monetization, pricing strategy</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,59 +1018,61 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Sanofi</t>
+          <t>Cutshort</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner Corporate</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks specific keywords, resulting in moderate ATS coverage; the most notable gap is the absence of explicit product‑management frameworks such as OKRs or A/B testing.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several core fintech and analytics keywords, lowering the ATS score; the biggest gap is the absence of explicit A/B testing and API experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, KPIs, User research, Metrics tracking, Product analytics (e.g., Mixpanel), RICE prioritization</t>
+          <t>A/B testing, Excel / Google Sheets, API integrations, Product roadmaps, OKRs or RICE prioritization, Fintech domain experience, Metrics‑driven optimization</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1084,7 +1086,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1093,52 +1095,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Shras It Solutions</t>
+          <t>QUEST Alliance</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Experience</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has relevant SaaS experience, but the resume lacks several JD‑specific terms such as product discovery, roadmap definition, KPIs, and GCC client travel, lowering the ATS score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management terms but misses several experience‑design and learning‑specific keywords, lowering the ATS score; the biggest gap is the lack of explicit "user research" and related terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>product discovery, roadmap definition, KPIs, dashboards, GCC client travel, Bachelor's in Computer Science</t>
+          <t>user research, stakeholder interviews, field immersions, experience design, journey mapping, measurement framework, A/B testing, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1152,61 +1152,61 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>Techdome</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and contains many Agile and product management keywords, but lacks healthcare-specific terms, lowering the ATS score; the biggest gap is the missing healthcare domain language.</t>
+          <t>The candidate meets the 3+ years requirement and has no senior title, so hard rules pass; however, key JD tools like Azure DevOps, AWS, and microservices are missing, lowering the ATS score. Strong GenAI and SaaS experience boosts the fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Healthcare claims administration, US healthcare experience, Backlog grooming, Definition of Ready, Definition of Done, Scrum ceremonies, AI-enabled requirements tools, HIPAA compliance</t>
+          <t>Azure DevOps, AWS or Azure cloud platforms, microservices, APIs, LLM integrations, change control, risk mitigation, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1224,29 +1224,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ModMed India</t>
+          <t>Shras It Solutions</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1255,24 +1255,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F12" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
+          <t>The candidate meets the 2‑year minimum and has relevant SaaS experience, but the resume lacks several JD‑specific terms such as product discovery, roadmap definition, KPIs, and GCC client travel, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
+          <t>product discovery, roadmap definition, KPIs, dashboards, GCC client travel, Bachelor's in Computer Science</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1290,55 +1292,57 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TIAA</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Greater Hyderabad Area</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Owner role, but the resume lacks several JD-specific keywords, lowering the ATS score; overall domain and skill fit are strong.</t>
+          <t>The resume meets the hard rules and contains many Agile and product management keywords, but lacks healthcare-specific terms, lowering the ATS score; the biggest gap is the missing healthcare domain language.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+          <t>Healthcare claims administration, US healthcare experience, Backlog grooming, Definition of Ready, Definition of Done, Scrum ceremonies, AI-enabled requirements tools, HIPAA compliance</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,38 +1356,38 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Atlas Copco Group</t>
+          <t>ModMed India</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Digital Technology</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune/Pimpri-Chinchwad Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -1392,19 +1396,19 @@
         <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the role title does not contain senior‑level terms, so hard rules pass; however the resume lacks several typical product‑owner keywords such as roadmap and OKRs, lowering the ATS score.</t>
+          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Product roadmap, OKRs, KPIs, Backlog grooming, A/B testing, User segmentation, Metrics dashboard</t>
+          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1418,66 +1422,66 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Vena Solutions</t>
+          <t>Toolyt</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Integrations</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; however the resume lacks several core integration‑related terms (API management, extensibility, KPI tracking) and the title does not exactly match "Product Owner", lowering the ATS score. The strongest keyword gap is "API management".</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) and no senior title triggers hard rules; the main gap is missing explicit roadmap and Confluence mentions.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>API management, data integration, extensibility platform, KPI, metrics, backlog grooming, OKRs, A/B testing</t>
+          <t>roadmaps, Confluence, OKRs, A/B testing, bug fixing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -1486,59 +1490,61 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Simpplr</t>
+          <t>Knorr-Bremse</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Product Discovery &amp; Strategy</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>MH, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core product and AI keywords but misses key discovery terms like market sizing and TAM, lowering the ATS score; overall domain and skill alignment is strong, yielding a solid fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, Power BI, Agile, SQL) but lacks several trailer‑specific portfolio and change‑management terms, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>market sizing, TAM/SAM analysis, pricing strategy, unit economics, customer interviews, low-code platform, employee engagement metrics, intranet product experience</t>
+          <t>Change Request (CR) process, Portfolio optimization, VaVe pipeline, Phase‑in/phase‑out tracking, Supply chain coordination, Cost‑value engineering, Trailer product wiring, Ramp‑up monitoring</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1556,62 +1562,62 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Freshot Robotics - Food Automation</t>
+          <t>Knorr-Bremse AG</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Project Coordinator (Scrum Master &amp; Product Owner)</t>
+          <t>Associate Product Manager Trailer Business</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Mulshi, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior‑level title conflict, but the resume lacks several core Scrum/PO terms (e.g., Scrum Master, Confluence, UAT) reducing the ATS score; overall experience aligns well with the role.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because key JD terms like Power BI, Jira, Agile, stakeholder management appear, but many portfolio‑ and change‑management keywords are missing. Fit score is lower due to limited trailer/vehicle product experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Scrum Master, Scrum, Product Owner, Confluence, User Acceptance Testing (UAT), Backlog grooming, Roadmap, Pipeline</t>
+          <t>portfolio optimization, change request (CR) process, VaVe pipeline, phase‑in / phase‑out tracking, cost optimization, Excel reporting, product lifecycle documentation</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1624,221 +1630,17 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Amazon.com</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, IN P3P</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate due to missing key fintech and finance-related keywords; the biggest gap is lack of financial technology and tax compliance terms.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>VBA, financial technology, eCommerce, tax compliance, cost/benefit analysis, business case development, strategic planning, annual planning</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Knorr-Bremse</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager Trailer Business</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>MH, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, Power BI, Agile, SQL) but lacks several trailer‑specific portfolio and change‑management terms, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Change Request (CR) process, Portfolio optimization, VaVe pipeline, Phase‑in/phase‑out tracking, Supply chain coordination, Cost‑value engineering, Trailer product wiring, Ramp‑up monitoring</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Knorr-Bremse AG</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager Trailer Business</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Mulshi, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is moderate because key JD terms like Power BI, Jira, Agile, stakeholder management appear, but many portfolio‑ and change‑management keywords are missing. Fit score is lower due to limited trailer/vehicle product experience.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>portfolio optimization, change request (CR) process, VaVe pipeline, phase‑in / phase‑out tracking, cost optimization, Excel reporting, product lifecycle documentation</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1860,9 +1662,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1874,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1980,38 +1779,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Eli Lilly and Company</t>
+          <t>Raveone Consultants</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Enterprise AI Operations &amp; Observability</t>
+          <t>Toys Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Greater Hyderabad Area</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>No explicit years or seniority violations, but the JD provides virtually no keyword detail, resulting in a low ATS match; the candidate's GenAI and enterprise SaaS background aligns well with an Enterprise AI Operations role.</t>
+          <t>Hard rules pass, but the resume lacks many toy‑specific keywords and domain experience, lowering both scores; the biggest gap is the absence of toy industry and supplier management terms.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Observability, AI Operations, ML Ops, Metrics &amp; Monitoring, Alerting frameworks, Kubernetes, Prometheus, Grafana, Data pipeline orchestration</t>
+          <t>toy industry, supplier management, marketing strategy, industry standards compliance, consumer research, product launch metrics</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2025,59 +1824,61 @@
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Logistics and Fulfillment</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
+          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2091,59 +1892,59 @@
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>Karle Infra Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - GO/JC/4605/2026</t>
+          <t>Nutra &amp; Herbal- Research and Development Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years experience while the JD requires 12+ years, triggering a hard rule that forces both scores below 30; also missing key terms like 'data warehousing' and 'GTM strategy'.</t>
+          <t>Hard rules pass, but the resume contains few of the domain-specific keywords required for a Nutra &amp; Herbal R&amp;D role, resulting in low ATS and fit scores; the biggest gap is the lack of any R&amp;D or nutraceutical terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>data warehousing, ETL pipelines, business intelligence dashboards, GTM strategy, product strategy</t>
+          <t>nutraceutical product development, herbal formulation, regulatory compliance (e.g., FSSAI, FDA), clinical trial management, supply chain optimization for consumables, quality assurance (QA) protocols, market research for consumer health products, product lifecycle management in pharma</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2157,59 +1958,61 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Broadridge India</t>
+          <t>GalaxEye</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager - Mission Systems</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years in capital markets and 3+ years as a Product Owner, which exceeds the candidate's 4 years of experience, triggering the hard rule and forcing both scores below 30; the resume also lacks key terms like 'Confluence' and 'post‑trade' expertise.</t>
+          <t>Hard rules are satisfied, but the resume lacks most aerospace-specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of mission analysis tools like STK and Python scripting.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Confluence, post‑trade, Clearance &amp; Settlement, Reference Data, Books &amp; Records</t>
+          <t>STK, Python scripting for mission analysis, Orbital mechanics, RFI/RFP/tender response process, Compliance matrix, Trade studies, ConOps, Ground segment architecture</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2223,59 +2026,61 @@
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>Partner Engineering Test Company</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CLOUD TECHNICAL PRODUCT OWNER - VOIS</t>
+          <t>Matthias Test Jobs 2 Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks most cloud‑native and DevOps keywords required for the role and the title is not aligned, resulting in a low ATS score; the biggest gap is missing CI/CD and Kubernetes terminology.</t>
+          <t>The candidate meets the years requirement, but the resume lacks iOS‑specific keywords and tools, resulting in a low ATS score; the biggest gap is the absence of iOS platform experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>CI/CD, Kubernetes, DevOps, GitOps, cloud infrastructure, incident management, governance, deployment frequency, lead time</t>
+          <t>iOS app development, App Store deployment, iOS design guidelines, User engagement metrics (e.g., MAU, DAU), A/B testing</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2289,64 +2094,66 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>GoReach</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>MH, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
+          <t>The JD specifies a Senior Product Manager role, triggering the senior title hard rule, so both scores must be below 30; the resume lacks senior‑level keywords such as "lead product strategy".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
+          <t>KYC, risk profiling, financial compliance, AI‑first conversational product, mutual funds</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -2355,127 +2162,127 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Qonevo Technologies Private Limited</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Product Manager (EdTech SaaS)</t>
+          <t>Product Manager - Ruminant</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience hard rule, but contains few of the marketing‑focused keywords required by the JD, resulting in a low ATS score; the biggest gap is the lack of brand and marketing terminology.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Brand Management, Marketing Strategy, Product Lifecycle Management, Inventory Management, Market Research, Promotional Strategies, KOL Engagement, Budget Planning</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year requirement and has no senior title, so hard rules pass, but the resume lacks many education‑specific SaaS keywords and business‑development terms, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>LMS, ERP, education SaaS, pre‑sales demos, pipeline management, RFP, ARR, churn, pricing strategy</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Broadridge</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>AA Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core Kafka and data‑integration keywords, resulting in a modest ATS score; the biggest gap is the absence of any mention of Apache Kafka.</t>
+          <t>Hard rules pass, but the resume lacks many marketing‑specific keywords and brand‑focused experience required for the role, leading to a modest ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Apache Kafka, Kafka architecture, Kafka topics, data modeling, data mapping, event-driven architecture, Kafka‑based integrations, integration with external systems</t>
+          <t>brand strategy, product launch planning, campaign development, multi‑channel marketing, KPIs, performance tracking, customer insight, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2493,151 +2300,17 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Magicmind Technologies</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>WB, India</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks core market research keywords, tools, and the target title, resulting in a low ATS score; the biggest gap is the absence of market research methodology terms.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Market research, Competitor analysis, Consumer insights, Surveys, Google Sheets, PowerPoint, Google Forms, Primary research, Secondary research, Data analysis</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>NatWest Group</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Manager, Agentic AI, VP</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>The JD title includes "VP", triggering hard rule 3, so both scores must be below 30 regardless of experience or keyword overlap. The most important missing keyword is "machine learning".</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>machine learning, risk management, OKRs, A/B testing, product roadmap</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2651,8 +2324,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-14
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fam</t>
+          <t>BimaKavach</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,9 +581,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>78</v>
       </c>
@@ -595,12 +593,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume misses several CRM‑specific keywords from the JD, lowering the ATS score slightly.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>CRM platform configuration, workflow automation, release coordination, user acceptance testing (UAT), integration with third‑party systems</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,34 +616,34 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Teamware Solutions</t>
+          <t>Fam</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -654,19 +652,19 @@
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the Associate Product Owner role, but the JD lacks specific keywords, leading to moderate ATS confidence; the biggest gap is the absence of explicit OKR and A/B testing terminology.</t>
+          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, User story mapping, Product roadmap, Metrics dashboard, Customer journey mapping, Mixpanel, Scrum ceremonies</t>
+          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,34 +682,34 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Carrier</t>
+          <t>Teamware Solutions</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Product Strategy &amp; Growth</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -720,19 +718,19 @@
         <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>79</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD likely contains several specific tools and frameworks not present in the resume, lowering the ATS score slightly.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the Associate Product Owner role, but the JD lacks specific keywords, leading to moderate ATS confidence; the biggest gap is the absence of explicit OKR and A/B testing terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>OKRs, A/B testing, User story mapping, Product roadmap, Metrics dashboard, Customer journey mapping, Mixpanel, Scrum ceremonies</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -760,19 +758,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Uplers</t>
+          <t>WisdomAI</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; AI Product Manager (Intelligence Pod)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,26 +779,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>79</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the years and location requirements and includes most core keywords, but lacks explicit AI/LLM pipeline, data quality, and data platform terms.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>AI/LLM pipelines, data quality, Data Platforms, OKRs, A/B testing</t>
+          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -823,19 +819,19 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>WisdomAI</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -854,19 +850,19 @@
         <v>72</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but it misses core JD terms like explicit KPI ownership and ROI focus, lowering the ATS score slightly.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
+          <t>product KPIs, product vision and strategy, A/B testing, OKRs, ROI analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -889,24 +885,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Doctor Experience</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,22 +913,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>76</v>
-      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but it misses core JD terms like explicit KPI ownership and ROI focus, lowering the ATS score slightly.</t>
+          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>product KPIs, product vision and strategy, A/B testing, OKRs, ROI analysis</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, PLG strategy</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -955,12 +951,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -981,7 +977,9 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
         <v>68</v>
       </c>
@@ -1026,19 +1024,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Justdial</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Doctor Experience</t>
+          <t>Justdial - Product Manager - Smart Assist</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1052,19 +1050,19 @@
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the JD lacks many specific keywords present in the resume, leading to a moderate ATS score; the biggest gap is the absence of common product analytics and prioritization terms.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, PLG strategy</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,7 +1080,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1092,19 +1090,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Justdial</t>
+          <t>DataWeave</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Justdial - Product Manager - Smart Assist</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1125,12 +1123,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the JD lacks many specific keywords present in the resume, leading to a moderate ATS score; the biggest gap is the absence of common product analytics and prioritization terms.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks explicit keywords, leading to moderate ATS confidence; the most notable gap is the absence of roadmap and OKR terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>Roadmap planning, OKRs, A/B testing, User research, Metrics tracking, Product analytics (e.g., Mixpanel), Customer segmentation</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,29 +1146,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>IKEA</t>
+          <t>Masai</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Change Governance</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,22 +1179,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>71</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit keywords present in the resume, leading to a moderate ATS score; the biggest gap is the absence of common product metrics and experimentation tools.</t>
+          <t>The candidate meets the 3‑year minimum and holds an Associate Product Manager title, but the resume lacks several JD‑specific tools and processes (e.g., Notion, Confluence, UAT, SOPs). Keyword density is moderate, leading to a solid but not high ATS score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Roadmap planning, Stakeholder alignment frameworks</t>
+          <t>Notion, Confluence, Google Sheets/Excel, User Acceptance Testing (UAT), Standard Operating Procedures (SOPs), Release notes, Process workflow documentation</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,34 +1212,34 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>DataWeave</t>
+          <t>People Prime Worldwide</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Greater Kolkata Area</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -1250,19 +1248,19 @@
         <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks explicit keywords, leading to moderate ATS confidence; the most notable gap is the absence of roadmap and OKR terminology.</t>
+          <t>The resume meets the hard rules and includes many core keywords like Jira, Agile, user stories, and stakeholder management, but lacks several specific marketing analytics and SAFe terms, leading to a moderate ATS score; the biggest gap is the absence of SAFe/PI planning terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Roadmap planning, OKRs, A/B testing, User research, Metrics tracking, Product analytics (e.g., Mixpanel), Customer segmentation</t>
+          <t>SAFe Agile framework, PI Planning, Release Train Engineer (RTE), Scrum Master coordination, Marketing analytics, Business analytics reporting, OKRs, Backlog grooming, Metrics and KPI tracking</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1276,59 +1274,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Masai</t>
+          <t>StarRez, Inc.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and holds an Associate Product Manager title, but the resume lacks several JD‑specific tools and processes (e.g., Notion, Confluence, UAT, SOPs). Keyword density is moderate, leading to a solid but not high ATS score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Notion, Confluence, Google Sheets/Excel, User Acceptance Testing (UAT), Standard Operating Procedures (SOPs), Release notes, Process workflow documentation</t>
+          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1342,38 +1340,38 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Mojro</t>
+          <t>Backbase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - I</t>
+          <t>(Agentic) Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -1389,12 +1387,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the generic JD provides few concrete keywords, leading to moderate ATS confidence and a decent overall fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core AI‑agent terminology from the JD, lowering the ATS score, while the candidate's GenAI and enterprise SaaS background gives a decent fit.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, User research, Product metrics (e.g., NPS, MAU), Roadmap planning</t>
+          <t>LLM, inference latency, enterprise‑grade compliance, AI agents, data connectors, durable processes, cross‑pillar integration, customer discovery, roadmap definition</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1408,59 +1406,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Alacriti</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Google Photos</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the location matches, but the resume lacks several core Google Photos product keywords, lowering the ATS score; the strongest gap is the absence of explicit photo‑related product experience.</t>
+          <t>The candidate meets the 3+ years requirement and title level, but the resume lacks many fintech‑specific keywords (API, payments, cloud‑native, latency, holdback testing) reducing both scores.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, User experience (UX) research, Mobile app product development, Machine learning for image analysis, Metrics such as MAU/DAU growth, OKR framework, Photo storage and sharing, Privacy and security compliance</t>
+          <t>API design, payment processing, cloud-native platform, holdback testing, revenue adoption metrics, latency optimization</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1474,64 +1472,66 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Cutshort</t>
+          <t>Toolyt</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, but the resume lacks several core fintech and analytics keywords, lowering the ATS score; the biggest gap is the absence of explicit A/B testing and API experience.</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) and no senior title triggers hard rules; the main gap is missing explicit roadmap and Confluence mentions.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Excel / Google Sheets, API integrations, Product roadmaps, OKRs or RICE prioritization, Fintech domain experience, Metrics‑driven optimization</t>
+          <t>roadmaps, Confluence, OKRs, A/B testing, bug fixing</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -1540,11 +1540,11 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1554,28 +1554,30 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Evernorth Health Services</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Technical product owner</t>
+          <t>Product Manager -II</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>TS, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
@@ -1587,17 +1589,17 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the JD provides few explicit keywords so keyword density is moderate, with notable gaps in common product tools and metrics.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; ATS score is moderate due to solid keyword overlap but missing several JD‑specific terms, while the fit score is higher because of strong GenAI and SaaS experience relevant to Copilot.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>Windows, Mac, A/B testing, OKRs, NPS improvement, User research, Roadmap planning, Growth metrics, Customer insights</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed, Linkedin</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1606,7 +1608,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -1615,29 +1617,29 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>SyndiGO</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>FBS Product Owner III</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1655,17 +1657,17 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because key tools and methodologies like OKRs, RICE, A/B testing, Mixpanel, Snowflake are missing; fit score is higher due to strong SaaS and GenAI experience aligning with the product owner role.</t>
+          <t>The candidate meets the 4-year experience requirement and title level, but the resume lacks several JD-specific terms such as AIDLC, PXM, and business analysis artifacts, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake, NPS improvement, Roadmap planning, Quality control metrics</t>
+          <t>AI-Driven Development Lifecycle (AIDLC), Product Experience Management (PXM) platform, Proof of Concept (POC) development, Business rules and process flow documentation, Product messaging and launch coordination, Customer productivity metrics, Two-sided network experience, OKR framework</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1674,38 +1676,38 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Backbase</t>
+          <t>StoneX Group</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>(Agentic) Product Manager</t>
+          <t>Associate Product Manager - Onboarding</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -1714,24 +1716,24 @@
         <v>68</v>
       </c>
       <c r="G19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H19" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core AI‑agent terminology from the JD, lowering the ATS score, while the candidate's GenAI and enterprise SaaS background gives a decent fit.</t>
+          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume contains many relevant terms but misses several core onboarding-specific keywords, lowering the ATS score; the strongest gap is the lack of KYC/AML terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>LLM, inference latency, enterprise‑grade compliance, AI agents, data connectors, durable processes, cross‑pillar integration, customer discovery, roadmap definition</t>
+          <t>KYC, AML, due diligence, risk management, reference data, account creation, entitlements, trading readiness</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -1740,485 +1742,21 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Shras It Solutions</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 2‑year minimum and has relevant SaaS experience, but the resume lacks several JD‑specific terms such as product discovery, roadmap definition, KPIs, and GCC client travel, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>product discovery, roadmap definition, KPIs, dashboards, GCC client travel, Bachelor's in Computer Science</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD provides no specific keywords, resulting in moderate ATS confidence and a few key product‑management terms missing.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, OKRs, Metrics tracking, User segmentation, Roadmap planning</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Arcesium</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Opterra - Performance &amp; Investor Allocations (PerformA)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑level title conflict, but the job description provides few concrete keywords, resulting in moderate ATS keyword coverage; the biggest gap is the lack of explicit mention of OKRs or A/B testing.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>HealthEdge</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Greater Hyderabad Area</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and contains many Agile and product management keywords, but lacks healthcare-specific terms, lowering the ATS score; the biggest gap is the missing healthcare domain language.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Healthcare claims administration, US healthcare experience, Backlog grooming, Definition of Ready, Definition of Done, Scrum ceremonies, AI-enabled requirements tools, HIPAA compliance</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>ModMed India</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume matches many generic product management keywords but lacks healthcare‑specific terms, lowering the ATS score and fit.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>medical billing, practice management, healthcare workflow diagrams, automation triggers, cloud platform, AI‑driven logic</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Toolyt</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 1‑year minimum (has 4 years) and no senior title triggers hard rules; the main gap is missing explicit roadmap and Confluence mentions.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>roadmaps, Confluence, OKRs, A/B testing, bug fixing</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>StoneX Group</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager - Onboarding</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume contains many relevant terms but misses several core onboarding-specific keywords, lowering the ATS score; the strongest gap is the lack of KYC/AML terminology.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>KYC, AML, due diligence, risk management, reference data, account creation, entitlements, trading readiness</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2242,13 +1780,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2260,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2366,12 +1897,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>StoneX Group Inc.</t>
+          <t>1% Club</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Onboarding</t>
+          <t>Product Manager - AI</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2382,22 +1913,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>58</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume lacks many typical onboarding‑specific keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience makes them a decent fit for the role.</t>
+          <t>Hard rules pass (4 years meets the 3‑year minimum). The resume contains some AI and GenAI keywords but misses many JD‑specific terms like orchestration, memory management, and evaluation frameworks, limiting the ATS score. The biggest keyword gap is the lack of explicit AI system evaluation and human‑in‑the‑loop terminology.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, OKRs, NPS improvement, User onboarding metrics, Customer journey mapping, Retention analysis, Product analytics (e.g., Amplitude), Growth hacking</t>
+          <t>human-in-the-loop, evaluation frameworks, success metrics, model orchestration, memory management, explainability, latency, trust, AI quality</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2415,29 +1946,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Metasys Technologies</t>
+          <t>StoneX Group Inc.</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Data Product Manager – Inventory Management</t>
+          <t>Associate Product Manager - Onboarding</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2446,26 +1977,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and title seniority rules, but the resume lacks many core data‑product keywords (e.g., Python, Tableau, data lakes) resulting in a modest ATS score and only a moderate fit for the retail supply‑chain focus.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume lacks many typical onboarding‑specific keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience makes them a decent fit for the role.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Python, Tableau, data lakes, APIs, event-driven architecture, demand/supply planning (e.g., SAP IBP), retail supply chain analytics, KPI tracking, external market trends</t>
+          <t>A/B testing, Mixpanel, OKRs, NPS improvement, User onboarding metrics, Customer journey mapping, Retention analysis, Product analytics (e.g., Amplitude), Growth hacking</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2483,29 +2012,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Logistics and Fulfillment</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2516,22 +2045,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2549,55 +2078,57 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Karle Infra Pvt. Ltd.</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nutra &amp; Herbal- Research and Development Product Manager</t>
+          <t>Product Manager - Logistics and Fulfillment</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume contains few of the domain-specific keywords required for a Nutra &amp; Herbal R&amp;D role, resulting in low ATS and fit scores; the biggest gap is the lack of any R&amp;D or nutraceutical terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>nutraceutical product development, herbal formulation, regulatory compliance (e.g., FSSAI, FDA), clinical trial management, supply chain optimization for consumables, quality assurance (QA) protocols, market research for consumer health products, product lifecycle management in pharma</t>
+          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2625,19 +2156,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GalaxEye</t>
+          <t>BitDelta India</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Mission Systems</t>
+          <t>Product Manager: Wallets &amp; Payments Infrastructure</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2648,22 +2179,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most aerospace-specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of mission analysis tools like STK and Python scripting.</t>
+          <t>The resume lacks many core payments‑wallet keywords and domain experience, resulting in a low ATS likelihood; the candidate's background is strong in SaaS and GenAI but not in payments infrastructure.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>STK, Python scripting for mission analysis, Orbital mechanics, RFI/RFP/tender response process, Compliance matrix, Trade studies, ConOps, Ground segment architecture</t>
+          <t>payments gateway integration, PCI DSS compliance, tokenization, KYC/AML workflows, API design for wallets, mobile wallet onboarding, transaction monitoring, A/B testing for pricing, OKR framework, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2681,29 +2212,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GoReach</t>
+          <t>GalaxEye</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager - Mission Systems</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2713,25 +2244,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD specifies a Senior Product Manager role, triggering the senior title hard rule, so both scores must be below 30; the resume lacks senior‑level keywords such as "lead product strategy".</t>
+          <t>Hard rules are satisfied, but the resume lacks most aerospace-specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of mission analysis tools like STK and Python scripting.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>KYC, risk profiling, financial compliance, AI‑first conversational product, mutual funds</t>
+          <t>STK, Python scripting for mission analysis, Orbital mechanics, RFI/RFP/tender response process, Compliance matrix, Trade studies, ConOps, Ground segment architecture</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2749,55 +2280,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Greater Kolkata Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any fraud prevention or financial crime terminology.</t>
+          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>fraud prevention, financial crime, AML transaction monitoring, KYC/CDD/EDD, payment fraud, scrums/Confluence, API integration, event‑driven architecture</t>
+          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2811,7 +2342,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -2820,24 +2351,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tenarai</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – eCommerce</t>
+          <t>Product Manager - HR Technology</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2848,22 +2379,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>No explicit years or seniority constraints were violated, but the job description provides virtually no keywords, resulting in a low ATS match; the strongest gap is the lack of eCommerce‑specific terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Marketplace dynamics, A/B testing, Conversion rate optimization, Customer journey mapping, OKRs, RICE prioritization, SQL analytics, Product analytics (e.g., Mixpanel), Growth metrics (MAU, NPS)</t>
+          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2881,60 +2412,62 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ghar4u.com</t>
+          <t>2070Health</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Diagnostics</t>
+          <t>Product Manager - Logistics and Fulfillment</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations, but the job description provides virtually no explicit keywords, resulting in low keyword density and a modest ATS score; the candidate’s SaaS and GenAI experience gives a decent fit.</t>
+          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many logistics‑specific keywords from the JD, lowering the ATS score; domain experience is only tangentially related, resulting in a moderate fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking (e.g., MAU, NPS), Roadmap planning, User research (e.g., JTBD), Data analytics tools (e.g., Mixpanel, Amplitude), Prioritization frameworks (e.g., RICE, MoSCoW)</t>
+          <t>order management, dispatch, 3PL integration, SLA tracking, reverse logistics, exception queues, delivery status notifications, rescheduling, address handling</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -2943,7 +2476,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2957,50 +2490,50 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AA Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
+          <t>Hard rules pass, but the resume lacks many marketing‑specific keywords and brand‑focused experience required for the role, leading to a modest ATS score and a lower fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
+          <t>brand strategy, product launch planning, campaign development, multi‑channel marketing, KPIs, performance tracking, customer insight, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -3009,64 +2542,66 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Tezo</t>
+          <t>xponentiate</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - US Taxation</t>
+          <t>Product Manager, Doctor Experience</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>No explicit JD keywords are present, resulting in a low ATS match; the candidate's experience is in SaaS and GenAI, not US taxation, leading to a modest fit.</t>
+          <t>The candidate meets the 3‑year minimum (4 years) and has no senior title, so hard rules pass, but the resume lacks many doctor‑centric and clinical workflow keywords, resulting in a modest ATS score and a moderate fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>US tax compliance, Tax calculation engine, Regulatory reporting, Integration with ERP systems, Tax filing automation</t>
+          <t>doctor-facing product roadmap, clinical workflow, patient records and charts, prescriptions and care plans, CGM (continuous glucose monitoring) data, doctor NPS, AI assistance for documentation, metrics such as consult duration and documentation time</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -3075,7 +2610,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -3089,7 +2624,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3101,7 +2636,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Logistics and Fulfillment</t>
+          <t>Product Manager, Doctor Experience</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3114,22 +2649,22 @@
         <v>3</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many logistics‑specific keywords from the JD, lowering the ATS score; domain experience is only tangentially related, resulting in a moderate fit score.</t>
+          <t>The candidate meets the 3‑year minimum (4 years) and no senior title triggers a hard rule, but the resume lacks many JD‑specific medical and doctor‑experience keywords, lowering both scores.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>order management, dispatch, 3PL integration, SLA tracking, reverse logistics, exception queues, delivery status notifications, rescheduling, address handling</t>
+          <t>doctor‑facing product roadmap, patient records and charts, prescription workflow, CGM (continuous glucose monitoring) data, doctor NPS / satisfaction metrics, clinical protocols and safety guardrails, care plan and follow‑up automation, health coach collaboration</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3157,277 +2692,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>xponentiate</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Logistics &amp; Fulfillment</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, lowering both ATS and fit scores; the biggest gap is the absence of order‑management and fulfillment terminology.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>order management, delivery partner integration, reverse logistics, SLA tracking, 3PL integration, exception queue, dashboard, cost per order, RTO rate</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>AbbVie</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>AA Product Manager</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many marketing‑specific keywords and brand‑focused experience required for the role, leading to a modest ATS score and a lower fit score.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>brand strategy, product launch planning, campaign development, multi‑channel marketing, KPIs, performance tracking, customer insight, A/B testing</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>xponentiate</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Doctor Experience</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (4 years) and has no senior title, so hard rules pass, but the resume lacks many doctor‑centric and clinical workflow keywords, resulting in a modest ATS score and a moderate fit score.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>doctor-facing product roadmap, clinical workflow, patient records and charts, prescriptions and care plans, CGM (continuous glucose monitoring) data, doctor NPS, AI assistance for documentation, metrics such as consult duration and documentation time</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>2070Health</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Doctor Experience</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>KA, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (4 years) and no senior title triggers a hard rule, but the resume lacks many JD‑specific medical and doctor‑experience keywords, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>doctor‑facing product roadmap, patient records and charts, prescription workflow, CGM (continuous glucose monitoring) data, doctor NPS / satisfaction metrics, clinical protocols and safety guardrails, care plan and follow‑up automation, health coach collaboration</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Indeed</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3445,10 +2710,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-15
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BimaKavach</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -581,24 +581,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume misses several CRM‑specific keywords from the JD, lowering the ATS score slightly.</t>
+          <t>The resume meets the 2‑year minimum and matches the Associate Product Manager title, with strong keyword overlap; the biggest gap is the absence of common product analytics and prioritization tools/methodologies.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>CRM platform configuration, workflow automation, release coordination, user acceptance testing (UAT), integration with third‑party systems</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, PLG, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,17 +618,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -647,7 +649,9 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
@@ -692,45 +696,47 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Teamware Solutions</t>
+          <t>WisdomAI</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>79</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the Associate Product Owner role, but the JD lacks specific keywords, leading to moderate ATS confidence; the biggest gap is the absence of explicit OKR and A/B testing terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, User story mapping, Product roadmap, Metrics dashboard, Customer journey mapping, Mixpanel, Scrum ceremonies</t>
+          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,24 +754,24 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>WisdomAI</t>
+          <t>Sense</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -781,22 +787,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but it lacks several typical product‑manager keywords from the JD, lowering the ATS score; the strongest gap is the absence of explicit metrics‑driven frameworks like OKRs or RICE.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -814,29 +820,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Doctor Experience</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -845,24 +851,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>76</v>
-      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but it misses core JD terms like explicit KPI ownership and ROI focus, lowering the ATS score slightly.</t>
+          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product KPIs, product vision and strategy, A/B testing, OKRs, ROI analysis</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, PLG strategy</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -885,24 +893,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Toast</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Doctor Experience</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -911,7 +919,9 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
@@ -923,12 +933,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics (e.g., NPS, MAU growth).</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, PLG strategy</t>
+          <t>NPS improvement, MAU growth, A/B testing, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -956,14 +966,14 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>GoodSpace AI</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -977,26 +987,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics (e.g., NPS, MAU growth).</t>
+          <t>The resume meets the 4‑year experience requirement and the title is a close match, but it lacks several core JD keywords (Shopify, ecommerce, live‑chat, churn metrics, API integration details), lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>NPS improvement, MAU growth, A/B testing, OKRs, RICE prioritization</t>
+          <t>Shopify, ecommerce, live chat, product analytics (e.g., Mixpanel), customer churn</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,17 +1022,17 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1053,9 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
@@ -1090,19 +1100,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DataWeave</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - AI/ SaaS Products</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1111,24 +1121,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F10" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>71</v>
-      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with an Associate Product Manager role, but the JD lacks explicit keywords, leading to moderate ATS confidence; the most notable gap is the absence of roadmap and OKR terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the resume lacks several core JD tools and methodologies, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Roadmap planning, OKRs, A/B testing, User research, Metrics tracking, Product analytics (e.g., Mixpanel), Customer segmentation</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, REST APIs, API monetization, pricing strategy</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1146,55 +1158,57 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Masai</t>
+          <t>Finkraft</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager — Travel &amp; Hospitality Tech</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and holds an Associate Product Manager title, but the resume lacks several JD‑specific tools and processes (e.g., Notion, Confluence, UAT, SOPs). Keyword density is moderate, leading to a solid but not high ATS score.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Notion, Confluence, Google Sheets/Excel, User Acceptance Testing (UAT), Standard Operating Procedures (SOPs), Release notes, Process workflow documentation</t>
+          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,55 +1226,55 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>People Prime Worldwide</t>
+          <t>WSA – Wonderful Sound for All</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Greater Kolkata Area</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and includes many core keywords like Jira, Agile, user stories, and stakeholder management, but lacks several specific marketing analytics and SAFe terms, leading to a moderate ATS score; the biggest gap is the absence of SAFe/PI planning terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but lacks several JD‑specific terms such as OKRs and release planning, which lowers the ATS score; the strongest keyword gap is the absence of OKRs/metrics language.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SAFe Agile framework, PI Planning, Release Train Engineer (RTE), Scrum Master coordination, Marketing analytics, Business analytics reporting, OKRs, Backlog grooming, Metrics and KPI tracking</t>
+          <t>OKRs, KPIs, release planning, DevOps, solution architecture</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1274,33 +1288,33 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>StarRez, Inc.</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>FBS Product Owner III</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1321,12 +1335,12 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to missing core JD terms like backlog, roadmap, and prioritization; fit score is higher because the candidate's SaaS and enterprise product experience aligns well with the role.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because key tools and methodologies like OKRs, RICE, A/B testing, Mixpanel, Snowflake are missing; fit score is higher due to strong SaaS and GenAI experience aligning with the product owner role.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>backlog management, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake, NPS improvement, Roadmap planning, Quality control metrics</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1349,24 +1363,24 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Backbase</t>
+          <t>Alacriti</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>(Agentic) Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1375,24 +1389,26 @@
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks several core AI‑agent terminology from the JD, lowering the ATS score, while the candidate's GenAI and enterprise SaaS background gives a decent fit.</t>
+          <t>The candidate meets the 3+ years requirement and title level, but the resume lacks many fintech‑specific keywords (API, payments, cloud‑native, latency, holdback testing) reducing both scores.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>LLM, inference latency, enterprise‑grade compliance, AI agents, data connectors, durable processes, cross‑pillar integration, customer discovery, roadmap definition</t>
+          <t>API design, payment processing, cloud-native platform, holdback testing, revenue adoption metrics, latency optimization</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1410,55 +1426,55 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Alacriti</t>
+          <t>WhiteSlips Job Management Consultants</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune/Pimpri-Chinchwad Area</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and title level, but the resume lacks many fintech‑specific keywords (API, payments, cloud‑native, latency, holdback testing) reducing both scores.</t>
+          <t>The resume meets the experience requirement and title level, but misses several core JD terms like backlog, roadmap, and instrumentation, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>API design, payment processing, cloud-native platform, holdback testing, revenue adoption metrics, latency optimization</t>
+          <t>product backlog, roadmap, specifications, trade‑off decision, instrumentation/metrics, UX assessment, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1472,66 +1488,64 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Toolyt</t>
+          <t>Ujjivan Small Finance Bank</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Asset Product Manager -Pune RO</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 1‑year minimum (has 4 years) and no senior title triggers hard rules; the main gap is missing explicit roadmap and Confluence mentions.</t>
+          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the job description provides no concrete keywords, resulting in a moderate ATS match and a decent overall fit.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>roadmaps, Confluence, OKRs, A/B testing, bug fixing</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -1540,38 +1554,38 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>TruckX Technologies Pvt Ltd</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1582,24 +1596,24 @@
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; ATS score is moderate due to solid keyword overlap but missing several JD‑specific terms, while the fit score is higher because of strong GenAI and SaaS experience relevant to Copilot.</t>
+          <t>The candidate meets the 3‑year minimum and has no senior title, so hard rules pass; however the resume lacks logistics/supply‑chain specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of logistics‑related terminology.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Windows, Mac, A/B testing, OKRs, NPS improvement, User research, Roadmap planning, Growth metrics, Customer insights</t>
+          <t>logistics, supply chain, load board, broker integration, Claude (or similar AI prototyping tool), pilot customer management, tagged request list, OKRs</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Indeed, Linkedin</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1608,66 +1622,64 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SyndiGO</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>FBS Product Owner III- Guidewire</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title level, but the resume lacks several JD-specific terms such as AIDLC, PXM, and business analysis artifacts, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>AI-Driven Development Lifecycle (AIDLC), Product Experience Management (PXM) platform, Proof of Concept (POC) development, Business rules and process flow documentation, Product messaging and launch coordination, Customer productivity metrics, Two-sided network experience, OKR framework</t>
+          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1676,7 +1688,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -1685,78 +1697,346 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>StoneX Group</t>
+          <t>Hirea4u</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Onboarding</t>
+          <t>Product Owner – Digital Manufacturing &amp; WMS | 10+ Yrs Exp</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SQL, GenAI, stakeholder management), but the fit score is low because the resume lacks experience in digital manufacturing, WMS, and supply‑chain domains.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Warehouse Management System (WMS), Digital Manufacturing, Supply Chain Optimization, IoT integration, Lean Manufacturing, KPIs and metrics tracking, Manufacturing execution system (MES), Production scheduling</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Owner</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G20" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>SyndiGO</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4-year experience requirement and title level, but the resume lacks several JD-specific terms such as AIDLC, PXM, and business analysis artifacts, lowering the ATS score; overall domain and skill alignment are strong.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>AI-Driven Development Lifecycle (AIDLC), Product Experience Management (PXM) platform, Proof of Concept (POC) development, Business rules and process flow documentation, Product messaging and launch coordination, Customer productivity metrics, Two-sided network experience, OKR framework</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>StoneX Group</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager - Onboarding</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Hard rules are satisfied (4 years experience, appropriate title). The resume contains many relevant terms but misses several core onboarding-specific keywords, lowering the ATS score; the strongest gap is the lack of KYC/AML terminology.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>KYC, AML, due diligence, risk management, reference data, account creation, entitlements, trading readiness</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Indeed</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager -II</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>TS, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; ATS score is moderate due to solid keyword overlap but missing several JD‑specific terms, while the fit score is higher because of strong GenAI and SaaS experience relevant to Copilot.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Windows, Mac, A/B testing, OKRs, NPS improvement, User research, Roadmap planning, Growth metrics, Customer insights</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Indeed, Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -1780,6 +2060,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1791,7 +2075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1911,7 +2195,9 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" s="2" t="n">
         <v>52</v>
       </c>
@@ -1956,19 +2242,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>StoneX Group Inc.</t>
+          <t>Levi Strauss &amp; Co.</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Onboarding</t>
+          <t>Product Manager – Shopify Markets, E-Commerce</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1979,22 +2265,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume lacks many typical onboarding‑specific keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience makes them a decent fit for the role.</t>
+          <t>No hard rule violations; however, the JD provides no specific keywords, resulting in limited keyword overlap and a modest ATS score, while the candidate's experience is only tangential to Shopify marketplace e‑commerce.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, OKRs, NPS improvement, User onboarding metrics, Customer journey mapping, Retention analysis, Product analytics (e.g., Amplitude), Growth hacking</t>
+          <t>Shopify, Marketplace dynamics, Two-sided platform, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2017,24 +2303,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Rippling</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager, Payroll Integrations</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2043,7 +2329,9 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F4" s="2" t="n">
         <v>55</v>
       </c>
@@ -2055,12 +2343,12 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2078,29 +2366,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Logistics and Fulfillment</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2110,25 +2398,25 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2146,29 +2434,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BitDelta India</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager: Wallets &amp; Payments Infrastructure</t>
+          <t>Product Manager - Logistics and Fulfillment</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2177,24 +2465,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many core payments‑wallet keywords and domain experience, resulting in a low ATS likelihood; the candidate's background is strong in SaaS and GenAI but not in payments infrastructure.</t>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>payments gateway integration, PCI DSS compliance, tokenization, KYC/AML workflows, API design for wallets, mobile wallet onboarding, transaction monitoring, A/B testing for pricing, OKR framework, NPS improvement</t>
+          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2212,29 +2502,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GalaxEye</t>
+          <t>BitDelta India</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Mission Systems</t>
+          <t>Product Manager: Wallets &amp; Payments Infrastructure</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2244,25 +2534,25 @@
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most aerospace-specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of mission analysis tools like STK and Python scripting.</t>
+          <t>The resume lacks many core payments‑wallet keywords and domain experience, resulting in a low ATS likelihood; the candidate's background is strong in SaaS and GenAI but not in payments infrastructure.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>STK, Python scripting for mission analysis, Orbital mechanics, RFI/RFP/tender response process, Compliance matrix, Trade studies, ConOps, Ground segment architecture</t>
+          <t>payments gateway integration, PCI DSS compliance, tokenization, KYC/AML workflows, API design for wallets, mobile wallet onboarding, transaction monitoring, A/B testing for pricing, OKR framework, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2280,24 +2570,24 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>AB InBev APAC</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -2307,28 +2597,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Greater Kolkata Area</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD provides no concrete keywords, so the resume matches very few explicit terms, resulting in a low ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably well with a typical Product Manager role.</t>
+          <t>Hard rules are satisfied, but the resume lacks many data platform specific terms from the JD, leading to a modest ATS score; the biggest keyword gap is the absence of 'data mesh' and related ingestion/transformation terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Roadmap planning, User research, Metrics and KPI tracking</t>
+          <t>data mesh, domain-driven design, ingestion, transformation, serving, cloud-native, integration-as-a-service, data engineering, ML pipelines</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2342,21 +2632,21 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2667,9 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F9" s="2" t="n">
         <v>28</v>
       </c>
@@ -2422,52 +2714,50 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2070Health</t>
+          <t>StoneX Group Inc.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Logistics and Fulfillment</t>
+          <t>Associate Product Manager - Onboarding</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and seniority constraints, but the resume lacks many logistics‑specific keywords from the JD, lowering the ATS score; domain experience is only tangentially related, resulting in a moderate fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume lacks many typical onboarding‑specific keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience makes them a decent fit for the role.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>order management, dispatch, 3PL integration, SLA tracking, reverse logistics, exception queues, delivery status notifications, rescheduling, address handling</t>
+          <t>A/B testing, Mixpanel, OKRs, NPS improvement, User onboarding metrics, Customer journey mapping, Retention analysis, Product analytics (e.g., Amplitude), Growth hacking</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -2476,7 +2766,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2490,50 +2780,50 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AbbVie</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>AA Product Manager</t>
+          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many marketing‑specific keywords and brand‑focused experience required for the role, leading to a modest ATS score and a lower fit score.</t>
+          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>brand strategy, product launch planning, campaign development, multi‑channel marketing, KPIs, performance tracking, customer insight, A/B testing</t>
+          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -2542,66 +2832,66 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>xponentiate</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Doctor Experience</t>
+          <t>Associate Product Manager / Project Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (4 years) and has no senior title, so hard rules pass, but the resume lacks many doctor‑centric and clinical workflow keywords, resulting in a modest ATS score and a moderate fit score.</t>
+          <t>Hard rules pass (4 years meets the 2-year minimum and no senior title). The resume lacks many security‑specific keywords from the JD, lowering the ATS score, and the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with vulnerability management.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>doctor-facing product roadmap, clinical workflow, patient records and charts, prescriptions and care plans, CGM (continuous glucose monitoring) data, doctor NPS, AI assistance for documentation, metrics such as consult duration and documentation time</t>
+          <t>Asset Discovery, Vulnerability Detection, Patch Management, RICE prioritization, ServiceNow, CISA KEV, EPSS, TruRisk, Threat Intelligence</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -2610,89 +2900,285 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2070Health</t>
+          <t>WhiteCrow Research</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Doctor Experience</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>48</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is low due to missing core product‑management terms like P&amp;L, pricing strategy, business case, VoC and sales enablement; title is one level below the target. Fit score is moderate because the candidate has strong SaaS and GenAI experience but the JD focuses on sustainable‑climate hardware products, creating a domain mismatch.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Product P&amp;L, Pricing strategy, Business case development, Voice of Customer (VoC) analysis, Sales enablement tools</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BNY</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Vice President, POM Product Owner</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pune/Pimpri-Chinchwad Area</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Hard rule 3 triggers because the target title contains 'VP', so both scores must be below 30 regardless of experience or keywords; the resume lacks senior‑level leadership keywords.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG strategy</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>AbbVie</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>AA Product Manager</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks many marketing‑specific keywords and brand‑focused experience required for the role, leading to a modest ATS score and a lower fit score.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>brand strategy, product launch planning, campaign development, multi‑channel marketing, KPIs, performance tracking, customer insight, A/B testing</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Commenda Technologies Inc.</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (4 years) and no senior title triggers a hard rule, but the resume lacks many JD‑specific medical and doctor‑experience keywords, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>doctor‑facing product roadmap, patient records and charts, prescription workflow, CGM (continuous glucose monitoring) data, doctor NPS / satisfaction metrics, clinical protocols and safety guardrails, care plan and follow‑up automation, health coach collaboration</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks many JD-specific compliance and workflow terms, resulting in a low ATS keyword match; the biggest gap is the absence of compliance/legal workflow experience.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>workflow builder, evaluation datasets, compliance, regulatory rules, customer feedback loops, traceability, entity management</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Indeed</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2710,6 +3196,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-10-16
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Trail</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and matches the Associate Product Manager title, with strong keyword overlap; the biggest gap is the absence of common product analytics and prioritization tools/methodologies.</t>
+          <t>The candidate meets the 3‑year minimum and has a relevant Associate Product Manager title, but the resume lacks several explicit JD terms such as machine learning and software engineering experience, lowering the ATS score slightly.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, PLG, NPS improvement</t>
+          <t>machine learning, hands‑on software engineering experience, executive presentation, product vision and roadmap, B.E/B.Tech degree</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -623,24 +623,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Fam</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Customer Incentives and Growth Platforms</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,9 +649,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
@@ -663,12 +661,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
+          <t>The resume meets all hard rules and contains many of the expected keywords, but lacks a few core growth‑product tools and frameworks common to Google PM roles.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>A/B testing, OKRs, Mixpanel, Snowflake, User segmentation, NPS improvement</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -686,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>WisdomAI</t>
+          <t>Conduent</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technology Product Owner Consultant</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the JD lacks many explicit tool keywords, resulting in a moderate ATS score; the strongest gap is the absence of explicit data‑analytics tools like Mixpanel or Snowflake.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the role, yielding strong scores; the main keyword gap is the absence of explicit OKR or A/B testing terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Snowflake, A/B testing, OKRs, Jobs-to-be-Done framework, NPS improvement, Customer journey mapping, Rapid experimentation</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -754,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Sense</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Ground Transport)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -785,24 +781,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but it lacks several typical product‑manager keywords from the JD, lowering the ATS score; the strongest gap is the absence of explicit metrics‑driven frameworks like OKRs or RICE.</t>
+          <t>The candidate meets the 4-year requirement and has a closely aligned title, yielding a solid ATS score despite missing several JD-specific tools and frameworks; the strongest keyword gap is the lack of A/B testing/OKR experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+          <t>A/B testing, OKRs, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,29 +818,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>BimaKavach</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Doctor Experience</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,26 +849,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the location matches, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns with the role, but the resume misses several CRM‑specific keywords from the JD, lowering the ATS score slightly.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, PLG strategy</t>
+          <t>CRM platform configuration, workflow automation, release coordination, user acceptance testing (UAT), integration with third‑party systems</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -888,29 +884,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Toast</t>
+          <t>smallcase</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -923,22 +919,22 @@
         <v>3</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but the job description provides no concrete keywords, resulting in moderate ATS confidence; the strongest gap is the lack of explicit product metrics (e.g., NPS, MAU growth).</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules; the resume covers most core keywords but lacks several AI‑specific terms.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>NPS improvement, MAU growth, A/B testing, OKRs, RICE prioritization</t>
+          <t>LLMs, AI agents, observability &amp; orchestration, prompt management, evaluation frameworks for generative AI, A/B testing, Mixpanel, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -956,55 +952,57 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GoodSpace AI</t>
+          <t>Supernova AI</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title is a close match, but it lacks several core JD keywords (Shopify, ecommerce, live‑chat, churn metrics, API integration details), lowering the ATS score; overall domain and skill alignment are solid, giving a good fit score.</t>
+          <t>The resume meets the years and title requirements and contains many JD keywords, but lacks several core AI product terms such as A/B testing and evaluation metrics, lowering the ATS score; the candidate's GenAI and SaaS experience aligns well but is more enterprise‑focused than consumer AI.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Shopify, ecommerce, live chat, product analytics (e.g., Mixpanel), customer churn</t>
+          <t>A/B testing, evaluation metrics, user retention, latency, cost optimization, consumer AI, AI model selection, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1022,29 +1020,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Justdial</t>
+          <t>Sense</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Justdial - Product Manager - Smart Assist</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1054,25 +1052,25 @@
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has a relevant Associate Product Manager title, but the JD lacks many specific keywords present in the resume, leading to a moderate ATS score; the biggest gap is the absence of common product analytics and prioritization terms.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns with the target role, but it lacks several typical product‑manager keywords from the JD, lowering the ATS score; the strongest gap is the absence of explicit metrics‑driven frameworks like OKRs or RICE.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1090,29 +1088,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AIMLEAP</t>
+          <t>WhiteSlips Job Management Consultants</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI/ SaaS Products</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1121,26 +1119,24 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the resume lacks several core JD tools and methodologies, lowering the ATS score.</t>
+          <t>The resume meets the experience requirement and title level, but misses several core JD terms like backlog, roadmap, and instrumentation, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, REST APIs, API monetization, pricing strategy</t>
+          <t>product backlog, roadmap, specifications, trade‑off decision, instrumentation/metrics, UX assessment, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1158,34 +1154,34 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Finkraft</t>
+          <t>Applied Materials India</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager — Travel &amp; Hospitality Tech</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1193,22 +1189,22 @@
         <v>4</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>72</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
+          <t>The candidate meets the 4-year experience requirement and has no senior title conflict, but the resume lacks several core JD keywords (e.g., Python, product roadmap, supply chain), lowering the ATS score while still showing good overall fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
+          <t>Python, product roadmap, supply chain, manufacturing operations, data pipelines, scalable architecture, OKRs, quantitative opportunity sizing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1231,50 +1227,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>WSA – Wonderful Sound for All</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager AI</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H12" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but lacks several JD‑specific terms such as OKRs and release planning, which lowers the ATS score; the strongest keyword gap is the absence of OKRs/metrics language.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>OKRs, KPIs, release planning, DevOps, solution architecture</t>
+          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1288,7 +1284,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1297,50 +1293,52 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>AIMLEAP</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>FBS Product Owner III</t>
+          <t>Product Manager - AI/ SaaS Products</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate because key tools and methodologies like OKRs, RICE, A/B testing, Mixpanel, Snowflake are missing; fit score is higher due to strong SaaS and GenAI experience aligning with the product owner role.</t>
+          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the resume lacks several core JD tools and methodologies, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake, NPS improvement, Roadmap planning, Quality control metrics</t>
+          <t>Mixpanel, Amplitude, PostHog, GA4, Looker Studio, Tableau, Confluence, REST APIs, API monetization, pricing strategy</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1354,7 +1352,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1363,29 +1361,29 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Alacriti</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - Assisted Service</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -1393,22 +1391,22 @@
         <v>3</v>
       </c>
       <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>58</v>
-      </c>
       <c r="H14" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and title level, but the resume lacks many fintech‑specific keywords (API, payments, cloud‑native, latency, holdback testing) reducing both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI keywords but lacks several marketplace‑specific terms, lowering the ATS score; the biggest gap is the absence of financial‑services and risk‑management language.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>API design, payment processing, cloud-native platform, holdback testing, revenue adoption metrics, latency optimization</t>
+          <t>Financial Services, Risk Management, Trust &amp; Safety, AI‑powered decision flows, Customer Support tools, Marketplace dynamics, Two‑sided platform, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1422,59 +1420,61 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>WhiteSlips Job Management Consultants</t>
+          <t>Porter</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager-II</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune/Pimpri-Chinchwad Area</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F15" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H15" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement and title level, but misses several core JD terms like backlog, roadmap, and instrumentation, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 4‑year minimum and has no senior title, so hard rules are satisfied; however the resume lacks several core JD keywords such as OKRs and A/B testing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>product backlog, roadmap, specifications, trade‑off decision, instrumentation/metrics, UX assessment, OKRs</t>
+          <t>OKRs, A/B testing, PRD, impact sizing, metrics‑driven approach, roadmap planning, backlog management</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1488,59 +1488,61 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Ujjivan Small Finance Bank</t>
+          <t>GreyLabs AI</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Asset Product Manager -Pune RO</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Greater Bengaluru Area</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F16" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant SaaS and GenAI experience, but the job description provides no concrete keywords, resulting in a moderate ATS match and a decent overall fit.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, but lacks several voice‑AI and BFSI specific terms, lowering the ATS match; the biggest keyword gap is the absence of ASR/NLP/TTS terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, RICE prioritization</t>
+          <t>ASR, NLP, TTS, dialogue management, voice AI, BFSI, regulatory compliance, customer discovery, roadmap prioritization (OKRs)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1554,61 +1556,61 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TruckX Technologies Pvt Ltd</t>
+          <t>Finkraft</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager — Travel &amp; Hospitality Tech</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and has no senior title, so hard rules pass; however the resume lacks logistics/supply‑chain specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of logistics‑related terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>logistics, supply chain, load board, broker integration, Claude (or similar AI prototyping tool), pilot customer management, tagged request list, OKRs</t>
+          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1622,7 +1624,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -1631,50 +1633,50 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>WSA – Wonderful Sound for All</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>FBS Product Owner III- Guidewire</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority rules, but lacks several JD‑specific terms such as OKRs and release planning, which lowers the ATS score; the strongest keyword gap is the absence of OKRs/metrics language.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
+          <t>OKRs, KPIs, release planning, DevOps, solution architecture</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1688,59 +1690,59 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Hirea4u</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Digital Manufacturing &amp; WMS | 10+ Yrs Exp</t>
+          <t>FBS Product Owner III- Guidewire</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G19" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H19" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SQL, GenAI, stakeholder management), but the fit score is low because the resume lacks experience in digital manufacturing, WMS, and supply‑chain domains.</t>
+          <t>The resume contains many relevant Agile and stakeholder keywords but misses several JD-specific terms and the location does not clearly match Hyderabad, lowering the ATS score; overall domain and skill alignment are strong, especially in SaaS and GenAI.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Warehouse Management System (WMS), Digital Manufacturing, Supply Chain Optimization, IoT integration, Lean Manufacturing, KPIs and metrics tracking, Manufacturing execution system (MES), Production scheduling</t>
+          <t>roadmap, OKRs, RICE prioritization, product backlog grooming, release planning, KPIs, NPS improvement, A/B testing</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1754,59 +1756,61 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>Alacriti</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F20" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G20" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="H20" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
+          <t>The candidate meets the 3+ years requirement and title level, but the resume lacks many fintech‑specific keywords (API, payments, cloud‑native, latency, holdback testing) reducing both scores.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
+          <t>API design, payment processing, cloud-native platform, holdback testing, revenue adoption metrics, latency optimization</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1820,44 +1824,42 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SyndiGO</t>
+          <t>tripstack</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - Virtual Interlining</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
         <v>68</v>
       </c>
@@ -1869,17 +1871,17 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title level, but the resume lacks several JD-specific terms such as AIDLC, PXM, and business analysis artifacts, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is a close match, but the resume lacks several JD‑specific terms such as API, payments, and virtual interlining, lowering the ATS score. Domain experience in travel tech and SaaS is strong, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>AI-Driven Development Lifecycle (AIDLC), Product Experience Management (PXM) platform, Proof of Concept (POC) development, Business rules and process flow documentation, Product messaging and launch coordination, Customer productivity metrics, Two-sided network experience, OKR framework</t>
+          <t>API integration, payments processing, fraud prevention, pricing optimization, virtual interlining, B2B SaaS platform, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -1888,38 +1890,38 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>StoneX Group</t>
+          <t>Emerson</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Onboarding</t>
+          <t>Software Product Owner</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>KA, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1928,24 +1930,24 @@
         <v>68</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, appropriate title). The resume contains many relevant terms but misses several core onboarding-specific keywords, lowering the ATS score; the strongest gap is the lack of KYC/AML terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the JD lacks many explicit keywords, resulting in moderate ATS coverage; the biggest gap is the absence of common product analytics and prioritization terms.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>KYC, AML, due diligence, risk management, reference data, account creation, entitlements, trading readiness</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Linkedin</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1954,7 +1956,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -1963,29 +1965,29 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>TruckX Technologies Pvt Ltd</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>TS, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
@@ -1996,47 +1998,249 @@
         <v>68</v>
       </c>
       <c r="G23" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum and has no senior title, so hard rules pass; however the resume lacks logistics/supply‑chain specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of logistics‑related terminology.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>logistics, supply chain, load board, broker integration, Claude (or similar AI prototyping tool), pilot customer management, tagged request list, OKRs</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Owner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core product management keywords but misses several tools and domain-specific terms from the JD, lowering the ATS score. The biggest gap is the lack of financial‑services/payment terminology.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, MS Visio, Draw.io, SAFe (Scaled Agile Framework), Open Banking, PSD2, API integration, Competitive analysis, Payment experience</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>SyndiGO</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>KA, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4-year experience requirement and title level, but the resume lacks several JD-specific terms such as AIDLC, PXM, and business analysis artifacts, lowering the ATS score; overall domain and skill alignment are strong.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>AI-Driven Development Lifecycle (AIDLC), Product Experience Management (PXM) platform, Proof of Concept (POC) development, Business rules and process flow documentation, Product messaging and launch coordination, Customer productivity metrics, Two-sided network experience, OKR framework</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Indeed, Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager -II</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>TS, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title triggers hard rules; ATS score is moderate due to solid keyword overlap but missing several JD‑specific terms, while the fit score is higher because of strong GenAI and SaaS experience relevant to Copilot.</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Windows, Mac, A/B testing, OKRs, NPS improvement, User research, Roadmap planning, Growth metrics, Customer insights</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Indeed, Linkedin</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -2064,6 +2268,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2075,7 +2282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2242,19 +2449,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Levi Strauss &amp; Co.</t>
+          <t>Rippling</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Shopify Markets, E-Commerce</t>
+          <t>Product Manager, Payroll Integrations</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2263,7 +2470,9 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>55</v>
       </c>
@@ -2275,12 +2484,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; however, the JD provides no specific keywords, resulting in limited keyword overlap and a modest ATS score, while the candidate's experience is only tangential to Shopify marketplace e‑commerce.</t>
+          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Shopify, Marketplace dynamics, Two-sided platform, A/B testing, OKRs</t>
+          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2298,29 +2507,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Rippling</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Payroll Integrations</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2343,12 +2552,12 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks core payroll, ERP, and accounting automation keywords, lowering both ATS and fit scores.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Payroll integration, ERP synchronization, Journal entry automation, Finance team stakeholder management, Accounting automation, Error detection and correction</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2366,29 +2575,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>BitDelta India</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager: Wallets &amp; Payments Infrastructure</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2397,26 +2606,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>The resume lacks many core payments‑wallet keywords and domain experience, resulting in a low ATS likelihood; the candidate's background is strong in SaaS and GenAI but not in payments infrastructure.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>payments gateway integration, PCI DSS compliance, tokenization, KYC/AML workflows, API design for wallets, mobile wallet onboarding, transaction monitoring, A/B testing for pricing, OKR framework, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2434,29 +2641,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Jstack Solutions</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Logistics and Fulfillment</t>
+          <t>Product Manager — Payments</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2465,26 +2672,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many logistics‑specific keywords and domain experience, leading to a modest ATS score and only a moderate fit.</t>
+          <t>Hard rules pass, but the resume lacks core payments and fintech keywords required by the JD, resulting in low ATS and fit scores; the most important gap is the absence of any payments/API experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>order management, delivery partner integrations, reverse logistics, 3PL integration, SLA tracking, exception queues, member‑facing delivery experience, prescription‑linked workflow, cost per order</t>
+          <t>Payments, API integration, Fintech, Payment orchestration, Regulatory compliance, Roadmap development, Payouts, Adoption metrics</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2502,29 +2707,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BitDelta India</t>
+          <t>Wells Fargo</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager: Wallets &amp; Payments Infrastructure</t>
+          <t>Product Owner: Securities and Prime Services Delivery (VP)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2533,26 +2738,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many core payments‑wallet keywords and domain experience, resulting in a low ATS likelihood; the candidate's background is strong in SaaS and GenAI but not in payments infrastructure.</t>
+          <t>The job title includes VP, triggering a hard rule that forces both scores below 30 regardless of experience or keywords; the resume lacks senior‑level experience and many senior‑role expectations.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>payments gateway integration, PCI DSS compliance, tokenization, KYC/AML workflows, API design for wallets, mobile wallet onboarding, transaction monitoring, A/B testing for pricing, OKR framework, NPS improvement</t>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2570,55 +2773,57 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AB InBev APAC</t>
+          <t>Happiest Minds Technologies</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>PRODUCT MANAGER - Product Management</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Greater Kolkata Area</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks many data platform specific terms from the JD, leading to a modest ATS score; the biggest keyword gap is the absence of 'data mesh' and related ingestion/transformation terminology.</t>
+          <t>The JD title includes 'Senior' which triggers a hard rule, forcing both scores below 30 despite the candidate having 4 years of experience; the resume also lacks several senior‑level keywords such as CXO‑level communication and large‑scale platform ownership.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>data mesh, domain-driven design, ingestion, transformation, serving, cloud-native, integration-as-a-service, data engineering, ML pipelines</t>
+          <t>CXO-level presentations, large-scale platform ownership, system architecture, distributed systems, cloud platforms, OKRs, RICE prioritization, risk management</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2632,127 +2837,127 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>AB InBev APAC</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - HR Technology</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Greater Kolkata Area</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied, but the resume lacks many data platform specific terms from the JD, leading to a modest ATS score; the biggest keyword gap is the absence of 'data mesh' and related ingestion/transformation terminology.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>data mesh, domain-driven design, ingestion, transformation, serving, cloud-native, integration-as-a-service, data engineering, ML pipelines</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>StoneX Group Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager - Onboarding</t>
+          <t>Product Manager - HR Technology</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume lacks many typical onboarding‑specific keywords, lowering the ATS score, while the candidate's SaaS and GenAI experience makes them a decent fit for the role.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of API or headless access capabilities.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, OKRs, NPS improvement, User onboarding metrics, Customer journey mapping, Retention analysis, Product analytics (e.g., Amplitude), Growth hacking</t>
+          <t>API and headless access, SOC 2 compliance, responsible AI, release notes, risk identification</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2766,59 +2971,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
+          <t>FBS Agile Product Manager III- Guidewire</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
+          <t>The JD requires 9+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any Guidewire or Rally experience.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
+          <t>Guidewire, Rally, Cloud, Lean business case, Nonfunctional Requirements (NFRs), Agile Release Train (ART), Program Kanban, Enterprise vision roadmap</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2832,7 +3037,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2841,52 +3046,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Qualys</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager / Project Manager</t>
+          <t>Product Manager, Employee Channels, Platforms &amp; AI Utilities</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
         <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2-year minimum and no senior title). The resume lacks many security‑specific keywords from the JD, lowering the ATS score, and the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with vulnerability management.</t>
+          <t>Hard rules pass, but the resume lacks several HR‑specific platform and governance keywords, reducing ATS match; the biggest gap is missing HR Service/Document Management terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Asset Discovery, Vulnerability Detection, Patch Management, RICE prioritization, ServiceNow, CISA KEV, EPSS, TruRisk, Threat Intelligence</t>
+          <t>HR Service platform, Document Management platform, Release readiness, User acceptance testing, Vendor management, Technical debt, Security compliance</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2904,29 +3107,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>WhiteCrow Research</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager / Project Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2935,24 +3138,26 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is low due to missing core product‑management terms like P&amp;L, pricing strategy, business case, VoC and sales enablement; title is one level below the target. Fit score is moderate because the candidate has strong SaaS and GenAI experience but the JD focuses on sustainable‑climate hardware products, creating a domain mismatch.</t>
+          <t>Hard rules pass (4 years meets the 2-year minimum and no senior title). The resume lacks many security‑specific keywords from the JD, lowering the ATS score, and the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with vulnerability management.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Product P&amp;L, Pricing strategy, Business case development, Voice of Customer (VoC) analysis, Sales enablement tools</t>
+          <t>Asset Discovery, Vulnerability Detection, Patch Management, RICE prioritization, ServiceNow, CISA KEV, EPSS, TruRisk, Threat Intelligence</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2970,7 +3175,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -2980,50 +3185,50 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BNY</t>
+          <t>Commenda Technologies Inc.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Vice President, POM Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune/Pimpri-Chinchwad Area</t>
+          <t>KA, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rule 3 triggers because the target title contains 'VP', so both scores must be below 30 regardless of experience or keywords; the resume lacks senior‑level leadership keywords.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific compliance and workflow terms, resulting in a low ATS keyword match; the biggest gap is the absence of compliance/legal workflow experience.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, PLG strategy</t>
+          <t>workflow builder, evaluation datasets, compliance, regulatory rules, customer feedback loops, traceability, entity management</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Linkedin</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -3032,7 +3237,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -3041,24 +3246,24 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>AbbVie</t>
+          <t>Kotak Securities Ltd</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>AA Product Manager</t>
+          <t>Tech Product Manager 2_MK</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3069,22 +3274,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>48</v>
+     